<commit_message>
Fill in specs for Prog - Uber Journey Ad and Prog - Native Ad
Uber Journey Ad: condensed the 6 spec variants (Display/Video ×
Pedido/Espera/Viagem phases) from the Uber Retail Media reference
sheet into one row, kept as a single format per the decision to not
split it into per-phase rows.

Native Ad: merged the DV360 native image-ad and native video-ad
official specs (support.google.com/displayvideo) into the same row,
per the decision to keep them as one format despite covering two
different asset types — both links kept in the Link field.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011oqQvDMfneVTKoco4dHUSc
</commit_message>
<xml_diff>
--- a/data/base-formatos.xlsx
+++ b/data/base-formatos.xlsx
@@ -14667,10 +14667,26 @@
           <t>Prog - Native Ad</t>
         </is>
       </c>
-      <c r="G291" s="3" t="n"/>
-      <c r="H291" s="3" t="n"/>
-      <c r="I291" s="3" t="n"/>
-      <c r="J291" s="3" t="n"/>
+      <c r="G291" s="3" t="inlineStr">
+        <is>
+          <t>IMAGEM — Logo: 100x100 a 2000x2000px (1:1); Imagem: 1200x627 a 2000x1047px (1.91:1); Imagem quadrada (opcional, obrigatória em Programmatic Guaranteed): 627x627 a 2000x2000px (1:1). VÍDEO — Logo: 100x100 a 2000x2000px (1:1); Cover image: altura mín 627px, máx 2000x1047px (1.91:1 recomendado — para mais inventário, criar criativos adicionais com 16:9, 4:3 ou 1:1); Vídeo: ficheiro fonte com a maior qualidade disponível. COPY (igual para imagem e vídeo) — Nome do anunciante: máx 25c; Headline: máx 25c (ou Long headline obrigatório se headline não usado); Long headline: máx 50c; Body text: máx 90c (ou Long body obrigatório se body não usado); Long body text: máx 150c; Landing page URL: máx 1024c; Caption URL: máx 30c; Call to action: máx 15c.</t>
+        </is>
+      </c>
+      <c r="H291" s="3" t="inlineStr">
+        <is>
+          <t>Logo, Imagem, Imagem quadrada e Cover image: máx 1200 KB cada. Nome do ficheiro: ASCII, máx 50 caracteres.</t>
+        </is>
+      </c>
+      <c r="I291" s="3" t="inlineStr">
+        <is>
+          <t>Logo/Imagem/Imagem quadrada/Cover image: JPG, JPEG ou PNG (RGB ou CMYK). Vídeo: ficheiro de vídeo (specs à parte).</t>
+        </is>
+      </c>
+      <c r="J291" s="3" t="inlineStr">
+        <is>
+          <t>https://support.google.com/displayvideo/answer/7128458 | https://support.google.com/displayvideo/answer/7548780</t>
+        </is>
+      </c>
     </row>
     <row r="292">
       <c r="A292" s="3" t="inlineStr">
@@ -15115,9 +15131,21 @@
           <t>Prog - Uber Journey Ad</t>
         </is>
       </c>
-      <c r="G305" s="3" t="n"/>
-      <c r="H305" s="3" t="n"/>
-      <c r="I305" s="3" t="n"/>
+      <c r="G305" s="3" t="inlineStr">
+        <is>
+          <t>DISPLAY — Pedido: 975x861, mín 1/máx 5 imagens (todas com logo e diferentes), copy: título máx 25c, corpo máx 52c; Espera: 420x420 ou 314x420, máx 1 imagem, copy: título máx 25c, CTA máx 15c; Viagem: 1146x393, mín 1/máx 5 imagens (todas com logo e diferentes), copy: título máx 25c, corpo máx 52c, CTA máx 15c. VIDEO (MP4, 16:9, altura mín 486px, largura mín 864px) — Pedido: 3 a 6 seg, copy: título máx 25c, corpo máx 52c; Espera: 6 a 60 seg, copy: título máx 25c, CTA máx 15c; Viagem: 6 a 60 seg, copy: título máx 25c, corpo máx 52c, CTA máx 15c. URL — Display: parametrizado, não parametrizado ou Click Tag (Click Tag só disponível nas fases de Espera e Viagem); Video: parametrizado, não parametrizado ou Click Tag (todas as fases).</t>
+        </is>
+      </c>
+      <c r="H305" s="3" t="inlineStr">
+        <is>
+          <t>Display: máx 1 MB (todas as fases). Video: máx 1 MB (Pedido); máx 3 MB (Espera e Viagem).</t>
+        </is>
+      </c>
+      <c r="I305" s="3" t="inlineStr">
+        <is>
+          <t>Display: imagens. Video: MP4.</t>
+        </is>
+      </c>
       <c r="J305" s="3" t="n"/>
     </row>
     <row r="306">

</xml_diff>

<commit_message>
Correct the 3 YouTube VRC subtype rows to reflect their real format mix
The screenshots from Google Ads' campaign subtype picker show that
Efficient reach, Non-skippable reach, and Target frequency aren't
single-format products — each mixes multiple ad formats (Google
picks which one serves per impression, based on inventory). Replaced
the earlier single-format guesses with the real mix, built from the
specs already validated for each individual format (Bumper,
Skippable In-Stream, Non-skippable In-Stream, In-Feed, Shorts) — no
new specs invented, just correctly composed. Also captured that
"Non-skippable reach" includes both the standard (7-15s) and a
30-second non-skippable in-stream variant sharing the same technical
spec but longer duration.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011oqQvDMfneVTKoco4dHUSc
</commit_message>
<xml_diff>
--- a/data/base-formatos.xlsx
+++ b/data/base-formatos.xlsx
@@ -15280,17 +15280,13 @@
       </c>
       <c r="G292" t="inlineStr">
         <is>
-          <t>16:9 ou 9:16; recomendado 1920x1080; 7 a 15 segundos; não saltável</t>
-        </is>
-      </c>
-      <c r="H292" t="inlineStr">
-        <is>
-          <t>16:9</t>
-        </is>
-      </c>
+          <t>Mistura de formatos: BUMPER — 16:9 ou 9:16; recomendado 1920x1080, mín. 640x360; até 6 segundos; não saltável; NON-SKIPPABLE STANDARD — 16:9 ou 9:16; recomendado 1920x1080; 7 a 15 segundos; não saltável; NON-SKIPPABLE 30S — mesma especificação técnica do standard, mas com 30 segundos de duração.</t>
+        </is>
+      </c>
+      <c r="H292" t="inlineStr"/>
       <c r="I292" t="inlineStr">
         <is>
-          <t>Alojado no YouTube</t>
+          <t>Alojado no YouTube (sem limite de peso do Google Ads)</t>
         </is>
       </c>
       <c r="J292" t="inlineStr">
@@ -15495,17 +15491,13 @@
       </c>
       <c r="G297" t="inlineStr">
         <is>
-          <t>16:9 ou 9:16; recomendado 1920x1080, mín. 640x360; até 6 segundos; não saltável</t>
-        </is>
-      </c>
-      <c r="H297" t="inlineStr">
-        <is>
-          <t>16:9</t>
-        </is>
-      </c>
+          <t>Mistura de formatos (o Google escolhe consoante o inventário disponível): BUMPER — 16:9 ou 9:16; recomendado 1920x1080, mín. 640x360; até 6 segundos; não saltável; SKIPPABLE IN-STREAM — 16:9 ou 9:16; recomendado 1920x1080; saltável a partir dos 5s; sem duração máxima fixa; IN-FEED — Miniatura + até 2 linhas de texto; o vídeo mantém a proporção original; SHORTS — 9:16 vertical.</t>
+        </is>
+      </c>
+      <c r="H297" t="inlineStr"/>
       <c r="I297" t="inlineStr">
         <is>
-          <t>Alojado no YouTube</t>
+          <t>Alojado no YouTube (sem limite de peso do Google Ads)</t>
         </is>
       </c>
       <c r="J297" t="inlineStr">
@@ -15552,17 +15544,13 @@
       </c>
       <c r="G298" t="inlineStr">
         <is>
-          <t>16:9 ou 9:16; recomendado 1920x1080; 7 a 15 segundos; não saltável</t>
-        </is>
-      </c>
-      <c r="H298" t="inlineStr">
-        <is>
-          <t>16:9</t>
-        </is>
-      </c>
+          <t>Mistura de formatos: BUMPER — 16:9 ou 9:16; recomendado 1920x1080, mín. 640x360; até 6 segundos; não saltável; SKIPPABLE IN-STREAM — 16:9 ou 9:16; recomendado 1920x1080; saltável a partir dos 5s; sem duração máxima fixa; NON-SKIPPABLE IN-STREAM — 16:9 ou 9:16; recomendado 1920x1080; 7 a 15 segundos; não saltável; IN-FEED — Miniatura + até 2 linhas de texto; o vídeo mantém a proporção original; SHORTS — 9:16 vertical.</t>
+        </is>
+      </c>
+      <c r="H298" t="inlineStr"/>
       <c r="I298" t="inlineStr">
         <is>
-          <t>Alojado no YouTube</t>
+          <t>Alojado no YouTube (sem limite de peso do Google Ads)</t>
         </is>
       </c>
       <c r="J298" t="inlineStr">

</xml_diff>

<commit_message>
Correct VRC wording, align YouTube Social Media format names to platform
The 3 VRC subtype rows said "o Google escolhe consoante o inventário
disponível" (Google picks), which was wrong — it's the planning team
that picks which format(s) make sense for the campaign among the
options each subtype supports. Reworded to reflect that.

Renamed the 6 formats in the YouTube Social Media block to match the
platform's own labels from its "Ad formats" campaign setup screen
(e.g. "Skippable In-Stream" -> "Skippable in-stream ads", "In-Feed
Video Ad (ex-Discovery)" -> "In-feed ads") instead of the more
generic names inherited from the Google Ads rows they were copied
from. Scoped to just the YouTube/Social Media rows — the underlying
Google and Programmatic rows keep their existing names.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011oqQvDMfneVTKoco4dHUSc
</commit_message>
<xml_diff>
--- a/data/base-formatos.xlsx
+++ b/data/base-formatos.xlsx
@@ -15280,10 +15280,9 @@
       </c>
       <c r="G292" t="inlineStr">
         <is>
-          <t>Mistura de formatos: BUMPER — 16:9 ou 9:16; recomendado 1920x1080, mín. 640x360; até 6 segundos; não saltável; NON-SKIPPABLE STANDARD — 16:9 ou 9:16; recomendado 1920x1080; 7 a 15 segundos; não saltável; NON-SKIPPABLE 30S — mesma especificação técnica do standard, mas com 30 segundos de duração.</t>
-        </is>
-      </c>
-      <c r="H292" t="inlineStr"/>
+          <t>A equipa escolhe o(s) formato(s) mais adequado(s) de entre: BUMPER — 16:9 ou 9:16; recomendado 1920x1080, mín. 640x360; até 6 segundos; não saltável; NON-SKIPPABLE STANDARD — 16:9 ou 9:16; recomendado 1920x1080; 7 a 15 segundos; não saltável; NON-SKIPPABLE 30S — mesma especificação técnica do standard, mas com 30 segundos de duração.</t>
+        </is>
+      </c>
       <c r="I292" t="inlineStr">
         <is>
           <t>Alojado no YouTube (sem limite de peso do Google Ads)</t>
@@ -15491,10 +15490,9 @@
       </c>
       <c r="G297" t="inlineStr">
         <is>
-          <t>Mistura de formatos (o Google escolhe consoante o inventário disponível): BUMPER — 16:9 ou 9:16; recomendado 1920x1080, mín. 640x360; até 6 segundos; não saltável; SKIPPABLE IN-STREAM — 16:9 ou 9:16; recomendado 1920x1080; saltável a partir dos 5s; sem duração máxima fixa; IN-FEED — Miniatura + até 2 linhas de texto; o vídeo mantém a proporção original; SHORTS — 9:16 vertical.</t>
-        </is>
-      </c>
-      <c r="H297" t="inlineStr"/>
+          <t>A equipa escolhe o(s) formato(s) mais adequado(s) de entre: BUMPER — 16:9 ou 9:16; recomendado 1920x1080, mín. 640x360; até 6 segundos; não saltável; SKIPPABLE IN-STREAM — 16:9 ou 9:16; recomendado 1920x1080; saltável a partir dos 5s; sem duração máxima fixa; IN-FEED — Miniatura + até 2 linhas de texto; o vídeo mantém a proporção original; SHORTS — 9:16 vertical.</t>
+        </is>
+      </c>
       <c r="I297" t="inlineStr">
         <is>
           <t>Alojado no YouTube (sem limite de peso do Google Ads)</t>
@@ -15544,10 +15542,9 @@
       </c>
       <c r="G298" t="inlineStr">
         <is>
-          <t>Mistura de formatos: BUMPER — 16:9 ou 9:16; recomendado 1920x1080, mín. 640x360; até 6 segundos; não saltável; SKIPPABLE IN-STREAM — 16:9 ou 9:16; recomendado 1920x1080; saltável a partir dos 5s; sem duração máxima fixa; NON-SKIPPABLE IN-STREAM — 16:9 ou 9:16; recomendado 1920x1080; 7 a 15 segundos; não saltável; IN-FEED — Miniatura + até 2 linhas de texto; o vídeo mantém a proporção original; SHORTS — 9:16 vertical.</t>
-        </is>
-      </c>
-      <c r="H298" t="inlineStr"/>
+          <t>A equipa escolhe o(s) formato(s) mais adequado(s) de entre: BUMPER — 16:9 ou 9:16; recomendado 1920x1080, mín. 640x360; até 6 segundos; não saltável; SKIPPABLE IN-STREAM — 16:9 ou 9:16; recomendado 1920x1080; saltável a partir dos 5s; sem duração máxima fixa; NON-SKIPPABLE IN-STREAM — 16:9 ou 9:16; recomendado 1920x1080; 7 a 15 segundos; não saltável; IN-FEED — Miniatura + até 2 linhas de texto; o vídeo mantém a proporção original; SHORTS — 9:16 vertical.</t>
+        </is>
+      </c>
       <c r="I298" t="inlineStr">
         <is>
           <t>Alojado no YouTube (sem limite de peso do Google Ads)</t>
@@ -18071,7 +18068,7 @@
       </c>
       <c r="F346" t="inlineStr">
         <is>
-          <t>Skippable In-Stream</t>
+          <t>Skippable in-stream ads</t>
         </is>
       </c>
       <c r="G346" t="inlineStr">
@@ -18128,7 +18125,7 @@
       </c>
       <c r="F347" t="inlineStr">
         <is>
-          <t>Non-skippable In-Stream (standard)</t>
+          <t>Non-skippable in-stream ads</t>
         </is>
       </c>
       <c r="G347" t="inlineStr">
@@ -18185,7 +18182,7 @@
       </c>
       <c r="F348" t="inlineStr">
         <is>
-          <t>Bumper</t>
+          <t>Bumper ads</t>
         </is>
       </c>
       <c r="G348" t="inlineStr">
@@ -18242,7 +18239,7 @@
       </c>
       <c r="F349" t="inlineStr">
         <is>
-          <t>In-Feed Video Ad (ex-Discovery)</t>
+          <t>In-feed ads</t>
         </is>
       </c>
       <c r="G349" t="inlineStr">
@@ -18294,7 +18291,7 @@
       </c>
       <c r="F350" t="inlineStr">
         <is>
-          <t>YouTube Shorts Ads</t>
+          <t>Shorts ads</t>
         </is>
       </c>
       <c r="G350" t="inlineStr">
@@ -18346,7 +18343,7 @@
       </c>
       <c r="F351" t="inlineStr">
         <is>
-          <t>Masthead</t>
+          <t>Masthead ads</t>
         </is>
       </c>
       <c r="G351" t="inlineStr">

</xml_diff>

<commit_message>
Split the Google publisher block by campaign type
The single "Google" block mixed formats from six different campaign
types, so generic names like "Imagem" and "Vídeo" appeared 3 times
each with no visible distinction. Instead of just renaming those to
disambiguate, split Fornecedor itself into one block per campaign
type — Google Display Network, Google Demand Gen, Google App
Campaigns, Google Performance Max, Google Search, Google Vídeo (the
YouTube/video-ad formats bought through Google Ads, kept distinct
from the separate "YouTube" Social Media block) — mirroring how
YouTube already got its own block. categoriaDoPublisher and
canalExibicaoFormato now match any Fornecedor starting with "Google"
instead of the exact string, so all six still group under "Google ou
Search" in the sidebar, filters, and Excel export.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011oqQvDMfneVTKoco4dHUSc
</commit_message>
<xml_diff>
--- a/data/base-formatos.xlsx
+++ b/data/base-formatos.xlsx
@@ -13007,7 +13007,7 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Google Display Network</t>
         </is>
       </c>
       <c r="D243" t="inlineStr">
@@ -13059,7 +13059,7 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Google Display Network</t>
         </is>
       </c>
       <c r="D244" t="inlineStr">
@@ -13111,7 +13111,7 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Google Display Network</t>
         </is>
       </c>
       <c r="D245" t="inlineStr">
@@ -13163,7 +13163,7 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Google Display Network</t>
         </is>
       </c>
       <c r="D246" t="inlineStr">
@@ -13220,7 +13220,7 @@
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Google Display Network</t>
         </is>
       </c>
       <c r="D247" t="inlineStr">
@@ -13272,7 +13272,7 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Google Display Network</t>
         </is>
       </c>
       <c r="D248" t="inlineStr">
@@ -13329,7 +13329,7 @@
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Google Display Network</t>
         </is>
       </c>
       <c r="D249" t="inlineStr">
@@ -13386,7 +13386,7 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Google Vídeo</t>
         </is>
       </c>
       <c r="D250" t="inlineStr">
@@ -13443,7 +13443,7 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Google Vídeo</t>
         </is>
       </c>
       <c r="D251" t="inlineStr">
@@ -13500,7 +13500,7 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Google Vídeo</t>
         </is>
       </c>
       <c r="D252" t="inlineStr">
@@ -13557,7 +13557,7 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Google Vídeo</t>
         </is>
       </c>
       <c r="D253" t="inlineStr">
@@ -13609,7 +13609,7 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Google Vídeo</t>
         </is>
       </c>
       <c r="D254" t="inlineStr">
@@ -13666,7 +13666,7 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Google Vídeo</t>
         </is>
       </c>
       <c r="D255" t="inlineStr">
@@ -13723,7 +13723,7 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Google Vídeo</t>
         </is>
       </c>
       <c r="D256" t="inlineStr">
@@ -13780,7 +13780,7 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Google Demand Gen</t>
         </is>
       </c>
       <c r="D257" t="inlineStr">
@@ -13837,7 +13837,7 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Google Demand Gen</t>
         </is>
       </c>
       <c r="D258" t="inlineStr">
@@ -13889,7 +13889,7 @@
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Google Demand Gen</t>
         </is>
       </c>
       <c r="D259" t="inlineStr">
@@ -17793,7 +17793,7 @@
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Google App Campaigns</t>
         </is>
       </c>
       <c r="D341" t="inlineStr">
@@ -17850,7 +17850,7 @@
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Google App Campaigns</t>
         </is>
       </c>
       <c r="D342" t="inlineStr">
@@ -17907,7 +17907,7 @@
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Google Performance Max</t>
         </is>
       </c>
       <c r="D343" t="inlineStr">
@@ -17964,7 +17964,7 @@
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Google Performance Max</t>
         </is>
       </c>
       <c r="D344" t="inlineStr">
@@ -18021,7 +18021,7 @@
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Google Performance Max</t>
         </is>
       </c>
       <c r="D345" t="inlineStr">
@@ -18078,7 +18078,7 @@
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Google Search</t>
         </is>
       </c>
       <c r="D346" t="inlineStr">
@@ -18135,7 +18135,7 @@
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Google Search</t>
         </is>
       </c>
       <c r="D347" t="inlineStr">
@@ -18192,7 +18192,7 @@
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Google Search</t>
         </is>
       </c>
       <c r="D348" t="inlineStr">
@@ -18244,7 +18244,7 @@
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Google Vídeo</t>
         </is>
       </c>
       <c r="D349" t="inlineStr">
@@ -18301,7 +18301,7 @@
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Google Vídeo</t>
         </is>
       </c>
       <c r="D350" t="inlineStr">
@@ -18358,7 +18358,7 @@
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>Google</t>
+          <t>Google Vídeo</t>
         </is>
       </c>
       <c r="D351" t="inlineStr">

</xml_diff>

<commit_message>
Merge YouTube into Google Vídeo/YouTube, remove Social Media duplicate
YouTube ads have no standalone buying platform of their own (unlike
Meta, LinkedIn or TikTok, which each have their own ads manager) —
they're always bought through Google Ads or DV360. Keeping a
separate "YouTube" block under Social Media, as if it were a peer to
those platforms, duplicated the same 6 formats already present under
the Google campaign-type split, with real risk of the two drifting
out of sync on future updates (already had to fix one twice this
session). Renamed "Google Vídeo" to "Google Vídeo/YouTube" so it's
still easy to find, and removed the redundant Social Media block.
350 -> 344 total formats.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011oqQvDMfneVTKoco4dHUSc
</commit_message>
<xml_diff>
--- a/data/base-formatos.xlsx
+++ b/data/base-formatos.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K351"/>
+  <dimension ref="A1:K345"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="18.08984375" customWidth="1" style="2" min="1" max="1"/>
@@ -13386,7 +13386,7 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>Google Vídeo</t>
+          <t>Google Vídeo/YouTube</t>
         </is>
       </c>
       <c r="D250" t="inlineStr">
@@ -13443,7 +13443,7 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>Google Vídeo</t>
+          <t>Google Vídeo/YouTube</t>
         </is>
       </c>
       <c r="D251" t="inlineStr">
@@ -13500,7 +13500,7 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>Google Vídeo</t>
+          <t>Google Vídeo/YouTube</t>
         </is>
       </c>
       <c r="D252" t="inlineStr">
@@ -13557,7 +13557,7 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>Google Vídeo</t>
+          <t>Google Vídeo/YouTube</t>
         </is>
       </c>
       <c r="D253" t="inlineStr">
@@ -13609,7 +13609,7 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>Google Vídeo</t>
+          <t>Google Vídeo/YouTube</t>
         </is>
       </c>
       <c r="D254" t="inlineStr">
@@ -13666,7 +13666,7 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>Google Vídeo</t>
+          <t>Google Vídeo/YouTube</t>
         </is>
       </c>
       <c r="D255" t="inlineStr">
@@ -13723,7 +13723,7 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>Google Vídeo</t>
+          <t>Google Vídeo/YouTube</t>
         </is>
       </c>
       <c r="D256" t="inlineStr">
@@ -17446,52 +17446,52 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Paid Social</t>
+          <t>Internet</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>YouTube</t>
+          <t>Google App Campaigns</t>
         </is>
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>YouTube</t>
+          <t>Google App Campaigns</t>
         </is>
       </c>
       <c r="E335" t="inlineStr">
         <is>
-          <t>In-Stream Video</t>
+          <t>Single Image</t>
         </is>
       </c>
       <c r="F335" t="inlineStr">
         <is>
-          <t>Skippable in-stream ads</t>
+          <t>Imagem</t>
         </is>
       </c>
       <c r="G335" t="inlineStr">
         <is>
-          <t>16:9 ou 9:16; recomendado 1920x1080; saltável a partir dos 5s; sem duração máxima fixa</t>
+          <t>Horizontal 1.91:1: 1200x628 (mín. 600x314); Vertical 4:5: 1200x1500 (mín. 320x400); Square 1:1: 1200x1200 (mín. 200x200) — até 20 imagens, opcionais mas recomendadas</t>
         </is>
       </c>
       <c r="H335" t="inlineStr">
         <is>
-          <t>16:9</t>
+          <t>1.91:1 ou 4:5 ou 1:1</t>
         </is>
       </c>
       <c r="I335" t="inlineStr">
         <is>
-          <t>Alojado no YouTube (sem limite de peso do Google Ads)</t>
+          <t>5 MB</t>
         </is>
       </c>
       <c r="J335" t="inlineStr">
         <is>
-          <t>MP4, MOV (upload via YouTube)</t>
+          <t>JPG, PNG</t>
         </is>
       </c>
       <c r="K335" t="inlineStr">
         <is>
-          <t>https://support.google.com/google-ads/answer/17091270</t>
+          <t>https://support.google.com/google-ads/answer/17091671</t>
         </is>
       </c>
     </row>
@@ -17503,37 +17503,37 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Paid Social</t>
+          <t>Internet</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>YouTube</t>
+          <t>Google App Campaigns</t>
         </is>
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>YouTube</t>
+          <t>Google App Campaigns</t>
         </is>
       </c>
       <c r="E336" t="inlineStr">
         <is>
-          <t>In-Stream Video</t>
+          <t>Single Video</t>
         </is>
       </c>
       <c r="F336" t="inlineStr">
         <is>
-          <t>Non-skippable in-stream ads</t>
+          <t>Vídeo</t>
         </is>
       </c>
       <c r="G336" t="inlineStr">
         <is>
-          <t>16:9 ou 9:16; recomendado 1920x1080; 7 a 15 segundos; não saltável</t>
+          <t>Horizontal 16:9, Vertical 9:16, Square 1:1; 10 a 60 segundos — até 20 vídeos, opcionais mas recomendados</t>
         </is>
       </c>
       <c r="H336" t="inlineStr">
         <is>
-          <t>16:9</t>
+          <t>16:9 ou 9:16 ou 1:1</t>
         </is>
       </c>
       <c r="I336" t="inlineStr">
@@ -17548,7 +17548,7 @@
       </c>
       <c r="K336" t="inlineStr">
         <is>
-          <t>https://support.google.com/google-ads/answer/11462260</t>
+          <t>https://support.google.com/google-ads/answer/17091671</t>
         </is>
       </c>
     </row>
@@ -17560,52 +17560,52 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>Paid Social</t>
+          <t>Internet</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>YouTube</t>
+          <t>Google Performance Max</t>
         </is>
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>YouTube</t>
+          <t>Google Performance Max</t>
         </is>
       </c>
       <c r="E337" t="inlineStr">
         <is>
-          <t>In-Stream Video</t>
+          <t>Single Image</t>
         </is>
       </c>
       <c r="F337" t="inlineStr">
         <is>
-          <t>Bumper ads</t>
+          <t>Imagem</t>
         </is>
       </c>
       <c r="G337" t="inlineStr">
         <is>
-          <t>16:9 ou 9:16; recomendado 1920x1080, mín. 640x360; até 6 segundos; não saltável</t>
+          <t>Horizontal 1.91:1: 1200x628 (mín. 600x314); Square 1:1: 1200x1200 (mín. 300x300); Vertical 4:5: 960x1200 (mín. 480x600, opcional) — mín. 4 imagens de cada tipo obrigatório, até 20</t>
         </is>
       </c>
       <c r="H337" t="inlineStr">
         <is>
-          <t>16:9</t>
+          <t>1.91:1 ou 1:1 ou 4:5</t>
         </is>
       </c>
       <c r="I337" t="inlineStr">
         <is>
-          <t>Alojado no YouTube</t>
+          <t>5120 KB</t>
         </is>
       </c>
       <c r="J337" t="inlineStr">
         <is>
-          <t>MP4, MOV</t>
+          <t>JPG, PNG</t>
         </is>
       </c>
       <c r="K337" t="inlineStr">
         <is>
-          <t>https://support.google.com/google-ads/answer/11462260</t>
+          <t>https://support.google.com/google-ads/answer/9748775</t>
         </is>
       </c>
     </row>
@@ -17617,52 +17617,52 @@
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>Paid Social</t>
+          <t>Internet</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>YouTube</t>
+          <t>Google Performance Max</t>
         </is>
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>YouTube</t>
+          <t>Google Performance Max</t>
         </is>
       </c>
       <c r="E338" t="inlineStr">
         <is>
-          <t>In-Feed Video</t>
+          <t>Logo</t>
         </is>
       </c>
       <c r="F338" t="inlineStr">
         <is>
-          <t>In-feed ads</t>
+          <t>Logo</t>
         </is>
       </c>
       <c r="G338" t="inlineStr">
         <is>
-          <t>Horizontal 16:9: 1920x1080; Vertical 9:16: 1080x1920; Square 1:1: 1080x1080; 15 segundos recomendado. Texto — Título: 2 linhas, 40 caracteres cada; Descrição: 2 linhas, 35 caracteres cada.</t>
+          <t>Logo quadrado 1:1: 1200x1200 (mín. 128x128, obrigatório); Logo horizontal 4:1: 1200x300 (mín. 512x128, opcional) — até 5 de cada</t>
         </is>
       </c>
       <c r="H338" t="inlineStr">
         <is>
-          <t>16:9 ou 9:16 ou 1:1</t>
+          <t>1:1 ou 4:1</t>
         </is>
       </c>
       <c r="I338" t="inlineStr">
         <is>
-          <t>Alojado no YouTube</t>
+          <t>5120 KB</t>
         </is>
       </c>
       <c r="J338" t="inlineStr">
         <is>
-          <t>MP4, MOV</t>
+          <t>JPG, PNG</t>
         </is>
       </c>
       <c r="K338" t="inlineStr">
         <is>
-          <t>https://support.google.com/google-ads/answer/17091270</t>
+          <t>https://support.google.com/google-ads/answer/9748775</t>
         </is>
       </c>
     </row>
@@ -17674,37 +17674,37 @@
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>Paid Social</t>
+          <t>Internet</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>YouTube</t>
+          <t>Google Performance Max</t>
         </is>
       </c>
       <c r="D339" t="inlineStr">
         <is>
-          <t>YouTube</t>
+          <t>Google Performance Max</t>
         </is>
       </c>
       <c r="E339" t="inlineStr">
         <is>
-          <t>Vertical Video</t>
+          <t>Single Video</t>
         </is>
       </c>
       <c r="F339" t="inlineStr">
         <is>
-          <t>Shorts ads</t>
+          <t>Vídeo</t>
         </is>
       </c>
       <c r="G339" t="inlineStr">
         <is>
-          <t>9:16 vertical: 1080x1920; 6 a 60 segundos</t>
+          <t>Horizontal 16:9, Square 1:1, Vertical 9:16; mín. 10 segundos — até 15 vídeos de cada, opcional (gerado automaticamente se não for fornecido)</t>
         </is>
       </c>
       <c r="H339" t="inlineStr">
         <is>
-          <t>9:16</t>
+          <t>16:9 ou 1:1 ou 9:16</t>
         </is>
       </c>
       <c r="I339" t="inlineStr">
@@ -17719,7 +17719,7 @@
       </c>
       <c r="K339" t="inlineStr">
         <is>
-          <t>https://support.google.com/google-ads/answer/17091270</t>
+          <t>https://support.google.com/google-ads/answer/9748775</t>
         </is>
       </c>
     </row>
@@ -17731,52 +17731,52 @@
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>Paid Social</t>
+          <t>Internet</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>YouTube</t>
+          <t>Google Search</t>
         </is>
       </c>
       <c r="D340" t="inlineStr">
         <is>
-          <t>YouTube</t>
+          <t>Google Search</t>
         </is>
       </c>
       <c r="E340" t="inlineStr">
         <is>
-          <t>Open Door</t>
+          <t>Logo</t>
         </is>
       </c>
       <c r="F340" t="inlineStr">
         <is>
-          <t>Masthead ads</t>
+          <t>Business Information (Logo)</t>
         </is>
       </c>
       <c r="G340" t="inlineStr">
         <is>
-          <t>16:9, recomendado 1920x1080 ou superior; autoplay sem som até 30 segundos, depois miniatura clicável</t>
+          <t>Logo 1:1: 1200x1200 (mín. 128x128)</t>
         </is>
       </c>
       <c r="H340" t="inlineStr">
         <is>
-          <t>16:9</t>
+          <t>1:1</t>
         </is>
       </c>
       <c r="I340" t="inlineStr">
         <is>
-          <t>Alojado no YouTube</t>
+          <t>não especificado</t>
         </is>
       </c>
       <c r="J340" t="inlineStr">
         <is>
-          <t>MP4, MOV</t>
+          <t>JPG, PNG</t>
         </is>
       </c>
       <c r="K340" t="inlineStr">
         <is>
-          <t>https://support.google.com/google-ads/answer/17091270</t>
+          <t>https://support.google.com/google-ads/answer/12437745</t>
         </is>
       </c>
     </row>
@@ -17793,37 +17793,37 @@
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>Google App Campaigns</t>
+          <t>Google Search</t>
         </is>
       </c>
       <c r="D341" t="inlineStr">
         <is>
-          <t>Google App Campaigns</t>
+          <t>Google Search</t>
         </is>
       </c>
       <c r="E341" t="inlineStr">
         <is>
-          <t>Single Image</t>
+          <t>Ad Assets</t>
         </is>
       </c>
       <c r="F341" t="inlineStr">
         <is>
-          <t>Imagem</t>
+          <t>Ad Assets (Imagens)</t>
         </is>
       </c>
       <c r="G341" t="inlineStr">
         <is>
-          <t>Horizontal 1.91:1: 1200x628 (mín. 600x314); Vertical 4:5: 1200x1500 (mín. 320x400); Square 1:1: 1200x1200 (mín. 200x200) — até 20 imagens, opcionais mas recomendadas</t>
+          <t>Square 1:1: 1200x1200 (mín. 300x300), obrigatório; Horizontal 1.91:1: 1200x628 (mín. 600x314), opcional</t>
         </is>
       </c>
       <c r="H341" t="inlineStr">
         <is>
-          <t>1.91:1 ou 4:5 ou 1:1</t>
+          <t>1:1 ou 1.91:1</t>
         </is>
       </c>
       <c r="I341" t="inlineStr">
         <is>
-          <t>5 MB</t>
+          <t>não especificado</t>
         </is>
       </c>
       <c r="J341" t="inlineStr">
@@ -17833,7 +17833,7 @@
       </c>
       <c r="K341" t="inlineStr">
         <is>
-          <t>https://support.google.com/google-ads/answer/17091671</t>
+          <t>https://support.google.com/google-ads/answer/12437745</t>
         </is>
       </c>
     </row>
@@ -17850,47 +17850,42 @@
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>Google App Campaigns</t>
+          <t>Google Search</t>
         </is>
       </c>
       <c r="D342" t="inlineStr">
         <is>
-          <t>Google App Campaigns</t>
+          <t>Google Search</t>
         </is>
       </c>
       <c r="E342" t="inlineStr">
         <is>
-          <t>Single Video</t>
+          <t>Responsive Search Ad</t>
         </is>
       </c>
       <c r="F342" t="inlineStr">
         <is>
-          <t>Vídeo</t>
+          <t>Responsive Search Ads</t>
         </is>
       </c>
       <c r="G342" t="inlineStr">
         <is>
-          <t>Horizontal 16:9, Vertical 9:16, Square 1:1; 10 a 60 segundos — até 20 vídeos, opcionais mas recomendados</t>
-        </is>
-      </c>
-      <c r="H342" t="inlineStr">
-        <is>
-          <t>16:9 ou 9:16 ou 1:1</t>
+          <t>Só texto (sem imagem) — Títulos: até 30 caracteres, 1 a 15; Descrições: até 90 caracteres, 1 a 4</t>
         </is>
       </c>
       <c r="I342" t="inlineStr">
         <is>
-          <t>Alojado no YouTube</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="J342" t="inlineStr">
         <is>
-          <t>MP4, MOV</t>
+          <t>N/A (texto)</t>
         </is>
       </c>
       <c r="K342" t="inlineStr">
         <is>
-          <t>https://support.google.com/google-ads/answer/17091671</t>
+          <t>https://support.google.com/google-ads/answer/7684791</t>
         </is>
       </c>
     </row>
@@ -17907,47 +17902,47 @@
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>Google Performance Max</t>
+          <t>Google Vídeo/YouTube</t>
         </is>
       </c>
       <c r="D343" t="inlineStr">
         <is>
-          <t>Google Performance Max</t>
+          <t>YouTube</t>
         </is>
       </c>
       <c r="E343" t="inlineStr">
         <is>
-          <t>Single Image</t>
+          <t>In-Stream Video</t>
         </is>
       </c>
       <c r="F343" t="inlineStr">
         <is>
-          <t>Imagem</t>
+          <t>Video Action Campaigns</t>
         </is>
       </c>
       <c r="G343" t="inlineStr">
         <is>
-          <t>Horizontal 1.91:1: 1200x628 (mín. 600x314); Square 1:1: 1200x1200 (mín. 300x300); Vertical 4:5: 960x1200 (mín. 480x600, opcional) — mín. 4 imagens de cada tipo obrigatório, até 20</t>
+          <t>Horizontal 16:9: 1920x1080; Vertical 9:16: 1080x1920; Square 1:1: 1080x1080; mín. 10 segundos. Texto — Título: 30c; Título longo: 90c; Descrição: 90c; CTA: 10c.</t>
         </is>
       </c>
       <c r="H343" t="inlineStr">
         <is>
-          <t>1.91:1 ou 1:1 ou 4:5</t>
+          <t>16:9 ou 9:16 ou 1:1</t>
         </is>
       </c>
       <c r="I343" t="inlineStr">
         <is>
-          <t>5120 KB</t>
+          <t>Alojado no YouTube</t>
         </is>
       </c>
       <c r="J343" t="inlineStr">
         <is>
-          <t>JPG, PNG</t>
+          <t>MP4, MOV</t>
         </is>
       </c>
       <c r="K343" t="inlineStr">
         <is>
-          <t>https://support.google.com/google-ads/answer/9748775</t>
+          <t>https://support.google.com/google-ads/answer/12066387</t>
         </is>
       </c>
     </row>
@@ -17964,47 +17959,47 @@
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>Google Performance Max</t>
+          <t>Google Vídeo/YouTube</t>
         </is>
       </c>
       <c r="D344" t="inlineStr">
         <is>
-          <t>Google Performance Max</t>
+          <t>YouTube</t>
         </is>
       </c>
       <c r="E344" t="inlineStr">
         <is>
-          <t>Logo</t>
+          <t>Thumbnail</t>
         </is>
       </c>
       <c r="F344" t="inlineStr">
         <is>
-          <t>Logo</t>
+          <t>Thumbnail (vídeo)</t>
         </is>
       </c>
       <c r="G344" t="inlineStr">
         <is>
-          <t>Logo quadrado 1:1: 1200x1200 (mín. 128x128, obrigatório); Logo horizontal 4:1: 1200x300 (mín. 512x128, opcional) — até 5 de cada</t>
+          <t>16:9: 1280x720 (mín. 1280x640)</t>
         </is>
       </c>
       <c r="H344" t="inlineStr">
         <is>
-          <t>1:1 ou 4:1</t>
+          <t>16:9</t>
         </is>
       </c>
       <c r="I344" t="inlineStr">
         <is>
-          <t>5120 KB</t>
+          <t>&lt; 2 MB (vídeos); &lt; 10 MB (podcasts)</t>
         </is>
       </c>
       <c r="J344" t="inlineStr">
         <is>
-          <t>JPG, PNG</t>
+          <t>JPG, GIF ou PNG</t>
         </is>
       </c>
       <c r="K344" t="inlineStr">
         <is>
-          <t>https://support.google.com/google-ads/answer/9748775</t>
+          <t>https://support.google.com/google-ads/answer/17091270</t>
         </is>
       </c>
     </row>
@@ -18021,382 +18016,45 @@
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>Google Performance Max</t>
+          <t>Google Vídeo/YouTube</t>
         </is>
       </c>
       <c r="D345" t="inlineStr">
         <is>
-          <t>Google Performance Max</t>
+          <t>YouTube</t>
         </is>
       </c>
       <c r="E345" t="inlineStr">
         <is>
-          <t>Single Video</t>
+          <t>Companion Banner</t>
         </is>
       </c>
       <c r="F345" t="inlineStr">
         <is>
-          <t>Vídeo</t>
+          <t>Companion Banner</t>
         </is>
       </c>
       <c r="G345" t="inlineStr">
         <is>
-          <t>Horizontal 16:9, Square 1:1, Vertical 9:16; mín. 10 segundos — até 15 vídeos de cada, opcional (gerado automaticamente se não for fornecido)</t>
+          <t>5:1: 300x60 (só em desktop)</t>
         </is>
       </c>
       <c r="H345" t="inlineStr">
         <is>
-          <t>16:9 ou 1:1 ou 9:16</t>
+          <t>5:1</t>
         </is>
       </c>
       <c r="I345" t="inlineStr">
         <is>
-          <t>Alojado no YouTube</t>
+          <t>&lt; 150 KB</t>
         </is>
       </c>
       <c r="J345" t="inlineStr">
         <is>
-          <t>MP4, MOV</t>
+          <t>JPG, GIF ou PNG</t>
         </is>
       </c>
       <c r="K345" t="inlineStr">
-        <is>
-          <t>https://support.google.com/google-ads/answer/9748775</t>
-        </is>
-      </c>
-    </row>
-    <row r="346">
-      <c r="A346" t="inlineStr">
-        <is>
-          <t>INTERNET</t>
-        </is>
-      </c>
-      <c r="B346" t="inlineStr">
-        <is>
-          <t>Internet</t>
-        </is>
-      </c>
-      <c r="C346" t="inlineStr">
-        <is>
-          <t>Google Search</t>
-        </is>
-      </c>
-      <c r="D346" t="inlineStr">
-        <is>
-          <t>Google Search</t>
-        </is>
-      </c>
-      <c r="E346" t="inlineStr">
-        <is>
-          <t>Logo</t>
-        </is>
-      </c>
-      <c r="F346" t="inlineStr">
-        <is>
-          <t>Business Information (Logo)</t>
-        </is>
-      </c>
-      <c r="G346" t="inlineStr">
-        <is>
-          <t>Logo 1:1: 1200x1200 (mín. 128x128)</t>
-        </is>
-      </c>
-      <c r="H346" t="inlineStr">
-        <is>
-          <t>1:1</t>
-        </is>
-      </c>
-      <c r="I346" t="inlineStr">
-        <is>
-          <t>não especificado</t>
-        </is>
-      </c>
-      <c r="J346" t="inlineStr">
-        <is>
-          <t>JPG, PNG</t>
-        </is>
-      </c>
-      <c r="K346" t="inlineStr">
-        <is>
-          <t>https://support.google.com/google-ads/answer/12437745</t>
-        </is>
-      </c>
-    </row>
-    <row r="347">
-      <c r="A347" t="inlineStr">
-        <is>
-          <t>INTERNET</t>
-        </is>
-      </c>
-      <c r="B347" t="inlineStr">
-        <is>
-          <t>Internet</t>
-        </is>
-      </c>
-      <c r="C347" t="inlineStr">
-        <is>
-          <t>Google Search</t>
-        </is>
-      </c>
-      <c r="D347" t="inlineStr">
-        <is>
-          <t>Google Search</t>
-        </is>
-      </c>
-      <c r="E347" t="inlineStr">
-        <is>
-          <t>Ad Assets</t>
-        </is>
-      </c>
-      <c r="F347" t="inlineStr">
-        <is>
-          <t>Ad Assets (Imagens)</t>
-        </is>
-      </c>
-      <c r="G347" t="inlineStr">
-        <is>
-          <t>Square 1:1: 1200x1200 (mín. 300x300), obrigatório; Horizontal 1.91:1: 1200x628 (mín. 600x314), opcional</t>
-        </is>
-      </c>
-      <c r="H347" t="inlineStr">
-        <is>
-          <t>1:1 ou 1.91:1</t>
-        </is>
-      </c>
-      <c r="I347" t="inlineStr">
-        <is>
-          <t>não especificado</t>
-        </is>
-      </c>
-      <c r="J347" t="inlineStr">
-        <is>
-          <t>JPG, PNG</t>
-        </is>
-      </c>
-      <c r="K347" t="inlineStr">
-        <is>
-          <t>https://support.google.com/google-ads/answer/12437745</t>
-        </is>
-      </c>
-    </row>
-    <row r="348">
-      <c r="A348" t="inlineStr">
-        <is>
-          <t>INTERNET</t>
-        </is>
-      </c>
-      <c r="B348" t="inlineStr">
-        <is>
-          <t>Internet</t>
-        </is>
-      </c>
-      <c r="C348" t="inlineStr">
-        <is>
-          <t>Google Search</t>
-        </is>
-      </c>
-      <c r="D348" t="inlineStr">
-        <is>
-          <t>Google Search</t>
-        </is>
-      </c>
-      <c r="E348" t="inlineStr">
-        <is>
-          <t>Responsive Search Ad</t>
-        </is>
-      </c>
-      <c r="F348" t="inlineStr">
-        <is>
-          <t>Responsive Search Ads</t>
-        </is>
-      </c>
-      <c r="G348" t="inlineStr">
-        <is>
-          <t>Só texto (sem imagem) — Títulos: até 30 caracteres, 1 a 15; Descrições: até 90 caracteres, 1 a 4</t>
-        </is>
-      </c>
-      <c r="I348" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="J348" t="inlineStr">
-        <is>
-          <t>N/A (texto)</t>
-        </is>
-      </c>
-      <c r="K348" t="inlineStr">
-        <is>
-          <t>https://support.google.com/google-ads/answer/7684791</t>
-        </is>
-      </c>
-    </row>
-    <row r="349">
-      <c r="A349" t="inlineStr">
-        <is>
-          <t>INTERNET</t>
-        </is>
-      </c>
-      <c r="B349" t="inlineStr">
-        <is>
-          <t>Internet</t>
-        </is>
-      </c>
-      <c r="C349" t="inlineStr">
-        <is>
-          <t>Google Vídeo</t>
-        </is>
-      </c>
-      <c r="D349" t="inlineStr">
-        <is>
-          <t>YouTube</t>
-        </is>
-      </c>
-      <c r="E349" t="inlineStr">
-        <is>
-          <t>In-Stream Video</t>
-        </is>
-      </c>
-      <c r="F349" t="inlineStr">
-        <is>
-          <t>Video Action Campaigns</t>
-        </is>
-      </c>
-      <c r="G349" t="inlineStr">
-        <is>
-          <t>Horizontal 16:9: 1920x1080; Vertical 9:16: 1080x1920; Square 1:1: 1080x1080; mín. 10 segundos. Texto — Título: 30c; Título longo: 90c; Descrição: 90c; CTA: 10c.</t>
-        </is>
-      </c>
-      <c r="H349" t="inlineStr">
-        <is>
-          <t>16:9 ou 9:16 ou 1:1</t>
-        </is>
-      </c>
-      <c r="I349" t="inlineStr">
-        <is>
-          <t>Alojado no YouTube</t>
-        </is>
-      </c>
-      <c r="J349" t="inlineStr">
-        <is>
-          <t>MP4, MOV</t>
-        </is>
-      </c>
-      <c r="K349" t="inlineStr">
-        <is>
-          <t>https://support.google.com/google-ads/answer/12066387</t>
-        </is>
-      </c>
-    </row>
-    <row r="350">
-      <c r="A350" t="inlineStr">
-        <is>
-          <t>INTERNET</t>
-        </is>
-      </c>
-      <c r="B350" t="inlineStr">
-        <is>
-          <t>Internet</t>
-        </is>
-      </c>
-      <c r="C350" t="inlineStr">
-        <is>
-          <t>Google Vídeo</t>
-        </is>
-      </c>
-      <c r="D350" t="inlineStr">
-        <is>
-          <t>YouTube</t>
-        </is>
-      </c>
-      <c r="E350" t="inlineStr">
-        <is>
-          <t>Thumbnail</t>
-        </is>
-      </c>
-      <c r="F350" t="inlineStr">
-        <is>
-          <t>Thumbnail (vídeo)</t>
-        </is>
-      </c>
-      <c r="G350" t="inlineStr">
-        <is>
-          <t>16:9: 1280x720 (mín. 1280x640)</t>
-        </is>
-      </c>
-      <c r="H350" t="inlineStr">
-        <is>
-          <t>16:9</t>
-        </is>
-      </c>
-      <c r="I350" t="inlineStr">
-        <is>
-          <t>&lt; 2 MB (vídeos); &lt; 10 MB (podcasts)</t>
-        </is>
-      </c>
-      <c r="J350" t="inlineStr">
-        <is>
-          <t>JPG, GIF ou PNG</t>
-        </is>
-      </c>
-      <c r="K350" t="inlineStr">
-        <is>
-          <t>https://support.google.com/google-ads/answer/17091270</t>
-        </is>
-      </c>
-    </row>
-    <row r="351">
-      <c r="A351" t="inlineStr">
-        <is>
-          <t>INTERNET</t>
-        </is>
-      </c>
-      <c r="B351" t="inlineStr">
-        <is>
-          <t>Internet</t>
-        </is>
-      </c>
-      <c r="C351" t="inlineStr">
-        <is>
-          <t>Google Vídeo</t>
-        </is>
-      </c>
-      <c r="D351" t="inlineStr">
-        <is>
-          <t>YouTube</t>
-        </is>
-      </c>
-      <c r="E351" t="inlineStr">
-        <is>
-          <t>Companion Banner</t>
-        </is>
-      </c>
-      <c r="F351" t="inlineStr">
-        <is>
-          <t>Companion Banner</t>
-        </is>
-      </c>
-      <c r="G351" t="inlineStr">
-        <is>
-          <t>5:1: 300x60 (só em desktop)</t>
-        </is>
-      </c>
-      <c r="H351" t="inlineStr">
-        <is>
-          <t>5:1</t>
-        </is>
-      </c>
-      <c r="I351" t="inlineStr">
-        <is>
-          <t>&lt; 150 KB</t>
-        </is>
-      </c>
-      <c r="J351" t="inlineStr">
-        <is>
-          <t>JPG, GIF ou PNG</t>
-        </is>
-      </c>
-      <c r="K351" t="inlineStr">
         <is>
           <t>https://support.google.com/google-ads/answer/17091270</t>
         </is>

</xml_diff>

<commit_message>
Update Meta Single Image/Video with full official per-placement specs
The generic "1080x1080 (1:1), placement pode variar" was inaccurate —
the real official specs (from Meta's ads guide, pasted directly by
the user) show Feed/Explore use 4:5 and Stories/Reels use 9:16 across
both Facebook and Instagram; 1:1 isn't the current recommendation
for any of these placements. Replaced with the full per-placement
breakdown (Facebook Feed/Stories/Reels, Instagram Feed/Stories/
Reels/Explore) covering aspect ratio, resolution, minimum dimensions,
tolerance, and copy character limits (primary text/headline) for
each — kept as one row per format (Single Image, Single Video),
condensed by placement, matching the same approach used for Uber's
multi-phase specs.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011oqQvDMfneVTKoco4dHUSc
</commit_message>
<xml_diff>
--- a/data/base-formatos.xlsx
+++ b/data/base-formatos.xlsx
@@ -11144,12 +11144,12 @@
       </c>
       <c r="G209" t="inlineStr">
         <is>
-          <t>1080x1080 (1:1) ou 1080x1350 (4:5) recomendado; placement pode variar</t>
+          <t>FACEBOOK — Feed: 4:5, 1440x1800 (mín. 600px largura, mín. 750px altura), tolerância 3%, texto principal 50-150c, título 27c; Stories: 9:16, 1440x2560 (mín. 500px largura), tolerância 1%, texto principal 125c, título 40c; Reels: 9:16, 1440x2560 (mín. 600x600px), tolerância 3%, texto principal 40c, título 55c. INSTAGRAM — Feed: 4:5, 1440x1800 (mín. 500px largura; proporção mín. 400x500, máx. 191x100), tolerância 1%, texto principal 125c, título 40c, máx. 30 hashtags; Stories: 9:16, 1440x2560 (mín. 500px largura), tolerância 1%, texto principal 125c; Reels: 9:16, 1440x2560 (mín. 500px largura), tolerância 1%, texto principal 44c; Explorar: 4:5, 1440x1800 (mín. 500px largura; proporção mín. 400x500, máx. 191x100), tolerância 1%, texto principal 125c, título 40c, máx. 30 hashtags.</t>
         </is>
       </c>
       <c r="H209" t="inlineStr">
         <is>
-          <t>1:1 ou 4:5</t>
+          <t>4:5 ou 9:16</t>
         </is>
       </c>
       <c r="I209" t="inlineStr">
@@ -11164,7 +11164,7 @@
       </c>
       <c r="K209" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/business/ads-guide</t>
+          <t>https://www.facebook.com/business/ads-guide/update</t>
         </is>
       </c>
     </row>
@@ -11201,12 +11201,12 @@
       </c>
       <c r="G210" t="inlineStr">
         <is>
-          <t>1080x1920 (9:16) Stories/Reels; 1080x1350 (4:5) Feed recomendado</t>
+          <t>FACEBOOK — Feed: 4:5, 1440x1800 (mín. 120x120px), 1s a 241min, texto principal 50-150c, título 27c; Stories: 9:16, 1440x2560 (mín. 250px largura), tolerância 1%, 1s a 3min, texto principal 125c, título 40c; Reels: 9:16 recomendado, 1440x2560, sem duração máxima, texto principal 40c, título 55c (sem legendas automáticas). INSTAGRAM — Feed: 9:16, 1080x1920 (mín. 250px largura), tolerância 1%, 1s a 60min, texto principal 125c, máx. 30 hashtags; Stories: 9:16, 1440x2560 (mín. 250px largura), tolerância 1%, 1s a 60min, texto principal 125c; Reels: 9:16, 1440x2560, 0 a 15min, mín. 250px largura (&lt;30s) ou 500px (≥30s), texto principal 44c. Todos: compressão H.264, píxeis quadrados, taxa de fotogramas fixa, áudio AAC estéreo ≥128 Kbps.</t>
         </is>
       </c>
       <c r="H210" t="inlineStr">
         <is>
-          <t>9:16 ou 4:5</t>
+          <t>4:5 ou 9:16</t>
         </is>
       </c>
       <c r="I210" t="inlineStr">
@@ -11216,12 +11216,12 @@
       </c>
       <c r="J210" t="inlineStr">
         <is>
-          <t>MP4, MOV</t>
+          <t>MP4, MOV ou GIF (Reels do Instagram: só MP4 ou MOV)</t>
         </is>
       </c>
       <c r="K210" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/business/ads-guide</t>
+          <t>https://www.facebook.com/business/ads-guide/update</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Meta Carousel with full official per-placement specs
Same treatment as Single Image/Video: replaced the generic "1080x1080,
placement pode variar" with the real per-placement breakdown from
Meta's ads guide — Facebook Feed/Stories/Reels and Instagram
Feed/Stories/Reels each have different aspect ratios, card count
ranges, and whether video is supported at all (Facebook Stories and
both Reels placements are image-only for Carousel).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011oqQvDMfneVTKoco4dHUSc
</commit_message>
<xml_diff>
--- a/data/base-formatos.xlsx
+++ b/data/base-formatos.xlsx
@@ -11030,27 +11030,27 @@
       </c>
       <c r="G207" t="inlineStr">
         <is>
-          <t>1080x1080 recomendado (1:1); placement pode variar</t>
+          <t>FACEBOOK — Feed: 1:1, 1080x1080 mín. (imagem ou vídeo), 2 a 10 cartões, tolerância 3%, texto principal 80c, título 20c, descrição 18c, URL obrigatório; Stories: 1:1 recomendado, 1080x1920 mín. (só imagem, sem suporte a vídeo), 3 a 10 cartões, largura mín. 500px, texto principal 125c, título 40c, URL obrigatório; Reels: 9:16, 1080x1920 mín. (só imagem), 2 a 10 cartões, largura mín. 500px, altura mín. 262px, tolerância 1%, texto principal 40c. INSTAGRAM — Feed: 4:5 (carrosséis só de imagem) ou 1:1 (se tiver vídeo), 1080x1080 mín., 2 a 10 cartões, tolerância 1%, texto principal 125c, máx. 30 hashtags, URL obrigatório; Stories: 9:16, 1080x1920 mín. (imagem ou vídeo), 2 a 10 cartões, tolerância 1%, texto principal 125c, título 40c, URL obrigatório; Reels: 9:16, 1080x1080 mín. (só imagem), 2 a 10 cartões, tolerância 1%.</t>
         </is>
       </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t>1:1</t>
+          <t>1:1 ou 4:5 ou 9:16</t>
         </is>
       </c>
       <c r="I207" t="inlineStr">
         <is>
-          <t>Imagem 30 MB; vídeo 4 GB</t>
+          <t>Imagem: 30 MB por cartão (todos os placements). Vídeo (só Feed do Facebook e Instagram, e Stories do Instagram): 4 GB por cartão; duração — Feed Facebook 1s-240min, Feed Instagram 1s-2min, Stories Instagram 1s-15s.</t>
         </is>
       </c>
       <c r="J207" t="inlineStr">
         <is>
-          <t>JPG/PNG ou MP4/MOV por cartão</t>
+          <t>JPG ou PNG (todos os placements); MP4/MOV/GIF também aceite em Feed Facebook, Feed Instagram e Stories Instagram</t>
         </is>
       </c>
       <c r="K207" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/business/ads-guide</t>
+          <t>https://www.facebook.com/business/ads-guide/update</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add a Copies column, separate it from Dimensão
Dimensão had become a catch-all for both real dimensions and copy
character limits (headline/body/CTA/hashtag counts), which made it
hard to read at a glance. Added a new "Copies" column and moved all
text/copy constraints there across the 14 rows that had them mixed
in — Facebook, Instagram (Single Image/Video/Carousel/Collection),
Google (In-Feed Video, Demand Gen Carousel, Responsive Search Ads,
Video Action Campaigns), and the two DV360 rows with compound specs
(Native Ad, Uber Journey Ad). Dimensão now holds only actual
dimensions/ratios/durations. Also moved video encoding notes
(H.264/AAC compression details) out of Dimensão into Tipo de
Ficheiro, where they belong. Shown as a new column in the Biblioteca
de Formatos and the Excel export, right after Tipo de Ficheiro.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011oqQvDMfneVTKoco4dHUSc
</commit_message>
<xml_diff>
--- a/data/base-formatos.xlsx
+++ b/data/base-formatos.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K349"/>
+  <dimension ref="A1:L349"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="18.08984375" customWidth="1" style="2" min="1" max="1"/>
@@ -513,6 +513,11 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
+          <t>Copies</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
           <t>Link</t>
         </is>
       </c>
@@ -563,7 +568,7 @@
           <t>JPG ou PNG</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>https://publicidade.impresa.pt/onlinespecs/billboard.html</t>
         </is>
@@ -615,7 +620,7 @@
           <t>JPG</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>https://publicidade.impresa.pt/onlinespecs/cube.html</t>
         </is>
@@ -667,7 +672,7 @@
           <t>GIF, JPEG ou PNG</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>https://publicidade.impresa.pt/onlinespecs/floorad.html</t>
         </is>
@@ -724,7 +729,7 @@
           <t>HTML, JPG, PNG ou GIF</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>https://publicidade.impresa.pt/onlinespecs/halfpage.html</t>
         </is>
@@ -771,7 +776,7 @@
           <t>JPG</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>https://publicidade.impresa.pt/onlinespecs/headerxl.html</t>
         </is>
@@ -823,7 +828,7 @@
           <t>JPG</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>https://publicidade.impresa.pt/onlinespecs/hero.html</t>
         </is>
@@ -880,7 +885,7 @@
           <t>JPG ou PNG</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>https://publicidade.impresa.pt/onlinespecs/in-article.html</t>
         </is>
@@ -937,7 +942,7 @@
           <t>HTML, JPG ou GIF</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>https://publicidade.impresa.pt/onlinespecs/interscroller.html</t>
         </is>
@@ -994,7 +999,7 @@
           <t>JPG ou PNG</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>https://publicidade.impresa.pt/onlinespecs/interstitial.html</t>
         </is>
@@ -1046,7 +1051,7 @@
           <t>HTML, JPG, PNG ou GIF</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>https://publicidade.impresa.pt/onlinespecs/mrec.html</t>
         </is>
@@ -1098,7 +1103,7 @@
           <t>MP4</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="L12" t="inlineStr">
         <is>
           <t>https://publicidade.impresa.pt/onlinespecs/mrec_video.html</t>
         </is>
@@ -1155,7 +1160,7 @@
           <t>JPG</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>https://publicidade.impresa.pt/onlinespecs/pushdown.html</t>
         </is>
@@ -1212,7 +1217,7 @@
           <t>JPG</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="L14" t="inlineStr">
         <is>
           <t>https://publicidade.impresa.pt/onlinespecs/opendoor.html</t>
         </is>
@@ -1269,7 +1274,7 @@
           <t>MP4</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="L15" t="inlineStr">
         <is>
           <t>https://publicidade.impresa.pt/onlinespecs/video-instream.html</t>
         </is>
@@ -1326,7 +1331,7 @@
           <t>MP4</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
+      <c r="L16" t="inlineStr">
         <is>
           <t>https://publicidade.impresa.pt/onlinespecs/video-outstream.html</t>
         </is>
@@ -1378,7 +1383,7 @@
           <t>JPG, GIF ou PNG</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
+      <c r="L17" t="inlineStr">
         <is>
           <t>https://mediacapitalcomercial.pt/format/billboard/</t>
         </is>
@@ -1435,7 +1440,7 @@
           <t>PNG</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr">
+      <c r="L18" t="inlineStr">
         <is>
           <t>https://mediacapitalcomercial.pt/format/billboard-xl/</t>
         </is>
@@ -1492,7 +1497,7 @@
           <t>JPEG, PNG ou GIF</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
+      <c r="L19" t="inlineStr">
         <is>
           <t>https://mediacapitalcomercial.pt/format/carrossel-incontent/</t>
         </is>
@@ -1549,7 +1554,7 @@
           <t>JPEG, PNG ou GIF</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr">
+      <c r="L20" t="inlineStr">
         <is>
           <t>https://mediacapitalcomercial.pt/format/carrossel-top/</t>
         </is>
@@ -1606,7 +1611,7 @@
           <t>JPEG</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr">
+      <c r="L21" t="inlineStr">
         <is>
           <t>https://mediacapitalcomercial.pt/format/dossier/</t>
         </is>
@@ -1663,7 +1668,7 @@
           <t>JPEG, PNG ou GIF</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr">
+      <c r="L22" t="inlineStr">
         <is>
           <t>https://mediacapitalcomercial.pt/format/full-frame/</t>
         </is>
@@ -1720,7 +1725,7 @@
           <t>HTML + Imagens</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr">
+      <c r="L23" t="inlineStr">
         <is>
           <t>https://mediacapitalcomercial.pt/format/halfpage/</t>
         </is>
@@ -1777,7 +1782,7 @@
           <t>JPG, GIF ou PNG</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr">
+      <c r="L24" t="inlineStr">
         <is>
           <t>https://mediacapitalcomercial.pt/format/interscroller/</t>
         </is>
@@ -1834,7 +1839,7 @@
           <t>HTML + Imagens</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr">
+      <c r="L25" t="inlineStr">
         <is>
           <t>https://mediacapitalcomercial.pt/format/intro-desktop/</t>
         </is>
@@ -1886,7 +1891,7 @@
           <t>JPEG, PNG ou GIF</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr">
+      <c r="L26" t="inlineStr">
         <is>
           <t>https://mediacapitalcomercial.pt/format/intro-splash/</t>
         </is>
@@ -1943,7 +1948,7 @@
           <t>JPEG, PNG ou GIF</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr">
+      <c r="L27" t="inlineStr">
         <is>
           <t>https://mediacapitalcomercial.pt/format/l-frame/</t>
         </is>
@@ -1995,7 +2000,7 @@
           <t>HTML + Imagens</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr">
+      <c r="L28" t="inlineStr">
         <is>
           <t>https://mediacapitalcomercial.pt/format/leaderboard/</t>
         </is>
@@ -2047,7 +2052,7 @@
           <t>Imagens (S, M, L e XL)</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr">
+      <c r="L29" t="inlineStr">
         <is>
           <t>https://mediacapitalcomercial.pt/format/megabillboard/</t>
         </is>
@@ -2099,7 +2104,7 @@
           <t>HTML + Imagens</t>
         </is>
       </c>
-      <c r="K30" t="inlineStr">
+      <c r="L30" t="inlineStr">
         <is>
           <t>https://mediacapitalcomercial.pt/format/mrec/</t>
         </is>
@@ -2156,7 +2161,7 @@
           <t>JPEG</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr">
+      <c r="L31" t="inlineStr">
         <is>
           <t>https://mediacapitalcomercial.pt/format/native/</t>
         </is>
@@ -2213,7 +2218,7 @@
           <t>JPG, GIF ou PNG</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr">
+      <c r="L32" t="inlineStr">
         <is>
           <t>https://mediacapitalcomercial.pt/format/open-door/</t>
         </is>
@@ -2260,7 +2265,7 @@
           <t>MP4</t>
         </is>
       </c>
-      <c r="K33" t="inlineStr">
+      <c r="L33" t="inlineStr">
         <is>
           <t>https://mediacapitalcomercial.pt/format/outstream/</t>
         </is>
@@ -2307,7 +2312,7 @@
           <t>Imagens</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr">
+      <c r="L34" t="inlineStr">
         <is>
           <t>https://mediacapitalcomercial.pt/format/pageflip/</t>
         </is>
@@ -2359,7 +2364,7 @@
           <t>JPEG, PNG ou GIF + Copies</t>
         </is>
       </c>
-      <c r="K35" t="inlineStr">
+      <c r="L35" t="inlineStr">
         <is>
           <t>https://mediacapitalcomercial.pt/format/pop-in/</t>
         </is>
@@ -2411,7 +2416,7 @@
           <t>JPG ou PNG</t>
         </is>
       </c>
-      <c r="K36" t="inlineStr">
+      <c r="L36" t="inlineStr">
         <is>
           <t>https://mediacapitalcomercial.pt/format/post-social-media/</t>
         </is>
@@ -2468,7 +2473,7 @@
           <t>MP4</t>
         </is>
       </c>
-      <c r="K37" t="inlineStr">
+      <c r="L37" t="inlineStr">
         <is>
           <t>https://mediacapitalcomercial.pt/format/pre-roll/</t>
         </is>
@@ -2525,7 +2530,7 @@
           <t>MP4</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr">
+      <c r="L38" t="inlineStr">
         <is>
           <t>https://mediacapitalcomercial.pt/format/7668/</t>
         </is>
@@ -2582,7 +2587,7 @@
           <t>JPG</t>
         </is>
       </c>
-      <c r="K39" t="inlineStr">
+      <c r="L39" t="inlineStr">
         <is>
           <t>https://mediacapitalcomercial.pt/format/push-down/</t>
         </is>
@@ -2639,7 +2644,7 @@
           <t>MP4 ou MOV</t>
         </is>
       </c>
-      <c r="K40" t="inlineStr">
+      <c r="L40" t="inlineStr">
         <is>
           <t>https://mediacapitalcomercial.pt/format/reel-social-media/</t>
         </is>
@@ -2691,7 +2696,7 @@
           <t>MP4 ou MOV</t>
         </is>
       </c>
-      <c r="K41" t="inlineStr">
+      <c r="L41" t="inlineStr">
         <is>
           <t>https://mediacapitalcomercial.pt/format/side-frame/</t>
         </is>
@@ -2733,7 +2738,7 @@
           <t>Link post Facebook ou Instagram</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr">
+      <c r="L42" t="inlineStr">
         <is>
           <t>https://mediacapitalcomercial.pt/format/social-card/</t>
         </is>
@@ -2785,7 +2790,7 @@
           <t>JPEG, PNG ou GIF</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr">
+      <c r="L43" t="inlineStr">
         <is>
           <t>https://mediacapitalcomercial.pt/format/splash/</t>
         </is>
@@ -2842,7 +2847,7 @@
           <t>MP4 ou MOV</t>
         </is>
       </c>
-      <c r="K44" t="inlineStr">
+      <c r="L44" t="inlineStr">
         <is>
           <t>https://mediacapitalcomercial.pt/format/story-social-media/</t>
         </is>
@@ -2894,7 +2899,7 @@
           <t>JPG, GIF ou PNG</t>
         </is>
       </c>
-      <c r="K45" t="inlineStr">
+      <c r="L45" t="inlineStr">
         <is>
           <t>https://mediacapitalcomercial.pt/format/brand-day-takeover/</t>
         </is>
@@ -2951,7 +2956,7 @@
           <t>PNG</t>
         </is>
       </c>
-      <c r="K46" t="inlineStr">
+      <c r="L46" t="inlineStr">
         <is>
           <t>https://mediacapitalcomercial.pt/format/ticker/</t>
         </is>
@@ -3008,7 +3013,7 @@
           <t>MP4</t>
         </is>
       </c>
-      <c r="K47" t="inlineStr">
+      <c r="L47" t="inlineStr">
         <is>
           <t>https://mediacapitalcomercial.pt/format/vertical-video/</t>
         </is>
@@ -3055,7 +3060,7 @@
           <t>MP4</t>
         </is>
       </c>
-      <c r="K48" t="inlineStr">
+      <c r="L48" t="inlineStr">
         <is>
           <t>https://mediacapitalcomercial.pt/format/videowall/</t>
         </is>
@@ -3107,7 +3112,7 @@
           <t>HTML / MP4</t>
         </is>
       </c>
-      <c r="K49" t="inlineStr">
+      <c r="L49" t="inlineStr">
         <is>
           <t>https://www.medialivreboostsolutions.pt/adspecs/cornerad/</t>
         </is>
@@ -3159,7 +3164,7 @@
           <t>HTML, JPEG, PNG ou GIF</t>
         </is>
       </c>
-      <c r="K50" t="inlineStr">
+      <c r="L50" t="inlineStr">
         <is>
           <t>https://www.medialivreboostsolutions.pt/adspecs/floorad/</t>
         </is>
@@ -3216,7 +3221,7 @@
           <t>HTML, JPEG, PNG ou GIF / MP4</t>
         </is>
       </c>
-      <c r="K51" t="inlineStr">
+      <c r="L51" t="inlineStr">
         <is>
           <t>https://www.medialivreboostsolutions.pt/adspecs/half-page/</t>
         </is>
@@ -3273,7 +3278,7 @@
           <t>JPEG, PNG ou GIF / MP4 ou WEBM</t>
         </is>
       </c>
-      <c r="K52" t="inlineStr">
+      <c r="L52" t="inlineStr">
         <is>
           <t>https://www.medialivreboostsolutions.pt/adspecs/incontent/</t>
         </is>
@@ -3330,7 +3335,7 @@
           <t>JPEG, PNG ou GIF / MP4 ou WEBM</t>
         </is>
       </c>
-      <c r="K53" t="inlineStr">
+      <c r="L53" t="inlineStr">
         <is>
           <t>https://www.medialivreboostsolutions.pt/adspecs/intro/</t>
         </is>
@@ -3382,7 +3387,7 @@
           <t>JPEG, PNG ou GIF / MP4 ou WEBM</t>
         </is>
       </c>
-      <c r="K54" t="inlineStr">
+      <c r="L54" t="inlineStr">
         <is>
           <t>https://www.medialivreboostsolutions.pt/adspecs/layer/</t>
         </is>
@@ -3434,7 +3439,7 @@
           <t>HTML, JPEG, PNG ou GIF</t>
         </is>
       </c>
-      <c r="K55" t="inlineStr">
+      <c r="L55" t="inlineStr">
         <is>
           <t>https://www.medialivreboostsolutions.pt/adspecs/leaderboard/</t>
         </is>
@@ -3486,7 +3491,7 @@
           <t>HTML, JPG, PNG ou GIF</t>
         </is>
       </c>
-      <c r="K56" t="inlineStr">
+      <c r="L56" t="inlineStr">
         <is>
           <t>https://www.medialivreboostsolutions.pt/adspecs/masthead/</t>
         </is>
@@ -3538,7 +3543,7 @@
           <t>HTML, JPG, PNG ou GIF</t>
         </is>
       </c>
-      <c r="K57" t="inlineStr">
+      <c r="L57" t="inlineStr">
         <is>
           <t>https://www.medialivreboostsolutions.pt/adspecs/masthead-sticky-companion/</t>
         </is>
@@ -3585,7 +3590,7 @@
           <t>JPG ou PNG</t>
         </is>
       </c>
-      <c r="K58" t="inlineStr">
+      <c r="L58" t="inlineStr">
         <is>
           <t>https://www.medialivreboostsolutions.pt/adspecs/moldura/</t>
         </is>
@@ -3637,7 +3642,7 @@
           <t>HTML, JPEG, PNG ou GIF</t>
         </is>
       </c>
-      <c r="K59" t="inlineStr">
+      <c r="L59" t="inlineStr">
         <is>
           <t>https://www.medialivreboostsolutions.pt/adspecs/m-rec/</t>
         </is>
@@ -3694,7 +3699,7 @@
           <t>JPG, GIF ou PNG / MP4</t>
         </is>
       </c>
-      <c r="K60" t="inlineStr">
+      <c r="L60" t="inlineStr">
         <is>
           <t>https://www.medialivreboostsolutions.pt/adspecs/open-door/</t>
         </is>
@@ -3746,7 +3751,7 @@
           <t>260 KB</t>
         </is>
       </c>
-      <c r="K61" t="inlineStr">
+      <c r="L61" t="inlineStr">
         <is>
           <t>https://www.medialivreboostsolutions.pt/adspecs/peel-off/</t>
         </is>
@@ -3803,7 +3808,7 @@
           <t>MP4 ou FLV</t>
         </is>
       </c>
-      <c r="K62" t="inlineStr">
+      <c r="L62" t="inlineStr">
         <is>
           <t>https://www.medialivreboostsolutions.pt/adspecs/pre-roll/</t>
         </is>
@@ -3840,7 +3845,7 @@
           <t>Showcase Rich Media</t>
         </is>
       </c>
-      <c r="K63" t="inlineStr">
+      <c r="L63" t="inlineStr">
         <is>
           <t>https://www.medialivreboostsolutions.pt/adspecs/showcase-richmedia/</t>
         </is>
@@ -3877,7 +3882,7 @@
           <t>Sideticker</t>
         </is>
       </c>
-      <c r="K64" t="inlineStr">
+      <c r="L64" t="inlineStr">
         <is>
           <t>https://www.medialivreboostsolutions.pt/adspecs/sideticker/</t>
         </is>
@@ -3914,7 +3919,7 @@
           <t>Slash</t>
         </is>
       </c>
-      <c r="K65" t="inlineStr">
+      <c r="L65" t="inlineStr">
         <is>
           <t>https://www.medialivreboostsolutions.pt/adspecs/slash/</t>
         </is>
@@ -3951,7 +3956,7 @@
           <t>Topo Extensivel</t>
         </is>
       </c>
-      <c r="K66" t="inlineStr">
+      <c r="L66" t="inlineStr">
         <is>
           <t>https://www.medialivreboostsolutions.pt/adspecs/topo-extensivel/</t>
         </is>
@@ -3998,7 +4003,7 @@
           <t>MP4</t>
         </is>
       </c>
-      <c r="K67" t="inlineStr">
+      <c r="L67" t="inlineStr">
         <is>
           <t>https://formatos.observador.pt/audio-desktop.html</t>
         </is>
@@ -4050,7 +4055,7 @@
           <t>JPG, PNG ou GIF</t>
         </is>
       </c>
-      <c r="K68" t="inlineStr">
+      <c r="L68" t="inlineStr">
         <is>
           <t>https://formatos.observador.pt/nl-desktop.html</t>
         </is>
@@ -4107,7 +4112,7 @@
           <t>JPG, PNG ou GIF</t>
         </is>
       </c>
-      <c r="K69" t="inlineStr">
+      <c r="L69" t="inlineStr">
         <is>
           <t>https://formatos.observador.pt/carrossel-desktop.html</t>
         </is>
@@ -4164,7 +4169,7 @@
           <t>JPG, PNG ou GIF</t>
         </is>
       </c>
-      <c r="K70" t="inlineStr">
+      <c r="L70" t="inlineStr">
         <is>
           <t>https://formatos.observador.pt/compare-desktop.html</t>
         </is>
@@ -4221,7 +4226,7 @@
           <t>JPG, PNG ou GIF</t>
         </is>
       </c>
-      <c r="K71" t="inlineStr">
+      <c r="L71" t="inlineStr">
         <is>
           <t>https://formatos.observador.pt/flipper-desktop.html</t>
         </is>
@@ -4278,7 +4283,7 @@
           <t>JPG, PNG ou GIF / HTML</t>
         </is>
       </c>
-      <c r="K72" t="inlineStr">
+      <c r="L72" t="inlineStr">
         <is>
           <t>https://formatos.observador.pt/halfpage-desktop.html</t>
         </is>
@@ -4330,7 +4335,7 @@
           <t>JPG, PNG ou GIF</t>
         </is>
       </c>
-      <c r="K73" t="inlineStr">
+      <c r="L73" t="inlineStr">
         <is>
           <t>https://formatos.observador.pt/header_xl-desktop.html</t>
         </is>
@@ -4382,7 +4387,7 @@
           <t>JPG, PNG ou GIF / HTML</t>
         </is>
       </c>
-      <c r="K74" t="inlineStr">
+      <c r="L74" t="inlineStr">
         <is>
           <t>https://formatos.observador.pt/interstitial-desktop.html</t>
         </is>
@@ -4434,7 +4439,7 @@
           <t>GIF ou WEBM</t>
         </is>
       </c>
-      <c r="K75" t="inlineStr">
+      <c r="L75" t="inlineStr">
         <is>
           <t>https://formatos.observador.pt/intro-dinamic-desktop.html</t>
         </is>
@@ -4481,7 +4486,7 @@
           <t>PDF</t>
         </is>
       </c>
-      <c r="K76" t="inlineStr">
+      <c r="L76" t="inlineStr">
         <is>
           <t>https://formatos.observador.pt/intro-folheto-desktop.html</t>
         </is>
@@ -4533,7 +4538,7 @@
           <t>JPG, PNG ou GIF / HTML</t>
         </is>
       </c>
-      <c r="K77" t="inlineStr">
+      <c r="L77" t="inlineStr">
         <is>
           <t>https://formatos.observador.pt/manchete-desktop.html</t>
         </is>
@@ -4585,7 +4590,7 @@
           <t>JPG, PNG ou GIF / HTML</t>
         </is>
       </c>
-      <c r="K78" t="inlineStr">
+      <c r="L78" t="inlineStr">
         <is>
           <t>https://formatos.observador.pt/mrec-desktop.html</t>
         </is>
@@ -4632,7 +4637,7 @@
           <t>JPG, PNG ou GIF / MP4 ou WEBM</t>
         </is>
       </c>
-      <c r="K79" t="inlineStr">
+      <c r="L79" t="inlineStr">
         <is>
           <t>https://formatos.observador.pt/opendoor-desktop.html</t>
         </is>
@@ -4689,7 +4694,7 @@
           <t>MP4</t>
         </is>
       </c>
-      <c r="K80" t="inlineStr">
+      <c r="L80" t="inlineStr">
         <is>
           <t>https://formatos.observador.pt/outstream-desktop.html</t>
         </is>
@@ -4746,7 +4751,7 @@
           <t>JPG, PNG ou GIF</t>
         </is>
       </c>
-      <c r="K81" t="inlineStr">
+      <c r="L81" t="inlineStr">
         <is>
           <t>https://formatos.observador.pt/pell-off-desktop.html</t>
         </is>
@@ -4803,7 +4808,7 @@
           <t>MP4</t>
         </is>
       </c>
-      <c r="K82" t="inlineStr">
+      <c r="L82" t="inlineStr">
         <is>
           <t>https://formatos.observador.pt/pre-roll-desktop.html</t>
         </is>
@@ -4855,7 +4860,7 @@
           <t>JPG, PNG ou GIF</t>
         </is>
       </c>
-      <c r="K83" t="inlineStr">
+      <c r="L83" t="inlineStr">
         <is>
           <t>https://formatos.observador.pt/skin-desktop.html</t>
         </is>
@@ -4907,7 +4912,7 @@
           <t>JPG, PNG ou GIF</t>
         </is>
       </c>
-      <c r="K84" t="inlineStr">
+      <c r="L84" t="inlineStr">
         <is>
           <t>https://formatos.observador.pt/sticky-dynamic-mobile.html</t>
         </is>
@@ -4959,7 +4964,7 @@
           <t>JPG, PNG ou GIF</t>
         </is>
       </c>
-      <c r="K85" t="inlineStr">
+      <c r="L85" t="inlineStr">
         <is>
           <t>https://formatos.observador.pt/sticky-footer-desktop.html</t>
         </is>
@@ -5016,7 +5021,7 @@
           <t>JPG, PNG ou GIF / MP4</t>
         </is>
       </c>
-      <c r="K86" t="inlineStr">
+      <c r="L86" t="inlineStr">
         <is>
           <t>https://formatos.observador.pt/sticky-to-intro-desktop.html</t>
         </is>
@@ -5073,7 +5078,7 @@
           <t>JPG, PNG ou GIF</t>
         </is>
       </c>
-      <c r="K87" t="inlineStr">
+      <c r="L87" t="inlineStr">
         <is>
           <t>https://formatos.observador.pt/twinad-desktop.html</t>
         </is>
@@ -5130,7 +5135,7 @@
           <t>JPG ou PNG</t>
         </is>
       </c>
-      <c r="K88" t="inlineStr">
+      <c r="L88" t="inlineStr">
         <is>
           <t>https://comunique.publico.pt/publicidade/formatos/ad-selector.html</t>
         </is>
@@ -5182,7 +5187,7 @@
           <t>HTML, JPG, PNG ou GIF</t>
         </is>
       </c>
-      <c r="K89" t="inlineStr">
+      <c r="L89" t="inlineStr">
         <is>
           <t>https://comunique.publico.pt/publicidade/formatos/barra-topo.html</t>
         </is>
@@ -5234,7 +5239,7 @@
           <t>HTML, JPG, PNG ou GIF / Video</t>
         </is>
       </c>
-      <c r="K90" t="inlineStr">
+      <c r="L90" t="inlineStr">
         <is>
           <t>https://comunique.publico.pt/publicidade/formatos/barra-topo-extensivel.html</t>
         </is>
@@ -5286,7 +5291,7 @@
           <t>HTML, JPG, PNG ou GIF / Video</t>
         </is>
       </c>
-      <c r="K91" t="inlineStr">
+      <c r="L91" t="inlineStr">
         <is>
           <t>https://comunique.publico.pt/publicidade/formatos/billboard.html</t>
         </is>
@@ -5338,7 +5343,7 @@
           <t>JPG ou PNG</t>
         </is>
       </c>
-      <c r="K92" t="inlineStr">
+      <c r="L92" t="inlineStr">
         <is>
           <t>https://comunique.publico.pt/publicidade/formatos/cubo-mrec.html</t>
         </is>
@@ -5390,7 +5395,7 @@
           <t>HTML</t>
         </is>
       </c>
-      <c r="K93" t="inlineStr">
+      <c r="L93" t="inlineStr">
         <is>
           <t>https://comunique.publico.pt/publicidade/formatos/floorad.html</t>
         </is>
@@ -5447,7 +5452,7 @@
           <t>JPG ou PNG</t>
         </is>
       </c>
-      <c r="K94" t="inlineStr">
+      <c r="L94" t="inlineStr">
         <is>
           <t>https://comunique.publico.pt/publicidade/formatos/gallery-flip.html</t>
         </is>
@@ -5504,7 +5509,7 @@
           <t>HTML, JPG, PNG ou GIF / Video</t>
         </is>
       </c>
-      <c r="K95" t="inlineStr">
+      <c r="L95" t="inlineStr">
         <is>
           <t>https://comunique.publico.pt/publicidade/formatos/halfpage.html</t>
         </is>
@@ -5561,7 +5566,7 @@
           <t>HTML, JPG, PNG ou GIF / Video</t>
         </is>
       </c>
-      <c r="K96" t="inlineStr">
+      <c r="L96" t="inlineStr">
         <is>
           <t>https://comunique.publico.pt/publicidade/formatos/interstitial.html</t>
         </is>
@@ -5613,7 +5618,7 @@
           <t>HTML, JPG, PNG ou GIF / Video</t>
         </is>
       </c>
-      <c r="K97" t="inlineStr">
+      <c r="L97" t="inlineStr">
         <is>
           <t>https://comunique.publico.pt/publicidade/formatos/mrec.html</t>
         </is>
@@ -5665,7 +5670,7 @@
           <t>JPG ou PNG</t>
         </is>
       </c>
-      <c r="K98" t="inlineStr">
+      <c r="L98" t="inlineStr">
         <is>
           <t>https://comunique.publico.pt/publicidade/formatos/newsletter.html</t>
         </is>
@@ -5717,7 +5722,7 @@
           <t>JPG / Video</t>
         </is>
       </c>
-      <c r="K99" t="inlineStr">
+      <c r="L99" t="inlineStr">
         <is>
           <t>https://comunique.publico.pt/publicidade/formatos/opendoor.html</t>
         </is>
@@ -5774,7 +5779,7 @@
           <t>JPG, PNG ou GIF</t>
         </is>
       </c>
-      <c r="K100" t="inlineStr">
+      <c r="L100" t="inlineStr">
         <is>
           <t>https://comunique.publico.pt/publicidade/formatos/parallax.html</t>
         </is>
@@ -5831,7 +5836,7 @@
           <t>JPG ou PNG</t>
         </is>
       </c>
-      <c r="K101" t="inlineStr">
+      <c r="L101" t="inlineStr">
         <is>
           <t>https://comunique.publico.pt/publicidade/formatos/prisma-halfpage.html</t>
         </is>
@@ -5888,7 +5893,7 @@
           <t>JPG ou PNG</t>
         </is>
       </c>
-      <c r="K102" t="inlineStr">
+      <c r="L102" t="inlineStr">
         <is>
           <t>https://comunique.publico.pt/publicidade/formatos/scratch-.html</t>
         </is>
@@ -5945,7 +5950,7 @@
           <t>JPG ou PNG</t>
         </is>
       </c>
-      <c r="K103" t="inlineStr">
+      <c r="L103" t="inlineStr">
         <is>
           <t>https://comunique.publico.pt/publicidade/formatos/shopping-ads-.html</t>
         </is>
@@ -6002,7 +6007,7 @@
           <t>JPG</t>
         </is>
       </c>
-      <c r="K104" t="inlineStr">
+      <c r="L104" t="inlineStr">
         <is>
           <t>https://comunique.publico.pt/publicidade/formatos/slidedoorvideo.html</t>
         </is>
@@ -6049,7 +6054,7 @@
           <t>JPEG, JPG ou PNG</t>
         </is>
       </c>
-      <c r="K105" t="inlineStr">
+      <c r="L105" t="inlineStr">
         <is>
           <t>https://comunique.publico.pt/publicidade/formatos/slidervideo.html</t>
         </is>
@@ -6101,7 +6106,7 @@
           <t>JPG, PNG ou GIF / Video para a área expandida</t>
         </is>
       </c>
-      <c r="K106" t="inlineStr">
+      <c r="L106" t="inlineStr">
         <is>
           <t>https://comunique.publico.pt/publicidade/formatos/xxl.html</t>
         </is>
@@ -6148,7 +6153,7 @@
           <t>JPG ou PNG</t>
         </is>
       </c>
-      <c r="K107" t="inlineStr">
+      <c r="L107" t="inlineStr">
         <is>
           <t>https://comunique.publico.pt/publicidade/formatos/galeria_header.html</t>
         </is>
@@ -6200,7 +6205,7 @@
           <t>HTML</t>
         </is>
       </c>
-      <c r="K108" t="inlineStr">
+      <c r="L108" t="inlineStr">
         <is>
           <t>https://comunique.publico.pt/publicidade/formatos/twinad.html</t>
         </is>
@@ -6257,7 +6262,7 @@
           <t>MP4 ou WEBM</t>
         </is>
       </c>
-      <c r="K109" t="inlineStr">
+      <c r="L109" t="inlineStr">
         <is>
           <t>https://comunique.publico.pt/publicidade/formatos/incontent.html</t>
         </is>
@@ -6314,7 +6319,7 @@
           <t>MP4 ou WEBM</t>
         </is>
       </c>
-      <c r="K110" t="inlineStr">
+      <c r="L110" t="inlineStr">
         <is>
           <t>https://comunique.publico.pt/publicidade/formatos/pre-roll.html</t>
         </is>
@@ -6366,7 +6371,7 @@
           <t>JPG ou PNG</t>
         </is>
       </c>
-      <c r="K111" t="inlineStr">
+      <c r="L111" t="inlineStr">
         <is>
           <t>https://support.teads.tv/support/solutions/articles/36000278437-cube-3d-viewable-display</t>
         </is>
@@ -6423,7 +6428,7 @@
           <t>JPG ou PNG</t>
         </is>
       </c>
-      <c r="K112" t="inlineStr">
+      <c r="L112" t="inlineStr">
         <is>
           <t>https://saleshouse.sapo.pt/formatos.html#format-app_install_native_outbrain</t>
         </is>
@@ -6470,7 +6475,7 @@
           <t>MPEG, MP3, WAV, ou OGG</t>
         </is>
       </c>
-      <c r="K113" t="inlineStr">
+      <c r="L113" t="inlineStr">
         <is>
           <t>https://ads.spotify.com/en-US/ad-specs/audio-ad-specs/</t>
         </is>
@@ -6517,7 +6522,7 @@
           <t>MP3</t>
         </is>
       </c>
-      <c r="K114" t="inlineStr">
+      <c r="L114" t="inlineStr">
         <is>
           <t>https://saleshouse.sapo.pt/formatos.html#format-audio_preroll_midroll_postroll</t>
         </is>
@@ -6564,7 +6569,7 @@
           <t>MP3</t>
         </is>
       </c>
-      <c r="K115" t="inlineStr">
+      <c r="L115" t="inlineStr">
         <is>
           <t>https://saleshouse.sapo.pt/formatos.html#format-audio_preroll_midroll_postroll</t>
         </is>
@@ -6611,7 +6616,7 @@
           <t>MP3</t>
         </is>
       </c>
-      <c r="K116" t="inlineStr">
+      <c r="L116" t="inlineStr">
         <is>
           <t>https://saleshouse.sapo.pt/formatos.html#format-audio_preroll_midroll_postroll</t>
         </is>
@@ -6663,7 +6668,7 @@
           <t>WEBP</t>
         </is>
       </c>
-      <c r="K117" t="inlineStr">
+      <c r="L117" t="inlineStr">
         <is>
           <t>https://saleshouse.sapo.pt/formatos.html#format-billboard_1a_2a_posicao</t>
         </is>
@@ -6720,7 +6725,7 @@
           <t>WEBP</t>
         </is>
       </c>
-      <c r="K118" t="inlineStr">
+      <c r="L118" t="inlineStr">
         <is>
           <t>https://saleshouse.sapo.pt/formatos.html#format-billboard_carousel</t>
         </is>
@@ -6767,7 +6772,7 @@
           <t>200 KB</t>
         </is>
       </c>
-      <c r="K119" t="inlineStr">
+      <c r="L119" t="inlineStr">
         <is>
           <t>https://saleshouse.sapo.pt/formatos.html#format-billboard_iab</t>
         </is>
@@ -6819,7 +6824,7 @@
           <t>WEBP</t>
         </is>
       </c>
-      <c r="K120" t="inlineStr">
+      <c r="L120" t="inlineStr">
         <is>
           <t>https://saleshouse.sapo.pt/formatos.html#format-billboard</t>
         </is>
@@ -6856,7 +6861,7 @@
           <t>Branded Content</t>
         </is>
       </c>
-      <c r="K121" t="inlineStr">
+      <c r="L121" t="inlineStr">
         <is>
           <t>https://saleshouse.sapo.pt/formatos.html#format-artigos_content_marketing</t>
         </is>
@@ -6913,7 +6918,7 @@
           <t>JPG, PNG ou GIF</t>
         </is>
       </c>
-      <c r="K122" t="inlineStr">
+      <c r="L122" t="inlineStr">
         <is>
           <t>https://saleshouse.sapo.pt/formatos.html#format-capa_falsa</t>
         </is>
@@ -6965,7 +6970,7 @@
           <t>JPG ou PNG</t>
         </is>
       </c>
-      <c r="K123" t="inlineStr">
+      <c r="L123" t="inlineStr">
         <is>
           <t>https://support.teads.tv/support/solutions/articles/36000206459-carousel-square,  https://support.teads.tv/support/solutions/articles/36000206458-carousel-landscape, https://support.teads.tv/support/solutions/articles/36000552432-carousel-vertical-</t>
         </is>
@@ -7017,7 +7022,7 @@
           <t>JPG ou PNG</t>
         </is>
       </c>
-      <c r="K124" t="inlineStr">
+      <c r="L124" t="inlineStr">
         <is>
           <t>https://www.outbrain.com/help/ads-specs/#carousel</t>
         </is>
@@ -7133,7 +7138,7 @@
           <t>WEBP</t>
         </is>
       </c>
-      <c r="K127" t="inlineStr">
+      <c r="L127" t="inlineStr">
         <is>
           <t>https://saleshouse.sapo.pt/formatos.html#format-companion_banner_resumo_artigo</t>
         </is>
@@ -7190,7 +7195,7 @@
           <t>PNG</t>
         </is>
       </c>
-      <c r="K128" t="inlineStr">
+      <c r="L128" t="inlineStr">
         <is>
           <t>https://saleshouse.sapo.pt/formatos.html#format-countdown</t>
         </is>
@@ -7343,7 +7348,7 @@
           <t>JPG, PNG ou GIF</t>
         </is>
       </c>
-      <c r="K132" t="inlineStr">
+      <c r="L132" t="inlineStr">
         <is>
           <t>https://saleshouse.sapo.pt/formatos.html#format-display_standard_cpc_surf</t>
         </is>
@@ -7395,7 +7400,7 @@
           <t>JPG ou PNG</t>
         </is>
       </c>
-      <c r="K133" t="inlineStr">
+      <c r="L133" t="inlineStr">
         <is>
           <t>https://support.teads.tv/support/solutions/articles/36000278434-drag-drop-viewable-display</t>
         </is>
@@ -7447,7 +7452,7 @@
           <t>JPG ou PNG</t>
         </is>
       </c>
-      <c r="K134" t="inlineStr">
+      <c r="L134" t="inlineStr">
         <is>
           <t>https://support.teads.tv/support/solutions/articles/36000552435-flip-flow-viewable-display</t>
         </is>
@@ -7499,7 +7504,7 @@
           <t>JPG ou PNG</t>
         </is>
       </c>
-      <c r="K135" t="inlineStr">
+      <c r="L135" t="inlineStr">
         <is>
           <t>https://support.teads.tv/support/solutions/articles/36000206460-flow-square, https://support.teads.tv/support/solutions/articles/36000206461-flow-landscape</t>
         </is>
@@ -7556,7 +7561,7 @@
           <t>JPG, PNG ou GIF / MP4 ou WEBM</t>
         </is>
       </c>
-      <c r="K136" t="inlineStr">
+      <c r="L136" t="inlineStr">
         <is>
           <t>https://saleshouse.sapo.pt/formatos.html#format-halfpage, https://saleshouse.sapo.pt/formatos.html#format-halfpage_video</t>
         </is>
@@ -7613,7 +7618,7 @@
           <t>JPG, PNG ou GIF</t>
         </is>
       </c>
-      <c r="K137" t="inlineStr">
+      <c r="L137" t="inlineStr">
         <is>
           <t>https://saleshouse.sapo.pt/formatos.html#format-halfpage_flip</t>
         </is>
@@ -7894,7 +7899,7 @@
           <t>JPG / MOV ou MP4</t>
         </is>
       </c>
-      <c r="K145" t="inlineStr">
+      <c r="L145" t="inlineStr">
         <is>
           <t>https://ads.spotify.com/en-SG/ad-experiences/display-homepage-takeover-ads-specs/</t>
         </is>
@@ -7951,7 +7956,7 @@
           <t>JPG ou PNG</t>
         </is>
       </c>
-      <c r="K146" t="inlineStr">
+      <c r="L146" t="inlineStr">
         <is>
           <t>https://support.teads.tv/support/solutions/articles/36000278440-hover-viewable-display</t>
         </is>
@@ -8008,7 +8013,7 @@
           <t>JPG ou PNG</t>
         </is>
       </c>
-      <c r="K147" t="inlineStr">
+      <c r="L147" t="inlineStr">
         <is>
           <t>https://ads.spotify.com/en-US/ad-specs/display-ad-specs/</t>
         </is>
@@ -8045,7 +8050,7 @@
           <t>In-feed Video (Spotify)</t>
         </is>
       </c>
-      <c r="K148" t="inlineStr">
+      <c r="L148" t="inlineStr">
         <is>
           <t>https://ads.spotify.com/en-US/ad-specs/in-feed-video-ad-specs/</t>
         </is>
@@ -8097,7 +8102,7 @@
           <t>JPG, PNG ou WEBP / MP4</t>
         </is>
       </c>
-      <c r="K149" t="inlineStr">
+      <c r="L149" t="inlineStr">
         <is>
           <t>https://www.adnami.io/specs/inline-midscroll-template</t>
         </is>
@@ -8154,7 +8159,7 @@
           <t>JPG ou PNG</t>
         </is>
       </c>
-      <c r="K150" t="inlineStr">
+      <c r="L150" t="inlineStr">
         <is>
           <t>https://support.teads.tv/support/solutions/articles/36000552431-interscroller-display</t>
         </is>
@@ -8211,7 +8216,7 @@
           <t>MP4</t>
         </is>
       </c>
-      <c r="K151" t="inlineStr">
+      <c r="L151" t="inlineStr">
         <is>
           <t>https://support.teads.tv/support/solutions/articles/36000552411-interscroller-video</t>
         </is>
@@ -8268,7 +8273,7 @@
           <t>JPG, PNG ou GIF</t>
         </is>
       </c>
-      <c r="K152" t="inlineStr">
+      <c r="L152" t="inlineStr">
         <is>
           <t>https://saleshouse.sapo.pt/formatos.html#format-intra</t>
         </is>
@@ -8320,7 +8325,7 @@
           <t>WEBP ou GIF</t>
         </is>
       </c>
-      <c r="K153" t="inlineStr">
+      <c r="L153" t="inlineStr">
         <is>
           <t>https://saleshouse.sapo.pt/formatos.html#format-intra_plus</t>
         </is>
@@ -8372,7 +8377,7 @@
           <t>HTML5 responsive com recursos em WEBP e MP4/WEBM, WEBP ou GIF (Leaderboard e Mobile)</t>
         </is>
       </c>
-      <c r="K154" t="inlineStr">
+      <c r="L154" t="inlineStr">
         <is>
           <t>https://saleshouse.sapo.pt/formatos.html#format-intra_plus_video</t>
         </is>
@@ -8429,7 +8434,7 @@
           <t>MP4 ou WEBP</t>
         </is>
       </c>
-      <c r="K155" t="inlineStr">
+      <c r="L155" t="inlineStr">
         <is>
           <t>https://saleshouse.sapo.pt/formatos.html#format-intra_video</t>
         </is>
@@ -8486,7 +8491,7 @@
           <t>MP4, WebM, ou MOV</t>
         </is>
       </c>
-      <c r="K156" t="inlineStr">
+      <c r="L156" t="inlineStr">
         <is>
           <t>https://ads.spotify.com/en-US/ad-specs/in-stream-video-ad-specs/</t>
         </is>
@@ -8523,7 +8528,7 @@
           <t>Landing Page</t>
         </is>
       </c>
-      <c r="K157" t="inlineStr">
+      <c r="L157" t="inlineStr">
         <is>
           <t>https://saleshouse.sapo.pt/formatos.html#format-microsites_landing_pages</t>
         </is>
@@ -8575,7 +8580,7 @@
           <t>WEBP</t>
         </is>
       </c>
-      <c r="K158" t="inlineStr">
+      <c r="L158" t="inlineStr">
         <is>
           <t>https://saleshouse.sapo.pt/formatos.html#format-leaderboard</t>
         </is>
@@ -8612,7 +8617,7 @@
           <t>Microsite</t>
         </is>
       </c>
-      <c r="K159" t="inlineStr">
+      <c r="L159" t="inlineStr">
         <is>
           <t>https://saleshouse.sapo.pt/formatos.html#format-microsites_landing_pages</t>
         </is>
@@ -8664,7 +8669,7 @@
           <t>WEBP</t>
         </is>
       </c>
-      <c r="K160" t="inlineStr">
+      <c r="L160" t="inlineStr">
         <is>
           <t>https://saleshouse.sapo.pt/formatos.html#format-mobile_banner</t>
         </is>
@@ -8716,7 +8721,7 @@
           <t>JPG, PNG ou GIF / MP4 ou WEBP</t>
         </is>
       </c>
-      <c r="K161" t="inlineStr">
+      <c r="L161" t="inlineStr">
         <is>
           <t>https://saleshouse.sapo.pt/formatos.html#format-mrec, https://saleshouse.sapo.pt/formatos.html#format-mrec_video</t>
         </is>
@@ -8768,7 +8773,7 @@
           <t>WEBP</t>
         </is>
       </c>
-      <c r="K162" t="inlineStr">
+      <c r="L162" t="inlineStr">
         <is>
           <t>https://saleshouse.sapo.pt/formatos.html#format-mrec_carousel</t>
         </is>
@@ -8825,7 +8830,7 @@
           <t>JPG ou PNG / MP4</t>
         </is>
       </c>
-      <c r="K163" t="inlineStr">
+      <c r="L163" t="inlineStr">
         <is>
           <t>https://support.teads.tv/support/solutions/articles/36000206444-video-overlay</t>
         </is>
@@ -8882,7 +8887,7 @@
           <t>JPG, PNG ou WEBP / MP4</t>
         </is>
       </c>
-      <c r="K164" t="inlineStr">
+      <c r="L164" t="inlineStr">
         <is>
           <t>https://www.adnami.io/specs/inline-expander-reel-template</t>
         </is>
@@ -8939,7 +8944,7 @@
           <t>JPG ou PNG</t>
         </is>
       </c>
-      <c r="K165" t="inlineStr">
+      <c r="L165" t="inlineStr">
         <is>
           <t>https://support.teads.tv/support/solutions/articles/36000278439-scratch-viewable-display</t>
         </is>
@@ -8991,7 +8996,7 @@
           <t>JPG ou PNG</t>
         </is>
       </c>
-      <c r="K166" t="inlineStr">
+      <c r="L166" t="inlineStr">
         <is>
           <t>https://support.teads.tv/support/solutions/articles/36000206455-scroller-square, https://support.teads.tv/support/solutions/articles/36000206453-scroller-landscape, https://support.teads.tv/support/solutions/articles/36000206456-scroller-vertical</t>
         </is>
@@ -9043,7 +9048,7 @@
           <t>JPG ou PNG</t>
         </is>
       </c>
-      <c r="K167" t="inlineStr">
+      <c r="L167" t="inlineStr">
         <is>
           <t>https://support.teads.tv/support/solutions/articles/36000434238-shoppable-carousel</t>
         </is>
@@ -9095,7 +9100,7 @@
           <t>JPG ou PNG / MP4</t>
         </is>
       </c>
-      <c r="K168" t="inlineStr">
+      <c r="L168" t="inlineStr">
         <is>
           <t>https://support.teads.tv/support/solutions/articles/36000206452-shoppable-square, https://support.teads.tv/support/solutions/articles/36000206451-shoppable-landscape, https://support.teads.tv/support/solutions/articles/36000552430-shoppable-vertical</t>
         </is>
@@ -9147,7 +9152,7 @@
           <t>JPG ou PNG</t>
         </is>
       </c>
-      <c r="K169" t="inlineStr">
+      <c r="L169" t="inlineStr">
         <is>
           <t>https://support.teads.tv/support/solutions/articles/36000208421-single-image</t>
         </is>
@@ -9194,7 +9199,7 @@
           <t>MP4</t>
         </is>
       </c>
-      <c r="K170" t="inlineStr">
+      <c r="L170" t="inlineStr">
         <is>
           <t>https://support.teads.tv/support/solutions/articles/36000297712-single-video</t>
         </is>
@@ -9236,7 +9241,7 @@
           <t>Várias, consultar o link</t>
         </is>
       </c>
-      <c r="K171" t="inlineStr">
+      <c r="L171" t="inlineStr">
         <is>
           <t>https://www.adnami.io/specs/fluid-skin-image-video</t>
         </is>
@@ -9293,7 +9298,7 @@
           <t>JPG ou PNG</t>
         </is>
       </c>
-      <c r="K172" t="inlineStr">
+      <c r="L172" t="inlineStr">
         <is>
           <t>https://support.teads.tv/support/solutions/articles/36000278442-slider-viewable-display</t>
         </is>
@@ -9350,7 +9355,7 @@
           <t>JPG ou PNG / MP4</t>
         </is>
       </c>
-      <c r="K173" t="inlineStr">
+      <c r="L173" t="inlineStr">
         <is>
           <t>https://support.teads.tv/support/solutions/articles/36000366159-inread-smart6</t>
         </is>
@@ -9392,7 +9397,7 @@
           <t>Várias, consultar o link</t>
         </is>
       </c>
-      <c r="K174" t="inlineStr">
+      <c r="L174" t="inlineStr">
         <is>
           <t>https://support.teads.tv/support/solutions/articles/36000238201-social-video-image-layout-1-, https://support.teads.tv/support/solutions/articles/36000238202-social-video-image-layout-2-</t>
         </is>
@@ -9434,7 +9439,7 @@
           <t>Várias, consultar o link</t>
         </is>
       </c>
-      <c r="K175" t="inlineStr">
+      <c r="L175" t="inlineStr">
         <is>
           <t>https://support.teads.tv/support/solutions/articles/36000297713-social-layout-1-performance, https://support.teads.tv/support/solutions/articles/36000297714-social-layout-2-performance</t>
         </is>
@@ -9476,7 +9481,7 @@
           <t>Várias, consultar o link</t>
         </is>
       </c>
-      <c r="K176" t="inlineStr">
+      <c r="L176" t="inlineStr">
         <is>
           <t>https://support.teads.tv/support/solutions/articles/36000238201-social-video-image-layout-1-, https://support.teads.tv/support/solutions/articles/36000238202-social-video-image-layout-2-</t>
         </is>
@@ -9528,7 +9533,7 @@
           <t>JPG ou PNG</t>
         </is>
       </c>
-      <c r="K177" t="inlineStr">
+      <c r="L177" t="inlineStr">
         <is>
           <t>https://support.teads.tv/support/solutions/articles/36000278441-spin-card-viewable-display</t>
         </is>
@@ -9580,7 +9585,7 @@
           <t>WEBP</t>
         </is>
       </c>
-      <c r="K178" t="inlineStr">
+      <c r="L178" t="inlineStr">
         <is>
           <t>https://saleshouse.sapo.pt/formatos.html#format-standard_green_ad</t>
         </is>
@@ -9637,7 +9642,7 @@
           <t>JPG ou PNG</t>
         </is>
       </c>
-      <c r="K179" t="inlineStr">
+      <c r="L179" t="inlineStr">
         <is>
           <t>https://www.outbrain.com/help/ads-specs/#native-image</t>
         </is>
@@ -9679,7 +9684,7 @@
           <t>Várias, consultar o link</t>
         </is>
       </c>
-      <c r="K180" t="inlineStr">
+      <c r="L180" t="inlineStr">
         <is>
           <t>https://support.teads.tv/support/solutions/articles/36000245892-stories-display-square, https://support.teads.tv/support/solutions/articles/36000245899-stories-display-vertical</t>
         </is>
@@ -9721,7 +9726,7 @@
           <t>Várias, consultar o link</t>
         </is>
       </c>
-      <c r="K181" t="inlineStr">
+      <c r="L181" t="inlineStr">
         <is>
           <t>https://support.teads.tv/support/solutions/articles/36000245891-stories-video-square, https://support.teads.tv/support/solutions/articles/36000245901-stories-video-vertical</t>
         </is>
@@ -9778,7 +9783,7 @@
           <t>JPG ou PNG</t>
         </is>
       </c>
-      <c r="K182" t="inlineStr">
+      <c r="L182" t="inlineStr">
         <is>
           <t>https://support.teads.tv/support/solutions/articles/36000278444-swipe-carousel-viewable-display</t>
         </is>
@@ -9835,7 +9840,7 @@
           <t>JPG, PNG ou WEBP</t>
         </is>
       </c>
-      <c r="K183" t="inlineStr">
+      <c r="L183" t="inlineStr">
         <is>
           <t>https://www.adnami.io/specs/topscroll-desktop-image</t>
         </is>
@@ -9877,7 +9882,7 @@
           <t>Várias, consultar o link</t>
         </is>
       </c>
-      <c r="K184" t="inlineStr">
+      <c r="L184" t="inlineStr">
         <is>
           <t>https://www.adnami.io/specs/fluid-product-carousel, https://www.adnami.io/specs/dynamic-hybrid-carousel, https://www.adnami.io/specs/product-lightbox</t>
         </is>
@@ -9929,7 +9934,7 @@
           <t>JPG ou WEBP</t>
         </is>
       </c>
-      <c r="K185" t="inlineStr">
+      <c r="L185" t="inlineStr">
         <is>
           <t>https://www.adnami.io/specs/topscroll-expand-template-image-desktop, https://www.adnami.io/specs/topscroll-expand-template-image-mobile</t>
         </is>
@@ -9981,7 +9986,7 @@
           <t>MP4</t>
         </is>
       </c>
-      <c r="K186" t="inlineStr">
+      <c r="L186" t="inlineStr">
         <is>
           <t>https://www.adnami.io/specs/topscroll-expand-template-desktop, https://www.adnami.io/specs/topscroll-expand-template-mobile</t>
         </is>
@@ -10033,7 +10038,7 @@
           <t>JPG ou WEBP</t>
         </is>
       </c>
-      <c r="K187" t="inlineStr">
+      <c r="L187" t="inlineStr">
         <is>
           <t>https://www.adnami.io/specs/prismo</t>
         </is>
@@ -10075,7 +10080,7 @@
           <t>Várias, consultar o link</t>
         </is>
       </c>
-      <c r="K188" t="inlineStr">
+      <c r="L188" t="inlineStr">
         <is>
           <t>https://www.adnami.io/specs/topscroll-desktop-video, https://www.adnami.io/specs/topscroll-mobile-video</t>
         </is>
@@ -10127,7 +10132,7 @@
           <t>WEBP</t>
         </is>
       </c>
-      <c r="K189" t="inlineStr">
+      <c r="L189" t="inlineStr">
         <is>
           <t>https://saleshouse.sapo.pt/formatos.html#format-twin_ad</t>
         </is>
@@ -10184,7 +10189,7 @@
           <t>MP4</t>
         </is>
       </c>
-      <c r="K190" t="inlineStr">
+      <c r="L190" t="inlineStr">
         <is>
           <t>https://saleshouse.sapo.pt/formatos.html#format-video_instream_preroll_midroll</t>
         </is>
@@ -10241,7 +10246,7 @@
           <t>MP4</t>
         </is>
       </c>
-      <c r="K191" t="inlineStr">
+      <c r="L191" t="inlineStr">
         <is>
           <t>https://saleshouse.sapo.pt/formatos.html#format-video_instream_preroll_midroll</t>
         </is>
@@ -10788,7 +10793,7 @@
           <t>JPG, PNG ou GIF</t>
         </is>
       </c>
-      <c r="K202" t="inlineStr">
+      <c r="L202" t="inlineStr">
         <is>
           <t>https://business.linkedin.com/advertise/ads/sponsored-content/single-image-ads-specs</t>
         </is>
@@ -11048,7 +11053,7 @@
           <t>PNG, JPEG; 2–5 imagens (non-Sales)</t>
         </is>
       </c>
-      <c r="K207" t="inlineStr">
+      <c r="L207" t="inlineStr">
         <is>
           <t>https://help.pinterest.com/en/business/article/pinterest-product-specs</t>
         </is>
@@ -11100,7 +11105,7 @@
           <t>PNG, JPEG, MP4/MOV/M4V + catálogo</t>
         </is>
       </c>
-      <c r="K208" t="inlineStr">
+      <c r="L208" t="inlineStr">
         <is>
           <t>https://help.pinterest.com/en/business/article/pinterest-product-specs</t>
         </is>
@@ -11157,7 +11162,7 @@
           <t>PNG, JPEG</t>
         </is>
       </c>
-      <c r="K209" t="inlineStr">
+      <c r="L209" t="inlineStr">
         <is>
           <t>https://help.pinterest.com/en/business/article/pinterest-product-specs</t>
         </is>
@@ -11214,7 +11219,7 @@
           <t>MP4, MOV, M4V</t>
         </is>
       </c>
-      <c r="K210" t="inlineStr">
+      <c r="L210" t="inlineStr">
         <is>
           <t>https://help.pinterest.com/en/business/article/pinterest-product-specs</t>
         </is>
@@ -11271,7 +11276,7 @@
           <t>JPG, PNG, GIF</t>
         </is>
       </c>
-      <c r="K211" t="inlineStr">
+      <c r="L211" t="inlineStr">
         <is>
           <t>https://www.business.reddit.com/advertise/ad-types/carousel-ads</t>
         </is>
@@ -11328,7 +11333,7 @@
           <t>JPG, PNG, GIF, MP4, MOV + rich text</t>
         </is>
       </c>
-      <c r="K212" t="inlineStr">
+      <c r="L212" t="inlineStr">
         <is>
           <t>https://www.business.reddit.com/advertise/ad-types/free-form</t>
         </is>
@@ -11385,7 +11390,7 @@
           <t>JPG, PNG, GIF (estático)</t>
         </is>
       </c>
-      <c r="K213" t="inlineStr">
+      <c r="L213" t="inlineStr">
         <is>
           <t>https://www.business.reddit.com/learning-hub/articles/reddit-image-ad-specs</t>
         </is>
@@ -11437,7 +11442,7 @@
           <t>Catálogo de produtos + JPG/PNG ou vídeo conforme configuração</t>
         </is>
       </c>
-      <c r="K214" t="inlineStr">
+      <c r="L214" t="inlineStr">
         <is>
           <t>https://www.business.reddit.com/advertise/ad-types</t>
         </is>
@@ -11489,7 +11494,7 @@
           <t>MP4, MOV</t>
         </is>
       </c>
-      <c r="K215" t="inlineStr">
+      <c r="L215" t="inlineStr">
         <is>
           <t>https://www.business.reddit.com/advertise/ad-types/video-ads</t>
         </is>
@@ -11541,7 +11546,7 @@
           <t>PNG (filtro estático), GIF (animado); Lens assets conforme Lens Studio</t>
         </is>
       </c>
-      <c r="K216" t="inlineStr">
+      <c r="L216" t="inlineStr">
         <is>
           <t>https://forbusiness.snapchat.com/advertising/ad-formats</t>
         </is>
@@ -11598,7 +11603,7 @@
           <t>JPG, PNG, MP4, MOV</t>
         </is>
       </c>
-      <c r="K217" t="inlineStr">
+      <c r="L217" t="inlineStr">
         <is>
           <t>https://forbusiness.snapchat.com/advertising/ad-formats</t>
         </is>
@@ -11655,7 +11660,7 @@
           <t>JPG, PNG, MP4, MOV + catálogo/produtos</t>
         </is>
       </c>
-      <c r="K218" t="inlineStr">
+      <c r="L218" t="inlineStr">
         <is>
           <t>https://forbusiness.snapchat.com/advertising/ad-formats</t>
         </is>
@@ -11712,7 +11717,7 @@
           <t>MP4, MOV (H.264)</t>
         </is>
       </c>
-      <c r="K219" t="inlineStr">
+      <c r="L219" t="inlineStr">
         <is>
           <t>https://forbusiness.snapchat.com/advertising/ad-formats</t>
         </is>
@@ -11769,7 +11774,7 @@
           <t>JPG, PNG</t>
         </is>
       </c>
-      <c r="K220" t="inlineStr">
+      <c r="L220" t="inlineStr">
         <is>
           <t>https://forbusiness.snapchat.com/advertising/ad-formats</t>
         </is>
@@ -11826,7 +11831,7 @@
           <t>MP4, MOV</t>
         </is>
       </c>
-      <c r="K221" t="inlineStr">
+      <c r="L221" t="inlineStr">
         <is>
           <t>https://forbusiness.snapchat.com/advertising/ad-formats</t>
         </is>
@@ -11883,7 +11888,7 @@
           <t>JPG, PNG, MP4, MOV</t>
         </is>
       </c>
-      <c r="K222" t="inlineStr">
+      <c r="L222" t="inlineStr">
         <is>
           <t>https://forbusiness.snapchat.com/advertising/ad-formats</t>
         </is>
@@ -11940,7 +11945,7 @@
           <t>PNG + assets de efeito conforme template</t>
         </is>
       </c>
-      <c r="K223" t="inlineStr">
+      <c r="L223" t="inlineStr">
         <is>
           <t>https://ads.tiktok.com/help/article/tiktok-branded-effect-asset-commercial-benefits-specs?lang=en</t>
         </is>
@@ -11992,7 +11997,7 @@
           <t>Vídeo de creator elegível / Spark Ads</t>
         </is>
       </c>
-      <c r="K224" t="inlineStr">
+      <c r="L224" t="inlineStr">
         <is>
           <t>https://ads.tiktok.com/resources/help/article/about-branded-mission?lang=pt</t>
         </is>
@@ -12049,7 +12054,7 @@
           <t>JPG/JPEG, PNG + MP3</t>
         </is>
       </c>
-      <c r="K225" t="inlineStr">
+      <c r="L225" t="inlineStr">
         <is>
           <t>https://ads.tiktok.com/resources/help/article/specifications-for-carousel-ads?lang=pt</t>
         </is>
@@ -12106,7 +12111,7 @@
           <t>MP4, MOV, MPEG, 3GP</t>
         </is>
       </c>
-      <c r="K226" t="inlineStr">
+      <c r="L226" t="inlineStr">
         <is>
           <t>https://ads.tiktok.com/resources/help/article/tiktok-reservation-topview?lang=pt</t>
         </is>
@@ -12158,7 +12163,7 @@
           <t>MP4, MOV / Spark Ads</t>
         </is>
       </c>
-      <c r="K227" t="inlineStr">
+      <c r="L227" t="inlineStr">
         <is>
           <t>https://ads.tiktok.com/help/article/split-testing-variables?lang=en</t>
         </is>
@@ -12215,7 +12220,7 @@
           <t>Vídeo orgânico autorizado ou MP4/MOV/MPEG/3GP</t>
         </is>
       </c>
-      <c r="K228" t="inlineStr">
+      <c r="L228" t="inlineStr">
         <is>
           <t>https://ads.tiktok.com/resources/help/article/tiktok-reservation-topview?lang=pt</t>
         </is>
@@ -12267,7 +12272,7 @@
           <t>MP4, MOV / Spark Ads</t>
         </is>
       </c>
-      <c r="K229" t="inlineStr">
+      <c r="L229" t="inlineStr">
         <is>
           <t>https://ads.tiktok.com/resources/help/article/topreach-ad-specifications?lang=pt</t>
         </is>
@@ -12324,7 +12329,7 @@
           <t>MP4, MOV, MPEG, 3GP</t>
         </is>
       </c>
-      <c r="K230" t="inlineStr">
+      <c r="L230" t="inlineStr">
         <is>
           <t>https://ads.tiktok.com/resources/help/article/tiktok-reservation-topview?lang=pt</t>
         </is>
@@ -12376,7 +12381,7 @@
           <t>MP4, MOV</t>
         </is>
       </c>
-      <c r="K231" t="inlineStr">
+      <c r="L231" t="inlineStr">
         <is>
           <t>https://business.x.com/en/help/campaign-setup/creative-ad-specifications</t>
         </is>
@@ -12433,7 +12438,7 @@
           <t>JPG, PNG; MP4/MOV para video carousel</t>
         </is>
       </c>
-      <c r="K232" t="inlineStr">
+      <c r="L232" t="inlineStr">
         <is>
           <t>https://business.x.com/en/help/campaign-setup/creative-ad-specifications</t>
         </is>
@@ -12490,7 +12495,7 @@
           <t>JPG, PNG + catálogo</t>
         </is>
       </c>
-      <c r="K233" t="inlineStr">
+      <c r="L233" t="inlineStr">
         <is>
           <t>https://business.x.com/en/help/campaign-setup/creative-ad-specifications</t>
         </is>
@@ -12542,7 +12547,7 @@
           <t>Feed/catálogo + JPG/PNG</t>
         </is>
       </c>
-      <c r="K234" t="inlineStr">
+      <c r="L234" t="inlineStr">
         <is>
           <t>https://business.x.com/en/help/campaign-setup/creative-ad-specifications</t>
         </is>
@@ -12599,7 +12604,7 @@
           <t>JPG, PNG</t>
         </is>
       </c>
-      <c r="K235" t="inlineStr">
+      <c r="L235" t="inlineStr">
         <is>
           <t>https://business.x.com/en/help/campaign-setup/creative-ad-specifications</t>
         </is>
@@ -12651,7 +12656,7 @@
           <t>JPG, PNG, MP4/MOV conforme takeover</t>
         </is>
       </c>
-      <c r="K236" t="inlineStr">
+      <c r="L236" t="inlineStr">
         <is>
           <t>https://business.x.com/en/help/campaign-setup/creative-ad-specifications</t>
         </is>
@@ -12703,7 +12708,7 @@
           <t>Texto/post + URL opcional</t>
         </is>
       </c>
-      <c r="K237" t="inlineStr">
+      <c r="L237" t="inlineStr">
         <is>
           <t>https://business.x.com/en/help/campaign-setup/creative-ad-specifications</t>
         </is>
@@ -12760,7 +12765,7 @@
           <t>MP4, MOV</t>
         </is>
       </c>
-      <c r="K238" t="inlineStr">
+      <c r="L238" t="inlineStr">
         <is>
           <t>https://business.x.com/en/help/campaign-setup/creative-ad-specifications</t>
         </is>
@@ -12812,7 +12817,7 @@
           <t>JPG, PNG, GIF</t>
         </is>
       </c>
-      <c r="K239" t="inlineStr">
+      <c r="L239" t="inlineStr">
         <is>
           <t>https://support.google.com/google-ads/answer/13676244</t>
         </is>
@@ -12864,7 +12869,7 @@
           <t>JPG, PNG, GIF</t>
         </is>
       </c>
-      <c r="K240" t="inlineStr">
+      <c r="L240" t="inlineStr">
         <is>
           <t>https://support.google.com/google-ads/answer/13676244</t>
         </is>
@@ -12916,7 +12921,7 @@
           <t>JPG, PNG, GIF</t>
         </is>
       </c>
-      <c r="K241" t="inlineStr">
+      <c r="L241" t="inlineStr">
         <is>
           <t>https://support.google.com/google-ads/answer/13676244</t>
         </is>
@@ -12973,7 +12978,7 @@
           <t>JPG, PNG, GIF</t>
         </is>
       </c>
-      <c r="K242" t="inlineStr">
+      <c r="L242" t="inlineStr">
         <is>
           <t>https://support.google.com/google-ads/answer/13676244</t>
         </is>
@@ -13025,7 +13030,7 @@
           <t>JPG, PNG, GIF</t>
         </is>
       </c>
-      <c r="K243" t="inlineStr">
+      <c r="L243" t="inlineStr">
         <is>
           <t>https://support.google.com/google-ads/answer/13676244</t>
         </is>
@@ -13082,7 +13087,7 @@
           <t>JPG, PNG</t>
         </is>
       </c>
-      <c r="K244" t="inlineStr">
+      <c r="L244" t="inlineStr">
         <is>
           <t>https://support.google.com/google-ads/answer/13676244</t>
         </is>
@@ -13139,7 +13144,7 @@
           <t>ZIP HTML5</t>
         </is>
       </c>
-      <c r="K245" t="inlineStr">
+      <c r="L245" t="inlineStr">
         <is>
           <t>https://support.google.com/google-ads/answer/13676244</t>
         </is>
@@ -13196,7 +13201,7 @@
           <t>MP4, MOV (upload via YouTube)</t>
         </is>
       </c>
-      <c r="K246" t="inlineStr">
+      <c r="L246" t="inlineStr">
         <is>
           <t>https://support.google.com/google-ads/answer/17091270</t>
         </is>
@@ -13253,7 +13258,7 @@
           <t>MP4, MOV</t>
         </is>
       </c>
-      <c r="K247" t="inlineStr">
+      <c r="L247" t="inlineStr">
         <is>
           <t>https://support.google.com/google-ads/answer/11462260</t>
         </is>
@@ -13310,7 +13315,7 @@
           <t>MP4, MOV</t>
         </is>
       </c>
-      <c r="K248" t="inlineStr">
+      <c r="L248" t="inlineStr">
         <is>
           <t>https://support.google.com/google-ads/answer/11462260</t>
         </is>
@@ -13362,7 +13367,7 @@
           <t>MP4, MOV</t>
         </is>
       </c>
-      <c r="K249" t="inlineStr">
+      <c r="L249" t="inlineStr">
         <is>
           <t>https://support.google.com/google-ads/answer/11462260</t>
         </is>
@@ -13401,7 +13406,7 @@
       </c>
       <c r="G250" t="inlineStr">
         <is>
-          <t>Horizontal 16:9: 1920x1080; Vertical 9:16: 1080x1920; Square 1:1: 1080x1080; 15 segundos recomendado. Texto — Título: 2 linhas, 40 caracteres cada; Descrição: 2 linhas, 35 caracteres cada.</t>
+          <t>Horizontal 16:9: 1920x1080; Vertical 9:16: 1080x1920; Square 1:1: 1080x1080; 15 segundos recomendado.</t>
         </is>
       </c>
       <c r="H250" t="inlineStr">
@@ -13420,6 +13425,11 @@
         </is>
       </c>
       <c r="K250" t="inlineStr">
+        <is>
+          <t>Título: 2 linhas, 40 caracteres cada; Descrição: 2 linhas, 35 caracteres cada.</t>
+        </is>
+      </c>
+      <c r="L250" t="inlineStr">
         <is>
           <t>https://support.google.com/google-ads/answer/17091270</t>
         </is>
@@ -13476,7 +13486,7 @@
           <t>MP4, MOV</t>
         </is>
       </c>
-      <c r="K251" t="inlineStr">
+      <c r="L251" t="inlineStr">
         <is>
           <t>https://support.google.com/google-ads/answer/17091270</t>
         </is>
@@ -13533,7 +13543,7 @@
           <t>MP4, MOV</t>
         </is>
       </c>
-      <c r="K252" t="inlineStr">
+      <c r="L252" t="inlineStr">
         <is>
           <t>https://support.google.com/google-ads/answer/17091270</t>
         </is>
@@ -13590,7 +13600,7 @@
           <t>JPG, PNG, GIF (não animado)</t>
         </is>
       </c>
-      <c r="K253" t="inlineStr">
+      <c r="L253" t="inlineStr">
         <is>
           <t>https://support.google.com/google-ads/answer/13704860</t>
         </is>
@@ -13642,7 +13652,7 @@
           <t>MP4, MOV</t>
         </is>
       </c>
-      <c r="K254" t="inlineStr">
+      <c r="L254" t="inlineStr">
         <is>
           <t>https://support.google.com/google-ads/answer/13704860</t>
         </is>
@@ -13681,7 +13691,7 @@
       </c>
       <c r="G255" t="inlineStr">
         <is>
-          <t>2 a 10 cartões, todos com a mesma proporção (1:1 ou 1.91:1); cada cartão com título até 40 caracteres</t>
+          <t>2 a 10 cartões, todos com a mesma proporção (1:1 ou 1.91:1)</t>
         </is>
       </c>
       <c r="I255" t="inlineStr">
@@ -13695,6 +13705,11 @@
         </is>
       </c>
       <c r="K255" t="inlineStr">
+        <is>
+          <t>Título por cartão: até 40 caracteres</t>
+        </is>
+      </c>
+      <c r="L255" t="inlineStr">
         <is>
           <t>https://support.google.com/google-ads/answer/13704860</t>
         </is>
@@ -14105,7 +14120,7 @@
           <t>MP4, MOV</t>
         </is>
       </c>
-      <c r="K268" t="inlineStr">
+      <c r="L268" t="inlineStr">
         <is>
           <t>https://support.google.com/google-ads/answer/17091270</t>
         </is>
@@ -14171,7 +14186,7 @@
       </c>
       <c r="G270" t="inlineStr">
         <is>
-          <t>IMAGEM — Logo: 100x100 a 2000x2000px (1:1); Imagem: 1200x627 a 2000x1047px (1.91:1); Imagem quadrada (opcional, obrigatória em Programmatic Guaranteed): 627x627 a 2000x2000px (1:1). VÍDEO — Logo: 100x100 a 2000x2000px (1:1); Cover image: altura mín 627px, máx 2000x1047px (1.91:1 recomendado — para mais inventário, criar criativos adicionais com 16:9, 4:3 ou 1:1); Vídeo: ficheiro fonte com a maior qualidade disponível. COPY (igual para imagem e vídeo) — Nome do anunciante: máx 25c; Headline: máx 25c (ou Long headline obrigatório se headline não usado); Long headline: máx 50c; Body text: máx 90c (ou Long body obrigatório se body não usado); Long body text: máx 150c; Landing page URL: máx 1024c; Caption URL: máx 30c; Call to action: máx 15c.</t>
+          <t>IMAGEM — Logo: 100x100 a 2000x2000px (1:1); Imagem: 1200x627 a 2000x1047px (1.91:1); Imagem quadrada (opcional, obrigatória em Programmatic Guaranteed): 627x627 a 2000x2000px (1:1). VÍDEO — Logo: 100x100 a 2000x2000px (1:1); Cover image: altura mín 627px, máx 2000x1047px (1.91:1 recomendado — para mais inventário, criar criativos adicionais com 16:9, 4:3 ou 1:1); Vídeo: ficheiro fonte com a maior qualidade disponível.</t>
         </is>
       </c>
       <c r="H270" t="inlineStr">
@@ -14190,6 +14205,11 @@
         </is>
       </c>
       <c r="K270" t="inlineStr">
+        <is>
+          <t>Igual para imagem e vídeo — Nome do anunciante: máx 25c; Headline: máx 25c (ou Long headline obrigatório se headline não usado); Long headline: máx 50c; Body text: máx 90c (ou Long body obrigatório se body não usado); Long body text: máx 150c; Landing page URL: máx 1024c; Caption URL: máx 30c; Call to action: máx 15c.</t>
+        </is>
+      </c>
+      <c r="L270" t="inlineStr">
         <is>
           <t>https://support.google.com/displayvideo/answer/7128458 | https://support.google.com/displayvideo/answer/7548780</t>
         </is>
@@ -14300,7 +14320,7 @@
           <t>MP4, MOV (upload via YouTube)</t>
         </is>
       </c>
-      <c r="K273" t="inlineStr">
+      <c r="L273" t="inlineStr">
         <is>
           <t>https://support.google.com/google-ads/answer/17091270</t>
         </is>
@@ -14357,7 +14377,7 @@
           <t>MP4, MOV (upload via YouTube)</t>
         </is>
       </c>
-      <c r="K274" t="inlineStr">
+      <c r="L274" t="inlineStr">
         <is>
           <t>https://support.google.com/google-ads/answer/17091270</t>
         </is>
@@ -14463,7 +14483,7 @@
           <t>MP4, MOV</t>
         </is>
       </c>
-      <c r="K277" t="inlineStr">
+      <c r="L277" t="inlineStr">
         <is>
           <t>https://support.google.com/google-ads/answer/11462260</t>
         </is>
@@ -14497,7 +14517,7 @@
       </c>
       <c r="G278" t="inlineStr">
         <is>
-          <t>DISPLAY — Pedido: 975x861, mín 1/máx 5 imagens (todas com logo e diferentes), copy: título máx 25c, corpo máx 52c; Espera: 420x420 ou 314x420, máx 1 imagem, copy: título máx 25c, CTA máx 15c; Viagem: 1146x393, mín 1/máx 5 imagens (todas com logo e diferentes), copy: título máx 25c, corpo máx 52c, CTA máx 15c. VIDEO (MP4, 16:9, altura mín 486px, largura mín 864px) — Pedido: 3 a 6 seg, copy: título máx 25c, corpo máx 52c; Espera: 6 a 60 seg, copy: título máx 25c, CTA máx 15c; Viagem: 6 a 60 seg, copy: título máx 25c, corpo máx 52c, CTA máx 15c. URL — Display: parametrizado, não parametrizado ou Click Tag (Click Tag só disponível nas fases de Espera e Viagem); Video: parametrizado, não parametrizado ou Click Tag (todas as fases).</t>
+          <t>DISPLAY — Pedido: 975x861, mín 1/máx 5 imagens (todas com logo e diferentes); Espera: 420x420 ou 314x420, máx 1 imagem; Viagem: 1146x393, mín 1/máx 5 imagens (todas com logo e diferentes). VIDEO (MP4, 16:9, altura mín 486px, largura mín 864px) — Pedido: 3 a 6 seg; Espera: 6 a 60 seg; Viagem: 6 a 60 seg.</t>
         </is>
       </c>
       <c r="H278" t="inlineStr">
@@ -14513,6 +14533,11 @@
       <c r="J278" t="inlineStr">
         <is>
           <t>Display: imagens. Video: MP4.</t>
+        </is>
+      </c>
+      <c r="K278" t="inlineStr">
+        <is>
+          <t>DISPLAY — Pedido: título máx 25c, corpo máx 52c; Espera: título máx 25c, CTA máx 15c; Viagem: título máx 25c, corpo máx 52c, CTA máx 15c. VIDEO — Pedido: título máx 25c, corpo máx 52c; Espera: título máx 25c, CTA máx 15c; Viagem: título máx 25c, corpo máx 52c, CTA máx 15c. URL — Display: parametrizado, não parametrizado ou Click Tag (só disponível nas fases de Espera e Viagem); Video: parametrizado, não parametrizado ou Click Tag (todas as fases).</t>
         </is>
       </c>
     </row>
@@ -14621,7 +14646,7 @@
           <t>MP4, MOV (upload via YouTube)</t>
         </is>
       </c>
-      <c r="K281" t="inlineStr">
+      <c r="L281" t="inlineStr">
         <is>
           <t>https://support.google.com/google-ads/answer/17091270</t>
         </is>
@@ -14673,7 +14698,7 @@
           <t>MP4, MOV</t>
         </is>
       </c>
-      <c r="K282" t="inlineStr">
+      <c r="L282" t="inlineStr">
         <is>
           <t>https://support.google.com/google-ads/answer/11462260</t>
         </is>
@@ -14725,7 +14750,7 @@
           <t>MP4, MOV</t>
         </is>
       </c>
-      <c r="K283" t="inlineStr">
+      <c r="L283" t="inlineStr">
         <is>
           <t>https://support.google.com/google-ads/answer/11462260</t>
         </is>
@@ -14777,7 +14802,7 @@
           <t>JPG ou PNG</t>
         </is>
       </c>
-      <c r="K284" t="inlineStr">
+      <c r="L284" t="inlineStr">
         <is>
           <t>https://publicidade.impresa.pt/onlinespecs/billboard.html</t>
         </is>
@@ -14829,7 +14854,7 @@
           <t>JPG, GIF ou PNG</t>
         </is>
       </c>
-      <c r="K285" t="inlineStr">
+      <c r="L285" t="inlineStr">
         <is>
           <t>https://mediacapitalcomercial.pt/format/billboard/</t>
         </is>
@@ -14881,7 +14906,7 @@
           <t>JPG, PNG ou GIF / HTML</t>
         </is>
       </c>
-      <c r="K286" t="inlineStr">
+      <c r="L286" t="inlineStr">
         <is>
           <t>https://formatos.observador.pt/manchete-desktop.html</t>
         </is>
@@ -14933,7 +14958,7 @@
           <t>HTML, JPG, PNG ou GIF / Video</t>
         </is>
       </c>
-      <c r="K287" t="inlineStr">
+      <c r="L287" t="inlineStr">
         <is>
           <t>https://comunique.publico.pt/publicidade/formatos/billboard.html</t>
         </is>
@@ -14980,7 +15005,7 @@
           <t>200 KB</t>
         </is>
       </c>
-      <c r="K288" t="inlineStr">
+      <c r="L288" t="inlineStr">
         <is>
           <t>https://saleshouse.sapo.pt/formatos.html#format-billboard_iab</t>
         </is>
@@ -15037,7 +15062,7 @@
           <t>HTML, JPG, PNG ou GIF</t>
         </is>
       </c>
-      <c r="K289" t="inlineStr">
+      <c r="L289" t="inlineStr">
         <is>
           <t>https://publicidade.impresa.pt/onlinespecs/halfpage.html</t>
         </is>
@@ -15094,7 +15119,7 @@
           <t>HTML + Imagens</t>
         </is>
       </c>
-      <c r="K290" t="inlineStr">
+      <c r="L290" t="inlineStr">
         <is>
           <t>https://mediacapitalcomercial.pt/format/halfpage/</t>
         </is>
@@ -15151,7 +15176,7 @@
           <t>HTML, JPEG, PNG ou GIF / MP4</t>
         </is>
       </c>
-      <c r="K291" t="inlineStr">
+      <c r="L291" t="inlineStr">
         <is>
           <t>https://www.medialivreboostsolutions.pt/adspecs/half-page/</t>
         </is>
@@ -15208,7 +15233,7 @@
           <t>JPG, PNG ou GIF / HTML</t>
         </is>
       </c>
-      <c r="K292" t="inlineStr">
+      <c r="L292" t="inlineStr">
         <is>
           <t>https://formatos.observador.pt/halfpage-desktop.html</t>
         </is>
@@ -15265,7 +15290,7 @@
           <t>HTML, JPG, PNG ou GIF / Video</t>
         </is>
       </c>
-      <c r="K293" t="inlineStr">
+      <c r="L293" t="inlineStr">
         <is>
           <t>https://comunique.publico.pt/publicidade/formatos/halfpage.html</t>
         </is>
@@ -15322,7 +15347,7 @@
           <t>JPG, PNG ou GIF / MP4 ou WEBM</t>
         </is>
       </c>
-      <c r="K294" t="inlineStr">
+      <c r="L294" t="inlineStr">
         <is>
           <t>https://saleshouse.sapo.pt/formatos.html#format-halfpage, https://saleshouse.sapo.pt/formatos.html#format-halfpage_video</t>
         </is>
@@ -15379,7 +15404,7 @@
           <t>JPG, PNG, GIF</t>
         </is>
       </c>
-      <c r="K295" t="inlineStr">
+      <c r="L295" t="inlineStr">
         <is>
           <t>https://support.google.com/google-ads/answer/13676244</t>
         </is>
@@ -15426,7 +15451,7 @@
           <t>JPG</t>
         </is>
       </c>
-      <c r="K296" t="inlineStr">
+      <c r="L296" t="inlineStr">
         <is>
           <t>https://publicidade.impresa.pt/onlinespecs/headerxl.html</t>
         </is>
@@ -15478,7 +15503,7 @@
           <t>HTML, JPG, PNG ou GIF</t>
         </is>
       </c>
-      <c r="K297" t="inlineStr">
+      <c r="L297" t="inlineStr">
         <is>
           <t>https://www.medialivreboostsolutions.pt/adspecs/masthead/</t>
         </is>
@@ -15530,7 +15555,7 @@
           <t>JPG, PNG ou GIF</t>
         </is>
       </c>
-      <c r="K298" t="inlineStr">
+      <c r="L298" t="inlineStr">
         <is>
           <t>https://formatos.observador.pt/header_xl-desktop.html</t>
         </is>
@@ -15619,7 +15644,7 @@
           <t>JPG ou PNG</t>
         </is>
       </c>
-      <c r="K300" t="inlineStr">
+      <c r="L300" t="inlineStr">
         <is>
           <t>https://publicidade.impresa.pt/onlinespecs/interstitial.html</t>
         </is>
@@ -15676,7 +15701,7 @@
           <t>HTML + Imagens</t>
         </is>
       </c>
-      <c r="K301" t="inlineStr">
+      <c r="L301" t="inlineStr">
         <is>
           <t>https://mediacapitalcomercial.pt/format/intro-desktop/</t>
         </is>
@@ -15733,7 +15758,7 @@
           <t>JPEG, PNG ou GIF / MP4 ou WEBM</t>
         </is>
       </c>
-      <c r="K302" t="inlineStr">
+      <c r="L302" t="inlineStr">
         <is>
           <t>https://www.medialivreboostsolutions.pt/adspecs/intro/</t>
         </is>
@@ -15785,7 +15810,7 @@
           <t>JPG, PNG ou GIF / HTML</t>
         </is>
       </c>
-      <c r="K303" t="inlineStr">
+      <c r="L303" t="inlineStr">
         <is>
           <t>https://formatos.observador.pt/interstitial-desktop.html</t>
         </is>
@@ -15842,7 +15867,7 @@
           <t>HTML, JPG, PNG ou GIF / Video</t>
         </is>
       </c>
-      <c r="K304" t="inlineStr">
+      <c r="L304" t="inlineStr">
         <is>
           <t>https://comunique.publico.pt/publicidade/formatos/interstitial.html</t>
         </is>
@@ -15899,7 +15924,7 @@
           <t>JPG, PNG ou GIF</t>
         </is>
       </c>
-      <c r="K305" t="inlineStr">
+      <c r="L305" t="inlineStr">
         <is>
           <t>https://saleshouse.sapo.pt/formatos.html#format-intra</t>
         </is>
@@ -15951,7 +15976,7 @@
           <t>HTML + Imagens</t>
         </is>
       </c>
-      <c r="K306" t="inlineStr">
+      <c r="L306" t="inlineStr">
         <is>
           <t>https://mediacapitalcomercial.pt/format/leaderboard/</t>
         </is>
@@ -16003,7 +16028,7 @@
           <t>HTML, JPEG, PNG ou GIF</t>
         </is>
       </c>
-      <c r="K307" t="inlineStr">
+      <c r="L307" t="inlineStr">
         <is>
           <t>https://www.medialivreboostsolutions.pt/adspecs/leaderboard/</t>
         </is>
@@ -16055,7 +16080,7 @@
           <t>HTML, JPG, PNG ou GIF</t>
         </is>
       </c>
-      <c r="K308" t="inlineStr">
+      <c r="L308" t="inlineStr">
         <is>
           <t>https://comunique.publico.pt/publicidade/formatos/barra-topo.html</t>
         </is>
@@ -16107,7 +16132,7 @@
           <t>WEBP</t>
         </is>
       </c>
-      <c r="K309" t="inlineStr">
+      <c r="L309" t="inlineStr">
         <is>
           <t>https://saleshouse.sapo.pt/formatos.html#format-leaderboard</t>
         </is>
@@ -16159,7 +16184,7 @@
           <t>JPG, PNG, GIF</t>
         </is>
       </c>
-      <c r="K310" t="inlineStr">
+      <c r="L310" t="inlineStr">
         <is>
           <t>https://support.google.com/google-ads/answer/13676244</t>
         </is>
@@ -16216,7 +16241,7 @@
           <t>JPG</t>
         </is>
       </c>
-      <c r="K311" t="inlineStr">
+      <c r="L311" t="inlineStr">
         <is>
           <t>https://publicidade.impresa.pt/onlinespecs/opendoor.html</t>
         </is>
@@ -16273,7 +16298,7 @@
           <t>JPG, GIF ou PNG</t>
         </is>
       </c>
-      <c r="K312" t="inlineStr">
+      <c r="L312" t="inlineStr">
         <is>
           <t>https://mediacapitalcomercial.pt/format/open-door/</t>
         </is>
@@ -16330,7 +16355,7 @@
           <t>JPG, GIF ou PNG / MP4</t>
         </is>
       </c>
-      <c r="K313" t="inlineStr">
+      <c r="L313" t="inlineStr">
         <is>
           <t>https://www.medialivreboostsolutions.pt/adspecs/open-door/</t>
         </is>
@@ -16377,7 +16402,7 @@
           <t>JPG, PNG ou GIF / MP4 ou WEBM</t>
         </is>
       </c>
-      <c r="K314" t="inlineStr">
+      <c r="L314" t="inlineStr">
         <is>
           <t>https://formatos.observador.pt/opendoor-desktop.html</t>
         </is>
@@ -16429,7 +16454,7 @@
           <t>JPG / Video</t>
         </is>
       </c>
-      <c r="K315" t="inlineStr">
+      <c r="L315" t="inlineStr">
         <is>
           <t>https://comunique.publico.pt/publicidade/formatos/opendoor.html</t>
         </is>
@@ -16486,7 +16511,7 @@
           <t>MP4, MOV</t>
         </is>
       </c>
-      <c r="K316" t="inlineStr">
+      <c r="L316" t="inlineStr">
         <is>
           <t>https://support.google.com/google-ads/answer/17091270</t>
         </is>
@@ -16543,7 +16568,7 @@
           <t>JPG, PNG ou GIF</t>
         </is>
       </c>
-      <c r="K317" t="inlineStr">
+      <c r="L317" t="inlineStr">
         <is>
           <t>https://comunique.publico.pt/publicidade/formatos/parallax.html</t>
         </is>
@@ -16590,7 +16615,7 @@
           <t>Imagens</t>
         </is>
       </c>
-      <c r="K318" t="inlineStr">
+      <c r="L318" t="inlineStr">
         <is>
           <t>https://mediacapitalcomercial.pt/format/pageflip/</t>
         </is>
@@ -16642,7 +16667,7 @@
           <t>260 KB</t>
         </is>
       </c>
-      <c r="K319" t="inlineStr">
+      <c r="L319" t="inlineStr">
         <is>
           <t>https://www.medialivreboostsolutions.pt/adspecs/peel-off/</t>
         </is>
@@ -16699,7 +16724,7 @@
           <t>JPG, PNG ou GIF</t>
         </is>
       </c>
-      <c r="K320" t="inlineStr">
+      <c r="L320" t="inlineStr">
         <is>
           <t>https://formatos.observador.pt/pell-off-desktop.html</t>
         </is>
@@ -16756,7 +16781,7 @@
           <t>MP4</t>
         </is>
       </c>
-      <c r="K321" t="inlineStr">
+      <c r="L321" t="inlineStr">
         <is>
           <t>https://mediacapitalcomercial.pt/format/pre-roll/</t>
         </is>
@@ -16813,7 +16838,7 @@
           <t>MP4 ou FLV</t>
         </is>
       </c>
-      <c r="K322" t="inlineStr">
+      <c r="L322" t="inlineStr">
         <is>
           <t>https://www.medialivreboostsolutions.pt/adspecs/pre-roll/</t>
         </is>
@@ -16870,7 +16895,7 @@
           <t>MP4</t>
         </is>
       </c>
-      <c r="K323" t="inlineStr">
+      <c r="L323" t="inlineStr">
         <is>
           <t>https://formatos.observador.pt/pre-roll-desktop.html</t>
         </is>
@@ -16927,7 +16952,7 @@
           <t>MP4 ou WEBM</t>
         </is>
       </c>
-      <c r="K324" t="inlineStr">
+      <c r="L324" t="inlineStr">
         <is>
           <t>https://comunique.publico.pt/publicidade/formatos/pre-roll.html</t>
         </is>
@@ -16984,7 +17009,7 @@
           <t>MP4</t>
         </is>
       </c>
-      <c r="K325" t="inlineStr">
+      <c r="L325" t="inlineStr">
         <is>
           <t>https://saleshouse.sapo.pt/formatos.html#format-video_instream_preroll_midroll</t>
         </is>
@@ -17036,7 +17061,7 @@
           <t>JPG, GIF ou PNG</t>
         </is>
       </c>
-      <c r="K326" t="inlineStr">
+      <c r="L326" t="inlineStr">
         <is>
           <t>https://mediacapitalcomercial.pt/format/brand-day-takeover/</t>
         </is>
@@ -17088,7 +17113,7 @@
           <t>JPG, PNG ou GIF / Video para a área expandida</t>
         </is>
       </c>
-      <c r="K327" t="inlineStr">
+      <c r="L327" t="inlineStr">
         <is>
           <t>https://comunique.publico.pt/publicidade/formatos/xxl.html</t>
         </is>
@@ -17172,7 +17197,7 @@
           <t>MP4, MOV</t>
         </is>
       </c>
-      <c r="K329" t="inlineStr">
+      <c r="L329" t="inlineStr">
         <is>
           <t>https://support.google.com/google-ads/answer/11462260</t>
         </is>
@@ -17261,7 +17286,7 @@
           <t>JPG, PNG</t>
         </is>
       </c>
-      <c r="K331" t="inlineStr">
+      <c r="L331" t="inlineStr">
         <is>
           <t>https://support.google.com/google-ads/answer/17091671</t>
         </is>
@@ -17318,7 +17343,7 @@
           <t>MP4, MOV</t>
         </is>
       </c>
-      <c r="K332" t="inlineStr">
+      <c r="L332" t="inlineStr">
         <is>
           <t>https://support.google.com/google-ads/answer/17091671</t>
         </is>
@@ -17375,7 +17400,7 @@
           <t>JPG, PNG</t>
         </is>
       </c>
-      <c r="K333" t="inlineStr">
+      <c r="L333" t="inlineStr">
         <is>
           <t>https://support.google.com/google-ads/answer/9748775</t>
         </is>
@@ -17432,7 +17457,7 @@
           <t>JPG, PNG</t>
         </is>
       </c>
-      <c r="K334" t="inlineStr">
+      <c r="L334" t="inlineStr">
         <is>
           <t>https://support.google.com/google-ads/answer/9748775</t>
         </is>
@@ -17489,7 +17514,7 @@
           <t>MP4, MOV</t>
         </is>
       </c>
-      <c r="K335" t="inlineStr">
+      <c r="L335" t="inlineStr">
         <is>
           <t>https://support.google.com/google-ads/answer/9748775</t>
         </is>
@@ -17546,7 +17571,7 @@
           <t>JPG, PNG</t>
         </is>
       </c>
-      <c r="K336" t="inlineStr">
+      <c r="L336" t="inlineStr">
         <is>
           <t>https://support.google.com/google-ads/answer/12437745</t>
         </is>
@@ -17603,7 +17628,7 @@
           <t>JPG, PNG</t>
         </is>
       </c>
-      <c r="K337" t="inlineStr">
+      <c r="L337" t="inlineStr">
         <is>
           <t>https://support.google.com/google-ads/answer/12437745</t>
         </is>
@@ -17642,7 +17667,7 @@
       </c>
       <c r="G338" t="inlineStr">
         <is>
-          <t>Só texto (sem imagem) — Títulos: até 30 caracteres, 1 a 15; Descrições: até 90 caracteres, 1 a 4</t>
+          <t>N/A (só texto, sem imagem)</t>
         </is>
       </c>
       <c r="I338" t="inlineStr">
@@ -17656,6 +17681,11 @@
         </is>
       </c>
       <c r="K338" t="inlineStr">
+        <is>
+          <t>Títulos: até 30 caracteres, 1 a 15; Descrições: até 90 caracteres, 1 a 4</t>
+        </is>
+      </c>
+      <c r="L338" t="inlineStr">
         <is>
           <t>https://support.google.com/google-ads/answer/7684791</t>
         </is>
@@ -17694,7 +17724,7 @@
       </c>
       <c r="G339" t="inlineStr">
         <is>
-          <t>Horizontal 16:9: 1920x1080; Vertical 9:16: 1080x1920; Square 1:1: 1080x1080; mín. 10 segundos. Texto — Título: 30c; Título longo: 90c; Descrição: 90c; CTA: 10c.</t>
+          <t>Horizontal 16:9: 1920x1080; Vertical 9:16: 1080x1920; Square 1:1: 1080x1080; mín. 10 segundos.</t>
         </is>
       </c>
       <c r="H339" t="inlineStr">
@@ -17713,6 +17743,11 @@
         </is>
       </c>
       <c r="K339" t="inlineStr">
+        <is>
+          <t>Título: 30c; Título longo: 90c; Descrição: 90c; CTA: 10c.</t>
+        </is>
+      </c>
+      <c r="L339" t="inlineStr">
         <is>
           <t>https://support.google.com/google-ads/answer/12066387</t>
         </is>
@@ -17769,7 +17804,7 @@
           <t>JPG, GIF ou PNG</t>
         </is>
       </c>
-      <c r="K340" t="inlineStr">
+      <c r="L340" t="inlineStr">
         <is>
           <t>https://support.google.com/google-ads/answer/17091270</t>
         </is>
@@ -17826,7 +17861,7 @@
           <t>JPG, GIF ou PNG</t>
         </is>
       </c>
-      <c r="K341" t="inlineStr">
+      <c r="L341" t="inlineStr">
         <is>
           <t>https://support.google.com/google-ads/answer/17091270</t>
         </is>
@@ -17865,7 +17900,7 @@
       </c>
       <c r="G342" t="inlineStr">
         <is>
-          <t>Feed: 4:5, 1440x1800 (mín. 600px largura, mín. 750px altura), tolerância 3%, texto principal 50-150c, título 27c; Stories: 9:16, 1440x2560 (mín. 500px largura), tolerância 1%, texto principal 125c, título 40c; Reels: 9:16, 1440x2560 (mín. 600x600px), tolerância 3%, texto principal 40c, título 55c.</t>
+          <t>Feed: 4:5, 1440x1800 (mín. 600px largura, mín. 750px altura), tolerância 3%; Stories: 9:16, 1440x2560 (mín. 500px largura), tolerância 1%; Reels: 9:16, 1440x2560 (mín. 600x600px), tolerância 3%.</t>
         </is>
       </c>
       <c r="H342" t="inlineStr">
@@ -17884,6 +17919,11 @@
         </is>
       </c>
       <c r="K342" t="inlineStr">
+        <is>
+          <t>Feed: texto principal 50-150c, título 27c; Stories: texto principal 125c, título 40c; Reels: texto principal 40c, título 55c.</t>
+        </is>
+      </c>
+      <c r="L342" t="inlineStr">
         <is>
           <t>https://www.facebook.com/business/ads-guide/update</t>
         </is>
@@ -17922,7 +17962,7 @@
       </c>
       <c r="G343" t="inlineStr">
         <is>
-          <t>Feed: 4:5, 1440x1800 (mín. 120x120px), 1s a 241min, texto principal 50-150c, título 27c; Stories: 9:16, 1440x2560 (mín. 250px largura), tolerância 1%, 1s a 3min, texto principal 125c, título 40c; Reels: 9:16 recomendado, 1440x2560, sem duração máxima, texto principal 40c, título 55c (sem legendas automáticas). Compressão H.264, píxeis quadrados, taxa de fotogramas fixa, áudio AAC estéreo ≥128 Kbps.</t>
+          <t>Feed: 4:5, 1440x1800 (mín. 120x120px), 1s a 241min; Stories: 9:16, 1440x2560 (mín. 250px largura), tolerância 1%, 1s a 3min; Reels: 9:16 recomendado, 1440x2560, sem duração máxima.</t>
         </is>
       </c>
       <c r="H343" t="inlineStr">
@@ -17937,10 +17977,15 @@
       </c>
       <c r="J343" t="inlineStr">
         <is>
-          <t>MP4, MOV ou GIF</t>
+          <t>MP4, MOV ou GIF. Compressão H.264, píxeis quadrados, taxa de fotogramas fixa, áudio AAC estéreo ≥128 Kbps.</t>
         </is>
       </c>
       <c r="K343" t="inlineStr">
+        <is>
+          <t>Feed: texto principal 50-150c, título 27c; Stories: texto principal 125c, título 40c; Reels: texto principal 40c, título 55c (sem legendas automáticas).</t>
+        </is>
+      </c>
+      <c r="L343" t="inlineStr">
         <is>
           <t>https://www.facebook.com/business/ads-guide/update</t>
         </is>
@@ -17979,7 +18024,7 @@
       </c>
       <c r="G344" t="inlineStr">
         <is>
-          <t>Feed: 1:1, 1080x1080 mín. (imagem ou vídeo), 2 a 10 cartões, tolerância 3%, texto principal 80c, título 20c, descrição 18c, URL obrigatório; Stories: 1:1 recomendado, 1080x1920 mín. (só imagem, sem suporte a vídeo), 3 a 10 cartões, largura mín. 500px, texto principal 125c, título 40c, URL obrigatório; Reels: 9:16, 1080x1920 mín. (só imagem), 2 a 10 cartões, largura mín. 500px, altura mín. 262px, tolerância 1%, texto principal 40c.</t>
+          <t>Feed: 1:1, 1080x1080 mín. (imagem ou vídeo), 2 a 10 cartões, tolerância 3%; Stories: 1:1 recomendado, 1080x1920 mín. (só imagem, sem suporte a vídeo), 3 a 10 cartões, largura mín. 500px; Reels: 9:16, 1080x1920 mín. (só imagem), 2 a 10 cartões, largura mín. 500px, altura mín. 262px, tolerância 1%.</t>
         </is>
       </c>
       <c r="H344" t="inlineStr">
@@ -17998,6 +18043,11 @@
         </is>
       </c>
       <c r="K344" t="inlineStr">
+        <is>
+          <t>Feed: texto principal 80c, título 20c, descrição 18c, URL obrigatório; Stories: texto principal 125c, título 40c, URL obrigatório; Reels: texto principal 40c.</t>
+        </is>
+      </c>
+      <c r="L344" t="inlineStr">
         <is>
           <t>https://www.facebook.com/business/ads-guide/update</t>
         </is>
@@ -18036,7 +18086,7 @@
       </c>
       <c r="G345" t="inlineStr">
         <is>
-          <t>Feed: 1.91:1 até 1:1, 1080x1080 mín. (capa: imagem ou vídeo) + 3 imagens de produto; Experiência Instantânea obrigatória; texto principal 125c, título 40c, URL obrigatório; Reels: 9:16 até 1:1, 1080x1080 mín.; requer Catálogo Advantage+ como fonte de conteúdo; texto principal 72c, título 10c, URL obrigatório; Experiência Instantânea obrigatória.</t>
+          <t>Feed: 1.91:1 até 1:1, 1080x1080 mín. (capa: imagem ou vídeo) + 3 imagens de produto, Experiência Instantânea obrigatória; Reels: 9:16 até 1:1, 1080x1080 mín., requer Catálogo Advantage+ como fonte de conteúdo, Experiência Instantânea obrigatória.</t>
         </is>
       </c>
       <c r="H345" t="inlineStr">
@@ -18055,6 +18105,11 @@
         </is>
       </c>
       <c r="K345" t="inlineStr">
+        <is>
+          <t>Feed: texto principal 125c, título 40c, URL obrigatório; Reels: texto principal 72c, título 10c, URL obrigatório.</t>
+        </is>
+      </c>
+      <c r="L345" t="inlineStr">
         <is>
           <t>https://www.facebook.com/business/ads-guide/update</t>
         </is>
@@ -18093,7 +18148,7 @@
       </c>
       <c r="G346" t="inlineStr">
         <is>
-          <t>Feed: 4:5, 1440x1800 (mín. 500px largura; proporção mín. 400x500, máx. 191x100), tolerância 1%, texto principal 125c, título 40c, máx. 30 hashtags; Stories: 9:16, 1440x2560 (mín. 500px largura), tolerância 1%, texto principal 125c; Reels: 9:16, 1440x2560 (mín. 500px largura), tolerância 1%, texto principal 44c; Explorar: 4:5, 1440x1800 (mín. 500px largura; proporção mín. 400x500, máx. 191x100), tolerância 1%, texto principal 125c, título 40c, máx. 30 hashtags.</t>
+          <t>Feed: 4:5, 1440x1800 (mín. 500px largura; proporção mín. 400x500, máx. 191x100), tolerância 1%; Stories: 9:16, 1440x2560 (mín. 500px largura), tolerância 1%; Reels: 9:16, 1440x2560 (mín. 500px largura), tolerância 1%; Explorar: 4:5, 1440x1800 (mín. 500px largura; proporção mín. 400x500, máx. 191x100), tolerância 1%.</t>
         </is>
       </c>
       <c r="H346" t="inlineStr">
@@ -18112,6 +18167,11 @@
         </is>
       </c>
       <c r="K346" t="inlineStr">
+        <is>
+          <t>Feed: texto principal 125c, título 40c, máx. 30 hashtags; Stories: texto principal 125c; Reels: texto principal 44c; Explorar: texto principal 125c, título 40c, máx. 30 hashtags.</t>
+        </is>
+      </c>
+      <c r="L346" t="inlineStr">
         <is>
           <t>https://www.facebook.com/business/ads-guide/update</t>
         </is>
@@ -18150,7 +18210,7 @@
       </c>
       <c r="G347" t="inlineStr">
         <is>
-          <t>Feed: 9:16, 1080x1920 (mín. 250px largura), tolerância 1%, 1s a 60min, texto principal 125c, máx. 30 hashtags; Stories: 9:16, 1440x2560 (mín. 250px largura), tolerância 1%, 1s a 60min, texto principal 125c; Reels: 9:16, 1440x2560, 0 a 15min, mín. 250px largura (&lt;30s) ou 500px (≥30s), texto principal 44c. Compressão H.264, píxeis quadrados, taxa de fotogramas fixa, áudio AAC estéreo ≥128 Kbps.</t>
+          <t>Feed: 9:16, 1080x1920 (mín. 250px largura), tolerância 1%, 1s a 60min; Stories: 9:16, 1440x2560 (mín. 250px largura), tolerância 1%, 1s a 60min; Reels: 9:16, 1440x2560, 0 a 15min, mín. 250px largura (&lt;30s) ou 500px (≥30s).</t>
         </is>
       </c>
       <c r="H347" t="inlineStr">
@@ -18165,10 +18225,15 @@
       </c>
       <c r="J347" t="inlineStr">
         <is>
-          <t>MP4, MOV ou GIF (Reels: só MP4 ou MOV)</t>
+          <t>MP4, MOV ou GIF (Reels: só MP4 ou MOV). Compressão H.264, píxeis quadrados, taxa de fotogramas fixa, áudio AAC estéreo ≥128 Kbps.</t>
         </is>
       </c>
       <c r="K347" t="inlineStr">
+        <is>
+          <t>Feed: texto principal 125c, máx. 30 hashtags; Stories: texto principal 125c; Reels: texto principal 44c.</t>
+        </is>
+      </c>
+      <c r="L347" t="inlineStr">
         <is>
           <t>https://www.facebook.com/business/ads-guide/update</t>
         </is>
@@ -18207,7 +18272,7 @@
       </c>
       <c r="G348" t="inlineStr">
         <is>
-          <t>Feed: 4:5 (carrosséis só de imagem) ou 1:1 (se tiver vídeo), 1080x1080 mín., 2 a 10 cartões, tolerância 1%, texto principal 125c, máx. 30 hashtags, URL obrigatório; Stories: 9:16, 1080x1920 mín. (imagem ou vídeo), 2 a 10 cartões, tolerância 1%, texto principal 125c, título 40c, URL obrigatório; Reels: 9:16, 1080x1080 mín. (só imagem), 2 a 10 cartões, tolerância 1%.</t>
+          <t>Feed: 4:5 (carrosséis só de imagem) ou 1:1 (se tiver vídeo), 1080x1080 mín., 2 a 10 cartões, tolerância 1%; Stories: 9:16, 1080x1920 mín. (imagem ou vídeo), 2 a 10 cartões, tolerância 1%; Reels: 9:16, 1080x1080 mín. (só imagem), 2 a 10 cartões, tolerância 1%.</t>
         </is>
       </c>
       <c r="H348" t="inlineStr">
@@ -18226,6 +18291,11 @@
         </is>
       </c>
       <c r="K348" t="inlineStr">
+        <is>
+          <t>Feed: texto principal 125c, máx. 30 hashtags, URL obrigatório; Stories: texto principal 125c, título 40c, URL obrigatório.</t>
+        </is>
+      </c>
+      <c r="L348" t="inlineStr">
         <is>
           <t>https://www.facebook.com/business/ads-guide/update</t>
         </is>
@@ -18264,7 +18334,7 @@
       </c>
       <c r="G349" t="inlineStr">
         <is>
-          <t>Feed: 1.91:1 até 1:1, 1080x1080 mín. (mín. 500x500), capa (imagem ou vídeo) + 3 imagens de produto; Experiência Instantânea obrigatória; texto principal 125c, título 40c, URL obrigatório; Stories: 1.91:1 até 1:1, 1080x1080 mín. (mín. 500x500), capa + 2 imagens de produto; Experiência Instantânea obrigatória; texto principal 125c, URL obrigatório; Reels: 9:16 (imagem de produto 1:1), mín. 500x888, capa + até 3 imagens de produto; Experiência Instantânea obrigatória.</t>
+          <t>Feed: 1.91:1 até 1:1, 1080x1080 mín. (mín. 500x500), capa (imagem ou vídeo) + 3 imagens de produto, Experiência Instantânea obrigatória; Stories: 1.91:1 até 1:1, 1080x1080 mín. (mín. 500x500), capa + 2 imagens de produto, Experiência Instantânea obrigatória; Reels: 9:16 (imagem de produto 1:1), mín. 500x888, capa + até 3 imagens de produto, Experiência Instantânea obrigatória.</t>
         </is>
       </c>
       <c r="H349" t="inlineStr">
@@ -18283,6 +18353,11 @@
         </is>
       </c>
       <c r="K349" t="inlineStr">
+        <is>
+          <t>Feed: texto principal 125c, título 40c, URL obrigatório; Stories: texto principal 125c, URL obrigatório.</t>
+        </is>
+      </c>
+      <c r="L349" t="inlineStr">
         <is>
           <t>https://www.facebook.com/business/ads-guide/update</t>
         </is>

</xml_diff>

<commit_message>
Fix Aspect Ratio duplication and or/and semantics for Facebook/Instagram
Two problems: the ratio was written both inside Dimensão ("Feed:
4:5, 1440x1800...") and in the separate Aspect Ratio column, and
Aspect Ratio joined multiple placements with "ou" (or) as if picking
one — but Feed, Stories and Reels each need their own delivered
creative, it's "and" not "or". Removed the ratio from inside
Dimensão text (kept resolution/minimums/duration only) and rebuilt
Aspect Ratio to mirror the same per-placement structure as Dimensão
("Feed: 4:5; Stories: 9:16; Reels: 9:16"), across all 8 Facebook/
Instagram rows (Single Image, Single Video, Carousel, Collection).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011oqQvDMfneVTKoco4dHUSc
</commit_message>
<xml_diff>
--- a/data/base-formatos.xlsx
+++ b/data/base-formatos.xlsx
@@ -17900,12 +17900,12 @@
       </c>
       <c r="G342" t="inlineStr">
         <is>
-          <t>Feed: 4:5, 1440x1800 (mín. 600px largura, mín. 750px altura), tolerância 3%; Stories: 9:16, 1440x2560 (mín. 500px largura), tolerância 1%; Reels: 9:16, 1440x2560 (mín. 600x600px), tolerância 3%.</t>
+          <t>Feed: 1440x1800 (mín. 600px largura, mín. 750px altura), tolerância 3%; Stories: 1440x2560 (mín. 500px largura), tolerância 1%; Reels: 1440x2560 (mín. 600x600px), tolerância 3%.</t>
         </is>
       </c>
       <c r="H342" t="inlineStr">
         <is>
-          <t>4:5 ou 9:16</t>
+          <t>Feed: 4:5; Stories: 9:16; Reels: 9:16</t>
         </is>
       </c>
       <c r="I342" t="inlineStr">
@@ -17962,12 +17962,12 @@
       </c>
       <c r="G343" t="inlineStr">
         <is>
-          <t>Feed: 4:5, 1440x1800 (mín. 120x120px), 1s a 241min; Stories: 9:16, 1440x2560 (mín. 250px largura), tolerância 1%, 1s a 3min; Reels: 9:16 recomendado, 1440x2560, sem duração máxima.</t>
+          <t>Feed: 1440x1800 (mín. 120x120px), 1s a 241min; Stories: 1440x2560 (mín. 250px largura), tolerância 1%, 1s a 3min; Reels: 1440x2560 recomendado, sem duração máxima.</t>
         </is>
       </c>
       <c r="H343" t="inlineStr">
         <is>
-          <t>4:5 ou 9:16</t>
+          <t>Feed: 4:5; Stories: 9:16; Reels: 9:16</t>
         </is>
       </c>
       <c r="I343" t="inlineStr">
@@ -18024,12 +18024,12 @@
       </c>
       <c r="G344" t="inlineStr">
         <is>
-          <t>Feed: 1:1, 1080x1080 mín. (imagem ou vídeo), 2 a 10 cartões, tolerância 3%; Stories: 1:1 recomendado, 1080x1920 mín. (só imagem, sem suporte a vídeo), 3 a 10 cartões, largura mín. 500px; Reels: 9:16, 1080x1920 mín. (só imagem), 2 a 10 cartões, largura mín. 500px, altura mín. 262px, tolerância 1%.</t>
+          <t>Feed: 1080x1080 mín. (imagem ou vídeo), 2 a 10 cartões, tolerância 3%; Stories: 1080x1920 mín. (só imagem, sem suporte a vídeo), 3 a 10 cartões, largura mín. 500px; Reels: 1080x1920 mín. (só imagem), 2 a 10 cartões, largura mín. 500px, altura mín. 262px, tolerância 1%.</t>
         </is>
       </c>
       <c r="H344" t="inlineStr">
         <is>
-          <t>1:1 ou 9:16</t>
+          <t>Feed: 1:1; Stories: 1:1 (recomendado); Reels: 9:16</t>
         </is>
       </c>
       <c r="I344" t="inlineStr">
@@ -18086,12 +18086,12 @@
       </c>
       <c r="G345" t="inlineStr">
         <is>
-          <t>Feed: 1.91:1 até 1:1, 1080x1080 mín. (capa: imagem ou vídeo) + 3 imagens de produto, Experiência Instantânea obrigatória; Reels: 9:16 até 1:1, 1080x1080 mín., requer Catálogo Advantage+ como fonte de conteúdo, Experiência Instantânea obrigatória.</t>
+          <t>Feed: 1080x1080 mín. (capa: imagem ou vídeo) + 3 imagens de produto, Experiência Instantânea obrigatória; Reels: 1080x1080 mín., requer Catálogo Advantage+ como fonte de conteúdo, Experiência Instantânea obrigatória.</t>
         </is>
       </c>
       <c r="H345" t="inlineStr">
         <is>
-          <t>1.91:1 até 1:1 ou 9:16</t>
+          <t>Feed: 1.91:1 até 1:1; Reels: 9:16 até 1:1</t>
         </is>
       </c>
       <c r="I345" t="inlineStr">
@@ -18148,12 +18148,12 @@
       </c>
       <c r="G346" t="inlineStr">
         <is>
-          <t>Feed: 4:5, 1440x1800 (mín. 500px largura; proporção mín. 400x500, máx. 191x100), tolerância 1%; Stories: 9:16, 1440x2560 (mín. 500px largura), tolerância 1%; Reels: 9:16, 1440x2560 (mín. 500px largura), tolerância 1%; Explorar: 4:5, 1440x1800 (mín. 500px largura; proporção mín. 400x500, máx. 191x100), tolerância 1%.</t>
+          <t>Feed: 1440x1800 (mín. 500px largura; proporção mín. 400x500, máx. 191x100), tolerância 1%; Stories: 1440x2560 (mín. 500px largura), tolerância 1%; Reels: 1440x2560 (mín. 500px largura), tolerância 1%; Explorar: 1440x1800 (mín. 500px largura; proporção mín. 400x500, máx. 191x100), tolerância 1%.</t>
         </is>
       </c>
       <c r="H346" t="inlineStr">
         <is>
-          <t>4:5 ou 9:16</t>
+          <t>Feed: 4:5; Stories: 9:16; Reels: 9:16; Explorar: 4:5</t>
         </is>
       </c>
       <c r="I346" t="inlineStr">
@@ -18210,12 +18210,12 @@
       </c>
       <c r="G347" t="inlineStr">
         <is>
-          <t>Feed: 9:16, 1080x1920 (mín. 250px largura), tolerância 1%, 1s a 60min; Stories: 9:16, 1440x2560 (mín. 250px largura), tolerância 1%, 1s a 60min; Reels: 9:16, 1440x2560, 0 a 15min, mín. 250px largura (&lt;30s) ou 500px (≥30s).</t>
+          <t>Feed: 1080x1920 (mín. 250px largura), tolerância 1%, 1s a 60min; Stories: 1440x2560 (mín. 250px largura), tolerância 1%, 1s a 60min; Reels: 1440x2560, 0 a 15min, mín. 250px largura (&lt;30s) ou 500px (≥30s).</t>
         </is>
       </c>
       <c r="H347" t="inlineStr">
         <is>
-          <t>9:16</t>
+          <t>Feed: 9:16; Stories: 9:16; Reels: 9:16</t>
         </is>
       </c>
       <c r="I347" t="inlineStr">
@@ -18272,12 +18272,12 @@
       </c>
       <c r="G348" t="inlineStr">
         <is>
-          <t>Feed: 4:5 (carrosséis só de imagem) ou 1:1 (se tiver vídeo), 1080x1080 mín., 2 a 10 cartões, tolerância 1%; Stories: 9:16, 1080x1920 mín. (imagem ou vídeo), 2 a 10 cartões, tolerância 1%; Reels: 9:16, 1080x1080 mín. (só imagem), 2 a 10 cartões, tolerância 1%.</t>
+          <t>Feed: 1080x1080 mín., 2 a 10 cartões, tolerância 1%; Stories: 1080x1920 mín. (imagem ou vídeo), 2 a 10 cartões, tolerância 1%; Reels: 1080x1080 mín. (só imagem), 2 a 10 cartões, tolerância 1%.</t>
         </is>
       </c>
       <c r="H348" t="inlineStr">
         <is>
-          <t>4:5 ou 1:1 ou 9:16</t>
+          <t>Feed: 4:5 (só imagem) ou 1:1 (com vídeo); Stories: 9:16; Reels: 9:16</t>
         </is>
       </c>
       <c r="I348" t="inlineStr">
@@ -18334,12 +18334,12 @@
       </c>
       <c r="G349" t="inlineStr">
         <is>
-          <t>Feed: 1.91:1 até 1:1, 1080x1080 mín. (mín. 500x500), capa (imagem ou vídeo) + 3 imagens de produto, Experiência Instantânea obrigatória; Stories: 1.91:1 até 1:1, 1080x1080 mín. (mín. 500x500), capa + 2 imagens de produto, Experiência Instantânea obrigatória; Reels: 9:16 (imagem de produto 1:1), mín. 500x888, capa + até 3 imagens de produto, Experiência Instantânea obrigatória.</t>
+          <t>Feed: 1080x1080 mín. (mín. 500x500), capa (imagem ou vídeo) + 3 imagens de produto, Experiência Instantânea obrigatória; Stories: 1080x1080 mín. (mín. 500x500), capa + 2 imagens de produto, Experiência Instantânea obrigatória; Reels: mín. 500x888 (imagem de produto 1:1), capa + até 3 imagens de produto, Experiência Instantânea obrigatória.</t>
         </is>
       </c>
       <c r="H349" t="inlineStr">
         <is>
-          <t>1.91:1 até 1:1 ou 9:16</t>
+          <t>Feed: 1.91:1 até 1:1; Stories: 1.91:1 até 1:1; Reels: 9:16 (imagem de produto: 1:1)</t>
         </is>
       </c>
       <c r="I349" t="inlineStr">

</xml_diff>

<commit_message>
Remove menções a tolerância dos textos de Dimensão (Facebook/Instagram)
Nas linhas Single Image, Single Video e Carousel do Facebook e do
Instagram, a Dimensão incluía "tolerância X%" para cada medida — informação
desnecessária que só acrescentava ruído ao que realmente é preciso
entregar. Removidas as 6 ocorrências, mantendo intactas as dimensões,
mínimos e durações reais de cada placement (Feed/Stories/Reels).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011oqQvDMfneVTKoco4dHUSc
</commit_message>
<xml_diff>
--- a/data/base-formatos.xlsx
+++ b/data/base-formatos.xlsx
@@ -17900,7 +17900,7 @@
       </c>
       <c r="G342" t="inlineStr">
         <is>
-          <t>Feed: 1440x1800 (mín. 600px largura, mín. 750px altura), tolerância 3%; Stories: 1440x2560 (mín. 500px largura), tolerância 1%; Reels: 1440x2560 (mín. 600x600px), tolerância 3%.</t>
+          <t>Feed: 1440x1800 (mín. 600px largura, mín. 750px altura); Stories: 1440x2560 (mín. 500px largura); Reels: 1440x2560 (mín. 600x600px).</t>
         </is>
       </c>
       <c r="H342" t="inlineStr">
@@ -17962,7 +17962,7 @@
       </c>
       <c r="G343" t="inlineStr">
         <is>
-          <t>Feed: 1440x1800 (mín. 120x120px), 1s a 241min; Stories: 1440x2560 (mín. 250px largura), tolerância 1%, 1s a 3min; Reels: 1440x2560 recomendado, sem duração máxima.</t>
+          <t>Feed: 1440x1800 (mín. 120x120px), 1s a 241min; Stories: 1440x2560 (mín. 250px largura), 1s a 3min; Reels: 1440x2560 recomendado, sem duração máxima.</t>
         </is>
       </c>
       <c r="H343" t="inlineStr">
@@ -18024,7 +18024,7 @@
       </c>
       <c r="G344" t="inlineStr">
         <is>
-          <t>Feed: 1080x1080 mín. (imagem ou vídeo), 2 a 10 cartões, tolerância 3%; Stories: 1080x1920 mín. (só imagem, sem suporte a vídeo), 3 a 10 cartões, largura mín. 500px; Reels: 1080x1920 mín. (só imagem), 2 a 10 cartões, largura mín. 500px, altura mín. 262px, tolerância 1%.</t>
+          <t>Feed: 1080x1080 mín. (imagem ou vídeo), 2 a 10 cartões; Stories: 1080x1920 mín. (só imagem, sem suporte a vídeo), 3 a 10 cartões, largura mín. 500px; Reels: 1080x1920 mín. (só imagem), 2 a 10 cartões, largura mín. 500px, altura mín. 262px.</t>
         </is>
       </c>
       <c r="H344" t="inlineStr">
@@ -18148,7 +18148,7 @@
       </c>
       <c r="G346" t="inlineStr">
         <is>
-          <t>Feed: 1440x1800 (mín. 500px largura; proporção mín. 400x500, máx. 191x100), tolerância 1%; Stories: 1440x2560 (mín. 500px largura), tolerância 1%; Reels: 1440x2560 (mín. 500px largura), tolerância 1%; Explorar: 1440x1800 (mín. 500px largura; proporção mín. 400x500, máx. 191x100), tolerância 1%.</t>
+          <t>Feed: 1440x1800 (mín. 500px largura; proporção mín. 400x500, máx. 191x100); Stories: 1440x2560 (mín. 500px largura); Reels: 1440x2560 (mín. 500px largura); Explorar: 1440x1800 (mín. 500px largura; proporção mín. 400x500, máx. 191x100).</t>
         </is>
       </c>
       <c r="H346" t="inlineStr">
@@ -18210,7 +18210,7 @@
       </c>
       <c r="G347" t="inlineStr">
         <is>
-          <t>Feed: 1080x1920 (mín. 250px largura), tolerância 1%, 1s a 60min; Stories: 1440x2560 (mín. 250px largura), tolerância 1%, 1s a 60min; Reels: 1440x2560, 0 a 15min, mín. 250px largura (&lt;30s) ou 500px (≥30s).</t>
+          <t>Feed: 1080x1920 (mín. 250px largura), 1s a 60min; Stories: 1440x2560 (mín. 250px largura), 1s a 60min; Reels: 1440x2560, 0 a 15min, mín. 250px largura (&lt;30s) ou 500px (≥30s).</t>
         </is>
       </c>
       <c r="H347" t="inlineStr">
@@ -18272,7 +18272,7 @@
       </c>
       <c r="G348" t="inlineStr">
         <is>
-          <t>Feed: 1080x1080 mín., 2 a 10 cartões, tolerância 1%; Stories: 1080x1920 mín. (imagem ou vídeo), 2 a 10 cartões, tolerância 1%; Reels: 1080x1080 mín. (só imagem), 2 a 10 cartões, tolerância 1%.</t>
+          <t>Feed: 1080x1080 mín., 2 a 10 cartões; Stories: 1080x1920 mín. (imagem ou vídeo), 2 a 10 cartões; Reels: 1080x1080 mín. (só imagem), 2 a 10 cartões.</t>
         </is>
       </c>
       <c r="H348" t="inlineStr">

</xml_diff>

<commit_message>
Atualiza specs oficiais do LinkedIn (15 formatos)
Substitui as specs resumidas do LinkedIn pelas specs completas e oficiais
fornecidas pela agência (Single Image, Video, Carousel, Event, Document,
Thought Leader, Article/Newsletter, Job, Conversation, Message, Spotlight,
Follower, Text Ads, Lead Gen Forms, Connected TV), mantendo a separação já
estabelecida na base: Dimensão só com dimensões/proporções/durações reais,
Copies com os limites de texto e URL, Tipo de Ficheiro com formatos e specs
técnicas de encoding (ex.: bitrate/frame rate/áudio do Connected TV).

Corrige também um dado antes assumido sem base real: Conversation/Message
Ads não têm imagem própria de 250x250 — usam a foto de perfil do
remetente no LinkedIn; só o banner (opcional, máx. 300x250) é um asset a
fornecer.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011oqQvDMfneVTKoco4dHUSc
</commit_message>
<xml_diff>
--- a/data/base-formatos.xlsx
+++ b/data/base-formatos.xlsx
@@ -10285,7 +10285,7 @@
       </c>
       <c r="G192" t="inlineStr">
         <is>
-          <t>Imagem do artigo/newsletter (conteúdo orgânico)</t>
+          <t>Imagem do artigo/newsletter (conteúdo orgânico) — specs iguais ao Single Image.</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
@@ -10296,6 +10296,11 @@
       <c r="J192" t="inlineStr">
         <is>
           <t>Post/artigo ou newsletter já publicado no LinkedIn</t>
+        </is>
+      </c>
+      <c r="K192" t="inlineStr">
+        <is>
+          <t>Sem título/texto introdutório editável — o criativo é o artigo/newsletter orgânico original.</t>
         </is>
       </c>
     </row>
@@ -10332,7 +10337,7 @@
       </c>
       <c r="G193" t="inlineStr">
         <is>
-          <t>1080x1080 recomendado; máx. 4320x4320</t>
+          <t>Recomendado mín. 1080x1080 (não suporta vídeo).</t>
         </is>
       </c>
       <c r="H193" t="inlineStr">
@@ -10347,7 +10352,12 @@
       </c>
       <c r="J193" t="inlineStr">
         <is>
-          <t>JPG, PNG, GIF não animado</t>
+          <t>JPG ou PNG; 2 a 10 cartões</t>
+        </is>
+      </c>
+      <c r="K193" t="inlineStr">
+        <is>
+          <t>Nome do anúncio (opcional): 255c; Título do cartão: 45c; Texto introdutório: 255c; Landing page URL: máx. 2000c.</t>
         </is>
       </c>
     </row>
@@ -10384,7 +10394,7 @@
       </c>
       <c r="G194" t="inlineStr">
         <is>
-          <t>1920x1080 recomendado; 1280x720 aceite</t>
+          <t>1920x1080 recomendado (ou 1280x720); duração 6 a 60s (recomendado 6, 15, 30, 45 ou 60s).</t>
         </is>
       </c>
       <c r="H194" t="inlineStr">
@@ -10399,7 +10409,7 @@
       </c>
       <c r="J194" t="inlineStr">
         <is>
-          <t>MP4 (H.264)</t>
+          <t>MP4, codec H.264, bitrate mín. 12 Mbps (recomendado 15–40 Mbps), frame rate constante (23,98/24/25/29,97/30 fps), áudio 2 canais -23 LUFS integrado, PCM (16/24 bit) ou AAC ≥192 Kbps, 48 kHz, chroma 4:2:0 (recomendado 4:2:2).</t>
         </is>
       </c>
     </row>
@@ -10436,22 +10446,22 @@
       </c>
       <c r="G195" t="inlineStr">
         <is>
-          <t>250x250 imagem; banner opcional máx. 300x250</t>
-        </is>
-      </c>
-      <c r="H195" t="inlineStr">
-        <is>
-          <t>1:1</t>
+          <t>Banner opcional: máx. 300x250 (só desktop); imagem do remetente = foto de perfil LinkedIn do remetente definido.</t>
         </is>
       </c>
       <c r="I195" t="inlineStr">
         <is>
-          <t>5 MB imagem; 2 MB banner</t>
+          <t>Banner: máx. 2 MB</t>
         </is>
       </c>
       <c r="J195" t="inlineStr">
         <is>
-          <t>JPG, PNG</t>
+          <t>Banner: JPG ou PNG (opcional)</t>
+        </is>
+      </c>
+      <c r="K195" t="inlineStr">
+        <is>
+          <t>Nome do anúncio (opcional): 255c; Texto da mensagem: máx. 8000c; Rodapé personalizado: máx. 20000c; CTA: máx. 25c; Landing page URL: máx. 2000c.</t>
         </is>
       </c>
     </row>
@@ -10488,7 +10498,7 @@
       </c>
       <c r="G196" t="inlineStr">
         <is>
-          <t>Sem dimensão fixa; layouts standard (A4, Letter, etc.)</t>
+          <t>Sem dimensão fixa em píxeis — layouts standard (A4, Letter, Legal, etc.); recomendado até 10 páginas (máx. 300 páginas ou 1M palavras).</t>
         </is>
       </c>
       <c r="I196" t="inlineStr">
@@ -10498,7 +10508,12 @@
       </c>
       <c r="J196" t="inlineStr">
         <is>
-          <t>PDF, PPT, PPTX, DOC, DOCX</t>
+          <t>PDF, DOC, DOCX, PPT, PPTX</t>
+        </is>
+      </c>
+      <c r="K196" t="inlineStr">
+        <is>
+          <t>Nome do anúncio (opcional): 255c; Título: 70c; Texto introdutório: 150c.</t>
         </is>
       </c>
     </row>
@@ -10535,7 +10550,12 @@
       </c>
       <c r="G197" t="inlineStr">
         <is>
-          <t>Usa imagem do evento LinkedIn</t>
+          <t>Imagem retirada automaticamente da página do Evento.</t>
+        </is>
+      </c>
+      <c r="H197" t="inlineStr">
+        <is>
+          <t>4:1</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">
@@ -10545,7 +10565,12 @@
       </c>
       <c r="J197" t="inlineStr">
         <is>
-          <t>Evento publicado no LinkedIn</t>
+          <t>Evento já publicado no LinkedIn</t>
+        </is>
+      </c>
+      <c r="K197" t="inlineStr">
+        <is>
+          <t>Nome do evento (opcional): 255c; Texto introdutório: 600c; Event URL: obrigatório, só páginas de Evento do LinkedIn.</t>
         </is>
       </c>
     </row>
@@ -10582,7 +10607,7 @@
       </c>
       <c r="G198" t="inlineStr">
         <is>
-          <t>Logo: 100x100 recomendado</t>
+          <t>Logo da empresa: 100x100.</t>
         </is>
       </c>
       <c r="H198" t="inlineStr">
@@ -10597,7 +10622,12 @@
       </c>
       <c r="J198" t="inlineStr">
         <is>
-          <t>JPG, PNG</t>
+          <t>JPG ou PNG</t>
+        </is>
+      </c>
+      <c r="K198" t="inlineStr">
+        <is>
+          <t>Título: 50c; Descrição: 70c; Nome da empresa: 25c.</t>
         </is>
       </c>
     </row>
@@ -10634,7 +10664,7 @@
       </c>
       <c r="G199" t="inlineStr">
         <is>
-          <t>Dinâmico; usa logo/elementos da Page e vaga</t>
+          <t>Dinâmico; usa logo/elementos da Page e vaga.</t>
         </is>
       </c>
       <c r="I199" t="inlineStr">
@@ -10645,6 +10675,11 @@
       <c r="J199" t="inlineStr">
         <is>
           <t>Vaga + Page LinkedIn</t>
+        </is>
+      </c>
+      <c r="K199" t="inlineStr">
+        <is>
+          <t>Texto introdutório: até 150c.</t>
         </is>
       </c>
     </row>
@@ -10681,7 +10716,7 @@
       </c>
       <c r="G200" t="inlineStr">
         <is>
-          <t>Sem asset gráfico próprio; associado ao anúncio</t>
+          <t>Sem asset gráfico próprio; associado ao anúncio.</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
@@ -10692,6 +10727,11 @@
       <c r="J200" t="inlineStr">
         <is>
           <t>Formulário criado no Campaign Manager</t>
+        </is>
+      </c>
+      <c r="K200" t="inlineStr">
+        <is>
+          <t>Nome do formulário: 256c; Título da oferta: 60c; Detalhe da oferta (opcional): 160c; Política de privacidade: 2000c; CTA: 20c; Mensagem de confirmação: 300c; Perguntas personalizadas: até 3, 100c cada; campos recomendados: 3-4 (máx. 12).</t>
         </is>
       </c>
     </row>
@@ -10728,17 +10768,22 @@
       </c>
       <c r="G201" t="inlineStr">
         <is>
-          <t>Banner opcional 300x250</t>
+          <t>Banner opcional: máx. 300x250 (só desktop); imagem do remetente = foto de perfil LinkedIn do remetente definido.</t>
         </is>
       </c>
       <c r="I201" t="inlineStr">
         <is>
-          <t>2 MB</t>
+          <t>Banner: máx. 2 MB</t>
         </is>
       </c>
       <c r="J201" t="inlineStr">
         <is>
-          <t>JPG, PNG</t>
+          <t>Banner: JPG ou PNG (opcional)</t>
+        </is>
+      </c>
+      <c r="K201" t="inlineStr">
+        <is>
+          <t>Nome do anúncio (opcional): 255c; Texto da mensagem: máx. 8000c; Rodapé personalizado: máx. 20000c; CTA: máx. 25c; Landing page URL: máx. 2000c.</t>
         </is>
       </c>
     </row>
@@ -10775,12 +10820,12 @@
       </c>
       <c r="G202" t="inlineStr">
         <is>
-          <t>1200x628 (1.91:1); 1200x1200 (1:1); 720x900 (4:5)</t>
+          <t>Horizontal: 1200x628 recomendado (mín. 640x360, máx. 7680x4320); Quadrado: 1200x1200 recomendado (mín. 360x360, máx. 4320x4320); Vertical: 720x900 recomendado (mín. 360x640, máx. 2430x4320).</t>
         </is>
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>1.91:1 ou 1:1 ou 4:5</t>
+          <t>1,91:1 (horizontal) ou 1:1 (quadrado) ou 4:5 (vertical, recomendado)</t>
         </is>
       </c>
       <c r="I202" t="inlineStr">
@@ -10790,7 +10835,12 @@
       </c>
       <c r="J202" t="inlineStr">
         <is>
-          <t>JPG, PNG ou GIF</t>
+          <t>JPG, PNG ou GIF (GIF animado até 250 frames)</t>
+        </is>
+      </c>
+      <c r="K202" t="inlineStr">
+        <is>
+          <t>Nome do anúncio (opcional): 255c; Título: 70c; Texto introdutório: 150c (máx. 3000c); Descrição (só LAN): 70c; Landing page URL: máx. 2000c.</t>
         </is>
       </c>
       <c r="L202" t="inlineStr">
@@ -10832,22 +10882,27 @@
       </c>
       <c r="G203" t="inlineStr">
         <is>
-          <t>1920x1080 / 720x900 / 720x1280; conforme rácio</t>
+          <t>Landscape: 1920x1080 recomendado (mín. 640x360, máx. 1920x1080); Square: mín. 360x360, máx. 1920x1920; Vertical 4:5: mín. 360x450, máx. 1080x1350; Vertical 9:16: 720x1280 recomendado (mín. 360x640, máx. 1080x1920). Duração: 3s a 30min (in-stream em streaming até 90s).</t>
         </is>
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>16:9 ou 4:5 ou 9:16</t>
+          <t>16:9 ou 1:1 ou 4:5 ou 9:16</t>
         </is>
       </c>
       <c r="I203" t="inlineStr">
         <is>
-          <t>75 KB–500 MB</t>
+          <t>75 KB a 500 MB</t>
         </is>
       </c>
       <c r="J203" t="inlineStr">
         <is>
-          <t>MP4; thumbnail JPG/PNG opcional</t>
+          <t>MP4, codec H.264 ou VP8, áudio AAC ou MPEG4 (&lt;64 KHz), 30 fps recomendado; thumbnail opcional JPG/PNG máx. 2 MB (rácio igual ao vídeo)</t>
+        </is>
+      </c>
+      <c r="K203" t="inlineStr">
+        <is>
+          <t>Nome do anúncio (opcional): 255c; Título: 70c (máx. 200c); Texto introdutório: 150c (máx. 600c).</t>
         </is>
       </c>
     </row>
@@ -10884,22 +10939,27 @@
       </c>
       <c r="G204" t="inlineStr">
         <is>
-          <t>Logo 100x100; background opcional 300x250</t>
+          <t>Logo da empresa: 100x100; Imagem de fundo opcional: 300x250.</t>
         </is>
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>1:1</t>
+          <t>Logo: 1:1</t>
         </is>
       </c>
       <c r="I204" t="inlineStr">
         <is>
-          <t>2 MB</t>
+          <t>Logo: 2 MB; Imagem de fundo: 2 MB</t>
         </is>
       </c>
       <c r="J204" t="inlineStr">
         <is>
-          <t>JPG, PNG</t>
+          <t>JPG ou PNG</t>
+        </is>
+      </c>
+      <c r="K204" t="inlineStr">
+        <is>
+          <t>Título: 50c; Descrição: 70c; Nome da empresa: 25c; CTA: 18c; Landing page URL: máx. 500c.</t>
         </is>
       </c>
     </row>
@@ -10936,7 +10996,7 @@
       </c>
       <c r="G205" t="inlineStr">
         <is>
-          <t>100x100</t>
+          <t>Logo: 100x100.</t>
         </is>
       </c>
       <c r="H205" t="inlineStr">
@@ -10951,7 +11011,12 @@
       </c>
       <c r="J205" t="inlineStr">
         <is>
-          <t>JPG, PNG</t>
+          <t>JPG ou PNG</t>
+        </is>
+      </c>
+      <c r="K205" t="inlineStr">
+        <is>
+          <t>Título: 25c; Descrição: 75c; Landing page URL: máx. 2000c.</t>
         </is>
       </c>
     </row>
@@ -10988,7 +11053,7 @@
       </c>
       <c r="G206" t="inlineStr">
         <is>
-          <t>Depende do post original (imagem/vídeo/documento/etc.)</t>
+          <t>Depende do post original (imagem/vídeo/documento/etc.) — specs iguais ao formato do post.</t>
         </is>
       </c>
       <c r="I206" t="inlineStr">
@@ -10999,6 +11064,11 @@
       <c r="J206" t="inlineStr">
         <is>
           <t>Post orgânico elegível de membro/Page</t>
+        </is>
+      </c>
+      <c r="K206" t="inlineStr">
+        <is>
+          <t>Sem título/texto introdutório editável — o criativo é o post orgânico original; sem CTA.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Adiciona os links oficiais de fonte a todos os 15 formatos do LinkedIn
Cada formato passa a ligar diretamente à respetiva página de specs em
business.linkedin.com (Single Image, Video, Carousel, Event, Document,
Thought Leader, Connected TV, Article/Newsletter, Job Ads, Conversation,
Message, Spotlight, Follower, Text Ads, Lead Gen Forms).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011oqQvDMfneVTKoco4dHUSc
</commit_message>
<xml_diff>
--- a/data/base-formatos.xlsx
+++ b/data/base-formatos.xlsx
@@ -10303,6 +10303,11 @@
           <t>Sem título/texto introdutório editável — o criativo é o artigo/newsletter orgânico original.</t>
         </is>
       </c>
+      <c r="L192" t="inlineStr">
+        <is>
+          <t>https://business.linkedin.com/advertise/ads/sponsored-content/articles-and-newsletters-ads/specs</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -10360,6 +10365,11 @@
           <t>Nome do anúncio (opcional): 255c; Título do cartão: 45c; Texto introdutório: 255c; Landing page URL: máx. 2000c.</t>
         </is>
       </c>
+      <c r="L193" t="inlineStr">
+        <is>
+          <t>https://business.linkedin.com/advertise/ads/sponsored-content/carousel-ads/specs</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -10412,6 +10422,11 @@
           <t>MP4, codec H.264, bitrate mín. 12 Mbps (recomendado 15–40 Mbps), frame rate constante (23,98/24/25/29,97/30 fps), áudio 2 canais -23 LUFS integrado, PCM (16/24 bit) ou AAC ≥192 Kbps, 48 kHz, chroma 4:2:0 (recomendado 4:2:2).</t>
         </is>
       </c>
+      <c r="L194" t="inlineStr">
+        <is>
+          <t>https://business.linkedin.com/advertise/ads/sponsored-content/connected-tv-ads/specs</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -10464,6 +10479,11 @@
           <t>Nome do anúncio (opcional): 255c; Texto da mensagem: máx. 8000c; Rodapé personalizado: máx. 20000c; CTA: máx. 25c; Landing page URL: máx. 2000c.</t>
         </is>
       </c>
+      <c r="L195" t="inlineStr">
+        <is>
+          <t>https://business.linkedin.com/advertise/ads/sponsored-messaging/conversation-ads/specs</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -10516,6 +10536,11 @@
           <t>Nome do anúncio (opcional): 255c; Título: 70c; Texto introdutório: 150c.</t>
         </is>
       </c>
+      <c r="L196" t="inlineStr">
+        <is>
+          <t>https://business.linkedin.com/advertise/ads/sponsored-content/document-ads/specs</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -10573,6 +10598,11 @@
           <t>Nome do evento (opcional): 255c; Texto introdutório: 600c; Event URL: obrigatório, só páginas de Evento do LinkedIn.</t>
         </is>
       </c>
+      <c r="L197" t="inlineStr">
+        <is>
+          <t>https://business.linkedin.com/advertise/ads/sponsored-content/event-ads/specs</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -10630,6 +10660,11 @@
           <t>Título: 50c; Descrição: 70c; Nome da empresa: 25c.</t>
         </is>
       </c>
+      <c r="L198" t="inlineStr">
+        <is>
+          <t>https://business.linkedin.com/advertise/ads/dynamic-ads/follower-ads</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -10682,6 +10717,11 @@
           <t>Texto introdutório: até 150c.</t>
         </is>
       </c>
+      <c r="L199" t="inlineStr">
+        <is>
+          <t>https://business.linkedin.com/advertise/ads/ads-guide</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -10734,6 +10774,11 @@
           <t>Nome do formulário: 256c; Título da oferta: 60c; Detalhe da oferta (opcional): 160c; Política de privacidade: 2000c; CTA: 20c; Mensagem de confirmação: 300c; Perguntas personalizadas: até 3, 100c cada; campos recomendados: 3-4 (máx. 12).</t>
         </is>
       </c>
+      <c r="L200" t="inlineStr">
+        <is>
+          <t>https://business.linkedin.com/advertise/ads/sponsored-content/lead-gen-ads/specs</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -10786,6 +10831,11 @@
           <t>Nome do anúncio (opcional): 255c; Texto da mensagem: máx. 8000c; Rodapé personalizado: máx. 20000c; CTA: máx. 25c; Landing page URL: máx. 2000c.</t>
         </is>
       </c>
+      <c r="L201" t="inlineStr">
+        <is>
+          <t>https://business.linkedin.com/advertise/ads/sponsored-messaging/message-ads/specs</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -10905,6 +10955,11 @@
           <t>Nome do anúncio (opcional): 255c; Título: 70c (máx. 200c); Texto introdutório: 150c (máx. 600c).</t>
         </is>
       </c>
+      <c r="L203" t="inlineStr">
+        <is>
+          <t>https://business.linkedin.com/advertise/ads/sponsored-content/video-ads/specs</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -10962,6 +11017,11 @@
           <t>Título: 50c; Descrição: 70c; Nome da empresa: 25c; CTA: 18c; Landing page URL: máx. 500c.</t>
         </is>
       </c>
+      <c r="L204" t="inlineStr">
+        <is>
+          <t>https://business.linkedin.com/advertise/ads/dynamic-ads/spotlight-ads</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -11019,6 +11079,11 @@
           <t>Título: 25c; Descrição: 75c; Landing page URL: máx. 2000c.</t>
         </is>
       </c>
+      <c r="L205" t="inlineStr">
+        <is>
+          <t>https://business.linkedin.com/advertise/ads/text-ads/specs</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -11069,6 +11134,11 @@
       <c r="K206" t="inlineStr">
         <is>
           <t>Sem título/texto introdutório editável — o criativo é o post orgânico original; sem CTA.</t>
+        </is>
+      </c>
+      <c r="L206" t="inlineStr">
+        <is>
+          <t>https://business.linkedin.com/advertise/ads/sponsored-content/thought-leader-ads/specs</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza specs completas do Pinterest e adiciona 3 formatos novos
Substitui as specs resumidas de Image Pin, Video Ad, Carousel Ad e
Collection pelas specs completas e oficiais fornecidas (dimensões,
duração de vídeo, peso por plataforma, limites de copy incluindo a
exceção para chinês/japonês/coreano/árabe nos títulos).

Adiciona 3 formatos interativos do Pinterest que ainda não estavam na
base: Idea Ad, Showcase Ad e Quiz Ad — cada um com zonas seguras, rácios
por elemento (title Pin/cartão/feature) e limites de texto próprios.

Base passa de 348 para 351 formatos. Traduzidas as 7 linhas afetadas
(as 4 atualizadas + as 3 novas) para EN/ES/FR em data/traducoes-specs.json,
mantendo a mesma qualidade e convenções já estabelecidas. Testado nas 4
línguas via Playwright, sem erros.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011oqQvDMfneVTKoco4dHUSc
</commit_message>
<xml_diff>
--- a/data/base-formatos.xlsx
+++ b/data/base-formatos.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L349"/>
+  <dimension ref="A1:L352"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="18.08984375" customWidth="1" style="2" min="1" max="1"/>
@@ -11175,22 +11175,27 @@
       </c>
       <c r="G207" t="inlineStr">
         <is>
-          <t>1:1 ou 2:3; 1000x1000 / 1000x1500 recomendado</t>
+          <t>Standard: 2 a 5 imagens, 1:1 ou 2:3; Sales (catálogo): 2 a 10 imagens/vídeos, dimensões herdadas do catálogo.</t>
         </is>
       </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t>1:1 ou 2:3</t>
+          <t>1:1 ou 2:3 (Standard); N/A no Sales (herdado do catálogo)</t>
         </is>
       </c>
       <c r="I207" t="inlineStr">
         <is>
-          <t>20 MB por imagem</t>
+          <t>Standard: 20 MB por imagem; Sales: N/A (herdado do catálogo)</t>
         </is>
       </c>
       <c r="J207" t="inlineStr">
         <is>
-          <t>PNG, JPEG; 2–5 imagens (non-Sales)</t>
+          <t>PNG ou JPEG (Standard); imagem ou vídeo via catálogo (Sales)</t>
+        </is>
+      </c>
+      <c r="K207" t="inlineStr">
+        <is>
+          <t>Título: até 100c (só os primeiros 40c podem mostrar no feed; 30c para chinês/japonês/coreano/árabe); Descrição: até 800c.</t>
         </is>
       </c>
       <c r="L207" t="inlineStr">
@@ -11232,17 +11237,27 @@
       </c>
       <c r="G208" t="inlineStr">
         <is>
-          <t>Hero 1:1 ou 2:3; assets secundários via catálogo</t>
+          <t>Hero: 1:1 ou 2:3 (pode diferir dos secundários); Secundários: mín. 3 recomendado, máx. 24, todos com o mesmo rácio entre si (1:1 ou 2:3); Hero em vídeo: duração mín. 4s, máx. 15min, rácio mais estreito que 1:2 e mais largo que 1,91:1 (recomendado 1:1, 2:3 ou 9:16).</t>
+        </is>
+      </c>
+      <c r="H208" t="inlineStr">
+        <is>
+          <t>Hero: 1:1 ou 2:3; Secundários: 1:1 ou 2:3 (recomendado 1:1)</t>
         </is>
       </c>
       <c r="I208" t="inlineStr">
         <is>
-          <t>Imagem 20 MB; vídeo até 2 GB</t>
+          <t>Imagem: 10 MB; Vídeo: até 2 GB</t>
         </is>
       </c>
       <c r="J208" t="inlineStr">
         <is>
-          <t>PNG, JPEG, MP4/MOV/M4V + catálogo</t>
+          <t>PNG ou JPEG (imagem); MP4, MOV ou M4V, codec H.264 ou H.265 (vídeo hero)</t>
+        </is>
+      </c>
+      <c r="K208" t="inlineStr">
+        <is>
+          <t>Título: até 100c (só os primeiros 40c podem mostrar no feed; 30c para chinês/japonês/coreano/árabe); Descrição: só aparece em Pins de Collection orgânicos vistos de perto, não em ads promovidos.</t>
         </is>
       </c>
       <c r="L208" t="inlineStr">
@@ -11284,22 +11299,27 @@
       </c>
       <c r="G209" t="inlineStr">
         <is>
-          <t>1000x1500 recomendado (2:3)</t>
+          <t>Recomendado 1000x1500 (2:3). Pins com rácio superior a 2:3 podem ficar cortados no feed.</t>
         </is>
       </c>
       <c r="H209" t="inlineStr">
         <is>
-          <t>2:3</t>
+          <t>2:3 (recomendado)</t>
         </is>
       </c>
       <c r="I209" t="inlineStr">
         <is>
-          <t>20 MB</t>
+          <t>Desktop: 20 MB; In-app: 32 MB</t>
         </is>
       </c>
       <c r="J209" t="inlineStr">
         <is>
-          <t>PNG, JPEG</t>
+          <t>PNG ou JPEG</t>
+        </is>
+      </c>
+      <c r="K209" t="inlineStr">
+        <is>
+          <t>Título: até 100c (só os primeiros 40c podem mostrar no feed; 30c para chinês/japonês/coreano/árabe); Descrição: até 800c.</t>
         </is>
       </c>
       <c r="L209" t="inlineStr">
@@ -11341,22 +11361,27 @@
       </c>
       <c r="G210" t="inlineStr">
         <is>
-          <t>1000x1500 (2:3), 1080x1920 (9:16) ou square conforme placement</t>
+          <t>Duração: mín. 4s, máx. 15min (recomendado 6-15s para ads). Rácio: mais estreito que 1:2, mais largo que 1,91:1; recomendado quadrado (1:1) ou vertical (2:3, 4:5 ou 9:16).</t>
         </is>
       </c>
       <c r="H210" t="inlineStr">
         <is>
-          <t>2:3 ou 9:16</t>
+          <t>1:1, 2:3, 4:5 ou 9:16 (recomendado); aceite entre 1:2 e 1,91:1</t>
         </is>
       </c>
       <c r="I210" t="inlineStr">
         <is>
-          <t>2 GB</t>
+          <t>Até 2 GB</t>
         </is>
       </c>
       <c r="J210" t="inlineStr">
         <is>
-          <t>MP4, MOV, M4V</t>
+          <t>MP4, MOV ou M4V; codec H.264 ou H.265</t>
+        </is>
+      </c>
+      <c r="K210" t="inlineStr">
+        <is>
+          <t>Título: até 100c (só os primeiros 40c podem mostrar no feed; 30c para chinês/japonês/coreano/árabe); Descrição: até 800c.</t>
         </is>
       </c>
       <c r="L210" t="inlineStr">
@@ -18500,6 +18525,192 @@
       <c r="L349" t="inlineStr">
         <is>
           <t>https://www.facebook.com/business/ads-guide/update</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>INTERNET</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>Paid Social</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>Pinterest</t>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t>Pinterest</t>
+        </is>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>Native</t>
+        </is>
+      </c>
+      <c r="F350" t="inlineStr">
+        <is>
+          <t>Idea Ad</t>
+        </is>
+      </c>
+      <c r="G350" t="inlineStr">
+        <is>
+          <t>Recomendado 1080x1920 para imagem/vídeo full-bleed. Duração de vídeo: máx. 5min. Zonas seguras: topo 270px, esquerda 65px, direita 195px, fundo 440px.</t>
+        </is>
+      </c>
+      <c r="H350" t="inlineStr">
+        <is>
+          <t>9:16 (recomendado, sem restrição rígida)</t>
+        </is>
+      </c>
+      <c r="I350" t="inlineStr">
+        <is>
+          <t>Recomendado 1 GB; Android/iOS: máx. 2 GB; Web: máx. 100 MB</t>
+        </is>
+      </c>
+      <c r="J350" t="inlineStr">
+        <is>
+          <t>Imagem: BMP, JPEG, PNG, TIFF, WEBP; Vídeo (só iOS/Android): MP4, M4V, MOV, codec H.264 ou H.265</t>
+        </is>
+      </c>
+      <c r="K350" t="inlineStr">
+        <is>
+          <t>Título: até 100c; Texto na página: até 250c.</t>
+        </is>
+      </c>
+      <c r="L350" t="inlineStr">
+        <is>
+          <t>https://help.pinterest.com/en/business/article/pinterest-product-specs</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>INTERNET</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>Paid Social</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>Pinterest</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>Pinterest</t>
+        </is>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>Native</t>
+        </is>
+      </c>
+      <c r="F351" t="inlineStr">
+        <is>
+          <t>Showcase Ad</t>
+        </is>
+      </c>
+      <c r="G351" t="inlineStr">
+        <is>
+          <t>Recomendado 1000x1500. Até 4 cartões além do title Pin principal; 1 a 3 features por cartão. Zona segura: 342x430px; evitar texto/logos nos últimos 80px do cartão.</t>
+        </is>
+      </c>
+      <c r="H351" t="inlineStr">
+        <is>
+          <t>Title Pin: 2:3; Cartão: 2:3; Feature: 1:1 estático</t>
+        </is>
+      </c>
+      <c r="I351" t="inlineStr">
+        <is>
+          <t>Até 32 MB</t>
+        </is>
+      </c>
+      <c r="J351" t="inlineStr">
+        <is>
+          <t>Imagem: BMP, JPEG, PNG, TIFF, WEBP; Vídeo (só iOS/Android): MP4, MOV ou M4V, 3 a 60s</t>
+        </is>
+      </c>
+      <c r="K351" t="inlineStr">
+        <is>
+          <t>Texto sobreposto: máx. 10 palavras; Feature: até 50c (título cortado a partir dos 50c).</t>
+        </is>
+      </c>
+      <c r="L351" t="inlineStr">
+        <is>
+          <t>https://help.pinterest.com/en/business/article/pinterest-product-specs</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>INTERNET</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>Paid Social</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>Pinterest</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>Pinterest</t>
+        </is>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>Native</t>
+        </is>
+      </c>
+      <c r="F352" t="inlineStr">
+        <is>
+          <t>Quiz Ad</t>
+        </is>
+      </c>
+      <c r="G352" t="inlineStr">
+        <is>
+          <t>Recomendado 1000x1500. Até 3 results Pins com 1 title Pin. Zona segura: 342x376px.</t>
+        </is>
+      </c>
+      <c r="H352" t="inlineStr">
+        <is>
+          <t>Title Pin: 2:3; Results Pin: 2:3</t>
+        </is>
+      </c>
+      <c r="I352" t="inlineStr">
+        <is>
+          <t>Até 32 MB</t>
+        </is>
+      </c>
+      <c r="J352" t="inlineStr">
+        <is>
+          <t>Imagem: BMP, JPEG, PNG, TIFF, WEBP; Vídeo (só iOS/Android): MP4, MOV ou M4V, 3 a 60s</t>
+        </is>
+      </c>
+      <c r="K352" t="inlineStr">
+        <is>
+          <t>Título: até 100c; Texto sobreposto: máx. 10 palavras; Perguntas: até 96c; Respostas: até 48c; Resultados: título até 100c, descrição até 800c.</t>
+        </is>
+      </c>
+      <c r="L352" t="inlineStr">
+        <is>
+          <t>https://help.pinterest.com/en/business/article/pinterest-product-specs</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza specs completas do Reddit (Image, Video, Carousel, Free-form Ad)
Substitui as specs resumidas pelas specs oficiais completas: dimensões
por dispositivo (cross-device/mobile/desktop) e rácio, duração de vídeo,
peso por tipo de ficheiro, limites de copy (título, URL de destino, URL
de exibição, legenda, corpo de texto no Free-form) — incluindo os
avisos de que qualquer rácio é aceite mas pode causar letterboxing.

Product Ad (catalog) não foi alterado — não fazia parte das specs
fornecidas desta vez.

Traduzidas as 4 linhas para EN/ES/FR em data/traducoes-specs.json.
Testado nas 4 línguas via Playwright, sem erros.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011oqQvDMfneVTKoco4dHUSc
</commit_message>
<xml_diff>
--- a/data/base-formatos.xlsx
+++ b/data/base-formatos.xlsx
@@ -11423,27 +11423,32 @@
       </c>
       <c r="G211" t="inlineStr">
         <is>
-          <t>2–6 cartões; 1080x1080 recomendado</t>
+          <t>2 a 6 imagens (mesmo rácio recomendado em todas). Cross-device recomendado: 1200x1500 (4:5), 1440x1080 (4:3) ou 1920x1080 (16:9). Mobile: 1200x1200 (1:1), 1080x1440 (3:4), 900x1200 (4:5), 1440x1080 (4:3), 1920x1080 (16:9). Desktop: 1200x1500 (4:5), 1440x1080 (4:3), 1920x1080 (16:9). Qualquer rácio é aceite mas pode causar letterboxing. GIF: duração recomendada 3-10s. Thumbnail (compact view, gerado automaticamente a partir da 1ª imagem ou substituível): recomendado 400x300 (4:3); aceite 300x300 (1:1).</t>
         </is>
       </c>
       <c r="H211" t="inlineStr">
         <is>
-          <t>1:1</t>
+          <t>1:1, 3:4, 4:5, 4:3 ou 16:9 (qualquer rácio aceite; mesmo rácio recomendado em todas as imagens)</t>
         </is>
       </c>
       <c r="I211" t="inlineStr">
         <is>
-          <t>20 MB por imagem; GIF 3 MB</t>
+          <t>GIF: 3 MB; Outros tipos: 20 MB; Thumbnail: 3 MB</t>
         </is>
       </c>
       <c r="J211" t="inlineStr">
         <is>
-          <t>JPG, PNG, GIF</t>
+          <t>JPG, PNG ou GIF</t>
+        </is>
+      </c>
+      <c r="K211" t="inlineStr">
+        <is>
+          <t>Título: até 300c, 1 (recomendado ≤100c, mais seguro ≤80c); URL de destino: até 268c, 1 por imagem; Legenda: até 50c, 1 por imagem; URL de exibição: até 100c, 1 por imagem (tem de corresponder ao domínio do destino); CTA: à escolha.</t>
         </is>
       </c>
       <c r="L211" t="inlineStr">
         <is>
-          <t>https://www.business.reddit.com/advertise/ad-types/carousel-ads</t>
+          <t>https://business.reddithelp.com/s/article/carousel-ad-specifications</t>
         </is>
       </c>
     </row>
@@ -11480,27 +11485,32 @@
       </c>
       <c r="G212" t="inlineStr">
         <is>
-          <t>Imagem: 1200x1200 (1:1) ou 1920x1080/1440x1080; vídeo conforme asset</t>
+          <t>Imagem (opcional): até 20 ficheiros, largura mín. recomendada 1000px; resoluções recomendadas 1200x1200 (1:1), 1440x1080 (4:3) ou 1920x1080 (16:9). Vídeo (opcional): até 5 ficheiros; duração recomendada 5-30s; resoluções recomendadas 1200x1200 (1:1), 1200x1500 (4:5), 1440x1080 (4:3) ou 1920x1080 (16:9). Thumbnail (opcional, NÃO gerado automaticamente — sem thumbnail não aparece media no feed): recomendado 400x300 ou 300x300 (1:1).</t>
         </is>
       </c>
       <c r="H212" t="inlineStr">
         <is>
-          <t>1:1</t>
+          <t>1:1, 4:5, 4:3 ou 16:9 (qualquer rácio aceite)</t>
         </is>
       </c>
       <c r="I212" t="inlineStr">
         <is>
-          <t>Imagem ≤20 MB; vídeo ≤1 GB</t>
+          <t>Imagem: 10 MB; Vídeo: até 1 GB (recomendado 50-100 MB); Thumbnail: 3 MB</t>
         </is>
       </c>
       <c r="J212" t="inlineStr">
         <is>
-          <t>JPG, PNG, GIF, MP4, MOV + rich text</t>
+          <t>Imagem: JPG, PNG ou GIF; Vídeo: MP4 ou MOV (ProRes não suportado), frame rate máx. 30 FPS; Thumbnail: JPG ou PNG</t>
+        </is>
+      </c>
+      <c r="K212" t="inlineStr">
+        <is>
+          <t>Título: até 300c, 1 (recomendado ≤100c, mais seguro ≤80c); Corpo: até 40.000c, 1 (recomendado 3-6 linhas em texto simples no feed); Legenda: até 50c, 1 por imagem/vídeo.</t>
         </is>
       </c>
       <c r="L212" t="inlineStr">
         <is>
-          <t>https://www.business.reddit.com/advertise/ad-types/free-form</t>
+          <t>https://business.reddithelp.com/s/article/free-form-ad-specifications</t>
         </is>
       </c>
     </row>
@@ -11537,27 +11547,32 @@
       </c>
       <c r="G213" t="inlineStr">
         <is>
-          <t>1080x1080 (1:1); 1080x1350 (4:5); 1440x1080 (4:3); 1920x1080 (16:9)</t>
+          <t>Imagem — Cross-device recomendado: 1440x1080 (4:3). Mobile: 1080x1080 (1:1), 1080x1440 (3:4), 1080x1350 (4:5), 1440x1080 (4:3), 1920x1080 (16:9). Desktop: 1440x1080, 1920x1080 (16:9). Qualquer rácio é aceite mas pode causar letterboxing. Thumbnail (só conversation/compact view, gerado automaticamente ou substituível): recomendado 400x300 (4:3); aceite 300x300 (1:1) ou 400x225 (16:9).</t>
         </is>
       </c>
       <c r="H213" t="inlineStr">
         <is>
-          <t>1:1 ou 4:5 ou 4:3 ou 16:9</t>
+          <t>1:1, 3:4, 4:5, 4:3 ou 16:9 (qualquer rácio aceite; recomendado 4:3 cross-device)</t>
         </is>
       </c>
       <c r="I213" t="inlineStr">
         <is>
-          <t>3 MB</t>
+          <t>Imagem: 3 MB; Thumbnail: 3 MB</t>
         </is>
       </c>
       <c r="J213" t="inlineStr">
         <is>
-          <t>JPG, PNG, GIF (estático)</t>
+          <t>JPG, PNG ou GIF (thumbnail: GIF convertido para imagem estática)</t>
+        </is>
+      </c>
+      <c r="K213" t="inlineStr">
+        <is>
+          <t>Título: até 300c (recomendado ≤100c, mais seguro ≤80c); URL de destino: até 268c; URL de exibição: até 100c (tem de corresponder ao domínio do destino); CTA: à escolha.</t>
         </is>
       </c>
       <c r="L213" t="inlineStr">
         <is>
-          <t>https://www.business.reddit.com/learning-hub/articles/reddit-image-ad-specs</t>
+          <t>https://business.reddithelp.com/s/article/image-ad-specifications</t>
         </is>
       </c>
     </row>
@@ -11646,22 +11661,32 @@
       </c>
       <c r="G215" t="inlineStr">
         <is>
-          <t>1:1 / 4:5 / 16:9; 1080p recomendado</t>
+          <t>Vídeo — Cross-device recomendado: 1440x1080 (4:3) ou 1920x1080 (16:9). Mobile: 1200x1200 (1:1), 900x1200 (3:4), 1200x1500 (4:5), 1440x1080 (4:3), 1920x1080 (16:9). Desktop: 1440x1080 (4:3), 1920x1080 (16:9). Qualquer rácio é aceite mas pode causar letterboxing. Duração: 2s a 15min (recomendado 5-30s). Thumbnail: resolução a acompanhar o rácio do vídeo (gerado automaticamente ou substituível).</t>
+        </is>
+      </c>
+      <c r="H215" t="inlineStr">
+        <is>
+          <t>1:1, 3:4, 4:5, 4:3 ou 16:9 (qualquer rácio aceite)</t>
         </is>
       </c>
       <c r="I215" t="inlineStr">
         <is>
-          <t>1 GB</t>
+          <t>Vídeo: até 1 GB; Thumbnail: 3 MB</t>
         </is>
       </c>
       <c r="J215" t="inlineStr">
         <is>
-          <t>MP4, MOV</t>
+          <t>MP4 ou MOV (ProRes não suportado); frame rate máx. 30 FPS; thumbnail: JPG, PNG ou GIF</t>
+        </is>
+      </c>
+      <c r="K215" t="inlineStr">
+        <is>
+          <t>Título: até 300c (recomendado ≤100c, mais seguro ≤80c); URL de destino: até 268c; URL de exibição: até 100c (tem de corresponder ao domínio do destino); CTA: à escolha.</t>
         </is>
       </c>
       <c r="L215" t="inlineStr">
         <is>
-          <t>https://www.business.reddit.com/advertise/ad-types/video-ads</t>
+          <t>https://business.reddithelp.com/s/article/video-ad-specifications</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Adiciona 8 formatos/features do X que faltavam (Amplify, Live, Takeovers, etc.)
Amplify Pre-roll, X Live (specs de streaming RTMP + página do evento),
Timeline Takeover, Spotlight Takeover, Branded Notifications, Dynamic
Product Ads (reposto, com specs de pré-requisitos: Pixel/Conversion API,
catálogo via Shopping Manager), Conversation Button e Polls — estes dois
últimos são features adicionáveis a Image/Video Ads, não formatos
standalone, mas com limites de copy próprios (hashtag, post pré-preenchido,
thank you post; opções de poll e duração).

Base passa de 349 para 357 formatos. Traduzidas as 8 linhas para EN/ES/FR.
Testado nas 4 línguas via Playwright, sem erros.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011oqQvDMfneVTKoco4dHUSc
</commit_message>
<xml_diff>
--- a/data/base-formatos.xlsx
+++ b/data/base-formatos.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L350"/>
+  <dimension ref="A1:L358"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="18.08984375" customWidth="1" style="2" min="1" max="1"/>
@@ -18719,16 +18719,454 @@
           <t>9:16 (recomendado); também aceites 4:5, 2:3, 1:1, 1.91:1 ou 16:9</t>
         </is>
       </c>
-      <c r="I350" t="inlineStr"/>
       <c r="J350" t="inlineStr">
         <is>
           <t>Codec vídeo H.264 (Baseline, Main ou High Profile, espaço de cor 4:2:0); áudio AAC LC</t>
         </is>
       </c>
-      <c r="K350" t="inlineStr"/>
       <c r="L350" t="inlineStr">
         <is>
           <t>https://business.x.com/en/products/vertical-video-ads</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>INTERNET</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>Paid Social</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>Single Video</t>
+        </is>
+      </c>
+      <c r="F351" t="inlineStr">
+        <is>
+          <t>Amplify Pre-roll</t>
+        </is>
+      </c>
+      <c r="G351" t="inlineStr">
+        <is>
+          <t>Recomendado 1200x1200 (mín. 600x600 para 1:1); se não for 1:1, mín. 640x360. Duração recomendada ≤15s (máx. 2:20). Bitrate: 1080p 6.000-10.000k (recomendado 6.000k); 720p 5.000-8.000k (recomendado 5.000k). Frame rate: 29,97 ou 30 FPS (superior aceite, não fazer upsample).</t>
+        </is>
+      </c>
+      <c r="H351" t="inlineStr">
+        <is>
+          <t>1:1 (recomendado — ocupa sempre espaço quadrado em desktop/mobile/timeline/perfil) ou 9:16 (vertical, ocupa o mesmo espaço); o anúncio é automaticamente combinado com conteúdo de rácio semelhante do publisher</t>
+        </is>
+      </c>
+      <c r="I351" t="inlineStr">
+        <is>
+          <t>Máx. 1 GB</t>
+        </is>
+      </c>
+      <c r="J351" t="inlineStr">
+        <is>
+          <t>MP4 ou MOV; codec H.264 (Baseline, Main ou High Profile, espaço de cor 4:2:0); áudio AAC LC</t>
+        </is>
+      </c>
+      <c r="K351" t="inlineStr">
+        <is>
+          <t>URL (opcional): tem de começar por http:// ou https://. Branding e legendas/closed captions fortemente recomendados.</t>
+        </is>
+      </c>
+      <c r="L351" t="inlineStr">
+        <is>
+          <t>https://business.x.com/en/advertising/campaign-types/amplify-pre-roll</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>INTERNET</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>Paid Social</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>Native</t>
+        </is>
+      </c>
+      <c r="F352" t="inlineStr">
+        <is>
+          <t>X Live</t>
+        </is>
+      </c>
+      <c r="G352" t="inlineStr">
+        <is>
+          <t>Resolução: 1280x720 recomendado, 1920x1080 máximo. Frame rate: 30 fps recomendado, 60 fps máximo. Keyframe interval: OBS a cada 3s; Wirecast varia por frame rate (24fps→72 frames, 30fps→90, 50fps→150, 60fps→180).</t>
+        </is>
+      </c>
+      <c r="H352" t="inlineStr"/>
+      <c r="I352" t="inlineStr">
+        <is>
+          <t>Bitrate de vídeo: 9 Mbps recomendado, 12 Mbps máximo. Bitrate de áudio: máx. 128 bps.</t>
+        </is>
+      </c>
+      <c r="J352" t="inlineStr">
+        <is>
+          <t>Protocolo RTMP; codec de vídeo H.264/AVC; codec de áudio AAC-LC. Encoders suportados: OBS, Wirecast, Restream, Golightstream, Socialive, Teradek, Elemental, Vmix, StreamYard, Streamlabs.</t>
+        </is>
+      </c>
+      <c r="K352" t="inlineStr">
+        <is>
+          <t>Descrição da página do evento: até 280c (pode incluir links externos). Carousel do evento: até 5 vídeos (live, VOD, GIFs ou fotos — investimento adicional). Timeline post: até 5 termos específicos (palavras-chave, nomes).</t>
+        </is>
+      </c>
+      <c r="L352" t="inlineStr">
+        <is>
+          <t>https://business.x.com/en/help/campaign-setup/creative-ad-specifications</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>INTERNET</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>Paid Social</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>Takeover</t>
+        </is>
+      </c>
+      <c r="F353" t="inlineStr">
+        <is>
+          <t>Timeline Takeover</t>
+        </is>
+      </c>
+      <c r="G353" t="inlineStr">
+        <is>
+          <t>Sem specs próprias — usa as specs do formato subjacente escolhido: Image Ads, Video Ads, Carousel Ads, X Live, Promoted Ads com Conversation Button/Polls, ou Branded Notifications.</t>
+        </is>
+      </c>
+      <c r="H353" t="inlineStr"/>
+      <c r="I353" t="inlineStr"/>
+      <c r="J353" t="inlineStr">
+        <is>
+          <t>Conforme o formato subjacente escolhido</t>
+        </is>
+      </c>
+      <c r="K353" t="inlineStr"/>
+      <c r="L353" t="inlineStr">
+        <is>
+          <t>https://business.x.com/en/help/campaign-setup/creative-ad-specifications</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>INTERNET</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>Paid Social</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>Takeover</t>
+        </is>
+      </c>
+      <c r="F354" t="inlineStr">
+        <is>
+          <t>Spotlight Takeover</t>
+        </is>
+      </c>
+      <c r="G354" t="inlineStr">
+        <is>
+          <t>Recomendado 1280x720. Companion Promoted Ads: 3 a 6 anúncios obrigatórios (imagem, vídeo, GIF, etc.) para apoiar o trend.</t>
+        </is>
+      </c>
+      <c r="H354" t="inlineStr">
+        <is>
+          <t>16:9</t>
+        </is>
+      </c>
+      <c r="I354" t="inlineStr">
+        <is>
+          <t>Imagem: máx. 5 MB; GIF: máx. 15 MB</t>
+        </is>
+      </c>
+      <c r="J354" t="inlineStr">
+        <is>
+          <t>Vídeo MP4 ou imagem estática (ou GIF); entrega via darkpost, só media (cartões não aceites)</t>
+        </is>
+      </c>
+      <c r="K354" t="inlineStr">
+        <is>
+          <t>Nome do trend (obrigatório): máx. 20c; Descrição do trend (opcional, muito recomendado): máx. 30c — evitar frases tipo clickbait ('50% off', 'compre um leve dois').</t>
+        </is>
+      </c>
+      <c r="L354" t="inlineStr">
+        <is>
+          <t>https://business.x.com/en/help/campaign-setup/creative-ad-specifications</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>INTERNET</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>Paid Social</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>Native</t>
+        </is>
+      </c>
+      <c r="F355" t="inlineStr">
+        <is>
+          <t>Branded Notifications</t>
+        </is>
+      </c>
+      <c r="G355" t="inlineStr">
+        <is>
+          <t>Segue as specs standard dos formatos suportados: Standalone Image/Video Ads; Image/Video Ads com botão Web ou App; Image/Video Carousel Ads com botão Web ou App (destino único); Image/Video Ads com Conversation Button; Moment Ads.</t>
+        </is>
+      </c>
+      <c r="H355" t="inlineStr"/>
+      <c r="I355" t="inlineStr"/>
+      <c r="J355" t="inlineStr">
+        <is>
+          <t>Configurado e lançado via Arrow (plataforma de terceiros, IC Group + X Next)</t>
+        </is>
+      </c>
+      <c r="K355" t="inlineStr">
+        <is>
+          <t>3 formatos de campanha: Scheduled (post de opt-in + 1 post agendado); Subscription (post de opt-in + vários posts agendados); Instant (1 post instantâneo por pessoa que fez opt-in). Requer conta X pública e verificada, e autorização via X OAuth à Arrow.</t>
+        </is>
+      </c>
+      <c r="L355" t="inlineStr">
+        <is>
+          <t>https://business.x.com/en/advertising/branded-notifications</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>INTERNET</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>Paid Social</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="D356" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>Catalog Ad</t>
+        </is>
+      </c>
+      <c r="F356" t="inlineStr">
+        <is>
+          <t>Dynamic Product Ads</t>
+        </is>
+      </c>
+      <c r="G356" t="inlineStr">
+        <is>
+          <t>Criativo gerado dinamicamente a partir do catálogo de produtos (X Shopping Manager, até 1M produtos ou feed de 8GB, sincronização agendada).</t>
+        </is>
+      </c>
+      <c r="H356" t="inlineStr"/>
+      <c r="I356" t="inlineStr"/>
+      <c r="J356" t="inlineStr">
+        <is>
+          <t>Requer X Pixel ou Conversion API configurado (eventos: Page View, Content View, Add to Cart, Purchase, com content parameters)</t>
+        </is>
+      </c>
+      <c r="K356" t="inlineStr"/>
+      <c r="L356" t="inlineStr">
+        <is>
+          <t>https://business.x.com/en/help/campaign-setup/creative-ad-specifications</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>INTERNET</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>Paid Social</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="D357" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>Native</t>
+        </is>
+      </c>
+      <c r="F357" t="inlineStr">
+        <is>
+          <t>Conversation Button</t>
+        </is>
+      </c>
+      <c r="G357" t="inlineStr"/>
+      <c r="H357" t="inlineStr"/>
+      <c r="I357" t="inlineStr"/>
+      <c r="J357" t="inlineStr">
+        <is>
+          <t>Feature adicionada a Image Ads ou Video Ads (tem de estar associada a media)</t>
+        </is>
+      </c>
+      <c r="K357" t="inlineStr">
+        <is>
+          <t>Conversation Card (post original): texto até 280c, hashtag até 21c (incl. o caracter #). Post pré-preenchido (após clique no CTA): texto até 256c, título até 23c. Thank You post: texto até 23c, URL opcional até 23c.</t>
+        </is>
+      </c>
+      <c r="L357" t="inlineStr">
+        <is>
+          <t>https://business.x.com/en/help/campaign-setup/creative-ad-specifications#conversation</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>INTERNET</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>Paid Social</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>Native</t>
+        </is>
+      </c>
+      <c r="F358" t="inlineStr">
+        <is>
+          <t>Polls</t>
+        </is>
+      </c>
+      <c r="G358" t="inlineStr">
+        <is>
+          <t>Duração: mín. 5 min, máx. 7 dias (conta a partir da criação do post, não da promoção). Pode ter ou não media associada (imagem ou vídeo).</t>
+        </is>
+      </c>
+      <c r="H358" t="inlineStr"/>
+      <c r="I358" t="inlineStr"/>
+      <c r="J358" t="inlineStr">
+        <is>
+          <t>Feature adicionada a um post, com ou sem media</t>
+        </is>
+      </c>
+      <c r="K358" t="inlineStr">
+        <is>
+          <t>Texto do post: até 280c; 2 a 4 opções de resposta, até 25c cada (não conta para os 280c do post).</t>
+        </is>
+      </c>
+      <c r="L358" t="inlineStr">
+        <is>
+          <t>https://business.x.com/en/help/campaign-setup/creative-ad-specifications#polls</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza TopView com specs completas e adiciona TopReach do TikTok
TopView: distingue Spark Ads Pull (sem duração fixa, usa o vídeo
orgânico) de Non-Spark/Spark Ads Push (vertical ≥540x960, 5-60s,
≤500 MB, bitrate ≥2.500kbps); acrescenta specs de foto de perfil, nome
da conta e limites de legenda (com a exceção CN/JP/KR), e o limite de
20 anúncios por ad group.

Adiciona "TopReach", produto de campanha novo que combina os placements
TopView + Top Feed com frequência garantida de 1 impressão por
utilizador — inclui duração (1 dia), targeting suportado, formatos de
anúncio, landing page, música, e regras de Duet/Stitch.

Base passa de 357 para 358 formatos. Traduzidas as 2 linhas para EN/ES/FR.
Testado nas 4 línguas via Playwright, sem erros.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011oqQvDMfneVTKoco4dHUSc
</commit_message>
<xml_diff>
--- a/data/base-formatos.xlsx
+++ b/data/base-formatos.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L358"/>
+  <dimension ref="A1:L359"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="18.08984375" customWidth="1" style="2" min="1" max="1"/>
@@ -12479,7 +12479,7 @@
       </c>
       <c r="G229" t="inlineStr">
         <is>
-          <t>≥540x960</t>
+          <t>Spark Ads Pull: sem duração mínima/máxima (usa o vídeo orgânico tal como publicado). Non-Spark Ads e Spark Ads Push: vertical, ≥540x960px; duração 5-60s (recomendado 9-15s).</t>
         </is>
       </c>
       <c r="H229" t="inlineStr">
@@ -12489,12 +12489,17 @@
       </c>
       <c r="I229" t="inlineStr">
         <is>
-          <t>500 MB</t>
+          <t>Non-Spark Ads e Spark Ads Push: ≤500 MB, bitrate ≥2.500kbps. Spark Ads Pull: sem limite próprio (usa o vídeo já publicado).</t>
         </is>
       </c>
       <c r="J229" t="inlineStr">
         <is>
-          <t>MP4, MOV, MPEG, 3GP</t>
+          <t>Spark Ads Pull: .mp4 ou .mov (normalmente). Non-Spark Ads e Spark Ads Push: .mp4, .mov, .mpeg, .3gp.</t>
+        </is>
+      </c>
+      <c r="K229" t="inlineStr">
+        <is>
+          <t>Foto de perfil: quadrada, 98x98px, &lt;50 KB, .jpg/.jpeg/.png (elemento-chave centrado numa área de 66x66px); em Spark Ads usa a foto de perfil da conta do vídeo. Nome da conta: 1 linha, máx. 10c (CN/JP/KR) ou 20c (outras línguas), sem emojis nem '{ }'. Legenda do anúncio: Spark Ads Pull até 100c (extraída do vídeo orgânico, pode ser vazia); Non-Spark/Spark Push até 100c, máx. 4 linhas visíveis (recomendado ≤50c CN/JP/KR ou ≤100c outras línguas para não ser coberta por 'Ver mais'), sem '{ }', emojis só a partir da versão 11. Máx. 20 anúncios por ad group.</t>
         </is>
       </c>
       <c r="L229" t="inlineStr">
@@ -18828,7 +18833,6 @@
           <t>Resolução: 1280x720 recomendado, 1920x1080 máximo. Frame rate: 30 fps recomendado, 60 fps máximo. Keyframe interval: OBS a cada 3s; Wirecast varia por frame rate (24fps→72 frames, 30fps→90, 50fps→150, 60fps→180).</t>
         </is>
       </c>
-      <c r="H352" t="inlineStr"/>
       <c r="I352" t="inlineStr">
         <is>
           <t>Bitrate de vídeo: 9 Mbps recomendado, 12 Mbps máximo. Bitrate de áudio: máx. 128 bps.</t>
@@ -18886,14 +18890,11 @@
           <t>Sem specs próprias — usa as specs do formato subjacente escolhido: Image Ads, Video Ads, Carousel Ads, X Live, Promoted Ads com Conversation Button/Polls, ou Branded Notifications.</t>
         </is>
       </c>
-      <c r="H353" t="inlineStr"/>
-      <c r="I353" t="inlineStr"/>
       <c r="J353" t="inlineStr">
         <is>
           <t>Conforme o formato subjacente escolhido</t>
         </is>
       </c>
-      <c r="K353" t="inlineStr"/>
       <c r="L353" t="inlineStr">
         <is>
           <t>https://business.x.com/en/help/campaign-setup/creative-ad-specifications</t>
@@ -18998,8 +18999,6 @@
           <t>Segue as specs standard dos formatos suportados: Standalone Image/Video Ads; Image/Video Ads com botão Web ou App; Image/Video Carousel Ads com botão Web ou App (destino único); Image/Video Ads com Conversation Button; Moment Ads.</t>
         </is>
       </c>
-      <c r="H355" t="inlineStr"/>
-      <c r="I355" t="inlineStr"/>
       <c r="J355" t="inlineStr">
         <is>
           <t>Configurado e lançado via Arrow (plataforma de terceiros, IC Group + X Next)</t>
@@ -19052,14 +19051,11 @@
           <t>Criativo gerado dinamicamente a partir do catálogo de produtos (X Shopping Manager, até 1M produtos ou feed de 8GB, sincronização agendada).</t>
         </is>
       </c>
-      <c r="H356" t="inlineStr"/>
-      <c r="I356" t="inlineStr"/>
       <c r="J356" t="inlineStr">
         <is>
           <t>Requer X Pixel ou Conversion API configurado (eventos: Page View, Content View, Add to Cart, Purchase, com content parameters)</t>
         </is>
       </c>
-      <c r="K356" t="inlineStr"/>
       <c r="L356" t="inlineStr">
         <is>
           <t>https://business.x.com/en/help/campaign-setup/creative-ad-specifications</t>
@@ -19097,9 +19093,6 @@
           <t>Conversation Button</t>
         </is>
       </c>
-      <c r="G357" t="inlineStr"/>
-      <c r="H357" t="inlineStr"/>
-      <c r="I357" t="inlineStr"/>
       <c r="J357" t="inlineStr">
         <is>
           <t>Feature adicionada a Image Ads ou Video Ads (tem de estar associada a media)</t>
@@ -19152,8 +19145,6 @@
           <t>Duração: mín. 5 min, máx. 7 dias (conta a partir da criação do post, não da promoção). Pode ter ou não media associada (imagem ou vídeo).</t>
         </is>
       </c>
-      <c r="H358" t="inlineStr"/>
-      <c r="I358" t="inlineStr"/>
       <c r="J358" t="inlineStr">
         <is>
           <t>Feature adicionada a um post, com ou sem media</t>
@@ -19167,6 +19158,60 @@
       <c r="L358" t="inlineStr">
         <is>
           <t>https://business.x.com/en/help/campaign-setup/creative-ad-specifications#polls</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>INTERNET</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>Paid Social</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>Native</t>
+        </is>
+      </c>
+      <c r="F359" t="inlineStr">
+        <is>
+          <t>TopReach</t>
+        </is>
+      </c>
+      <c r="G359" t="inlineStr">
+        <is>
+          <t>Combina os placements TopView (primeiro conteúdo ao abrir a app) e Top Feed (primeiro anúncio in-feed no For You), por 1 dia (24h). Sem dayparting. Frequência: 1 impressão por utilizador, por placement (alcance único garantido de frequência 1).</t>
+        </is>
+      </c>
+      <c r="H359" t="inlineStr"/>
+      <c r="I359" t="inlineStr"/>
+      <c r="J359" t="inlineStr">
+        <is>
+          <t>Suporta Spark Ads e Non-Spark Ads (recomendado 1-2 criativos por campanha); Duet/Stitch: Spark Ads segue os toggles do vídeo original, Non-Spark Ads não suportado.</t>
+        </is>
+      </c>
+      <c r="K359" t="inlineStr">
+        <is>
+          <t>Objetivo: Reach. Targeting disponível: idade (18+) e localização (país). Tracking de terceiros suportado (impressões e cliques). Landing page: webview standard (HTTPS) ou páginas internas TikTok (Branded Hashtag Challenge, Effect, TikTok Shop) — não suporta redirecionamento automático para app store nem link de TopView para LIVE. Música: mesma política dos in-feed ads reservation (Commercial Music Library ou faixas próprias autorizadas). Permite desativar comentários e download do vídeo. Add-ons: só os disponíveis em ambos os placements (TopView + Top Feed). Som: sempre ativo. Watermark: pode pedir vídeo descarregável sem marca de água.</t>
+        </is>
+      </c>
+      <c r="L359" t="inlineStr">
+        <is>
+          <t>https://ads.tiktok.com/resources/help/article/topreach-ad-specifications?lang=pt</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Separa Prog - Companion Banner em Audio e YouTube
O "Prog - Companion Banner" (640x640, 200 KB, JPEG/PNG) passa a
"Prog - Companion Banner (Audio)" — companion do Audio Ad.

Adiciona "Prog - Companion Banner (YouTube)" (300x60, só desktop,
<150 KB, JPG/GIF/PNG), com as specs copiadas diretamente da linha
"Google Vídeo/YouTube | Companion Banner" já existente na base.

Base passa de 295 para 296 formatos. Traduzidas as linhas para EN/ES/FR.
Testado nas 4 línguas via Playwright, sem erros.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011oqQvDMfneVTKoco4dHUSc
</commit_message>
<xml_diff>
--- a/data/base-formatos.xlsx
+++ b/data/base-formatos.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L296"/>
+  <dimension ref="A1:L297"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="18.08984375" customWidth="1" style="2" min="1" max="1"/>
@@ -16219,7 +16219,7 @@
       </c>
       <c r="F294" t="inlineStr">
         <is>
-          <t>Prog - Companion Banner</t>
+          <t>Prog - Companion Banner (Audio)</t>
         </is>
       </c>
       <c r="G294" t="inlineStr">
@@ -16242,8 +16242,6 @@
           <t>JPEG ou PNG</t>
         </is>
       </c>
-      <c r="K294" t="inlineStr"/>
-      <c r="L294" t="inlineStr"/>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
@@ -16296,8 +16294,6 @@
           <t>Vídeo MP4</t>
         </is>
       </c>
-      <c r="K295" t="inlineStr"/>
-      <c r="L295" t="inlineStr"/>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
@@ -16350,8 +16346,64 @@
           <t>Vídeo MP4</t>
         </is>
       </c>
-      <c r="K296" t="inlineStr"/>
-      <c r="L296" t="inlineStr"/>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>PROGRAMÁTICO</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>Programático</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>DV360</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>Companion Banner</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>Prog - Companion Banner (YouTube)</t>
+        </is>
+      </c>
+      <c r="G297" t="inlineStr">
+        <is>
+          <t>300x60 (só em desktop)</t>
+        </is>
+      </c>
+      <c r="H297" t="inlineStr">
+        <is>
+          <t>5:1</t>
+        </is>
+      </c>
+      <c r="I297" t="inlineStr">
+        <is>
+          <t>&lt; 150 KB</t>
+        </is>
+      </c>
+      <c r="J297" t="inlineStr">
+        <is>
+          <t>JPG, GIF ou PNG</t>
+        </is>
+      </c>
+      <c r="K297" t="inlineStr"/>
+      <c r="L297" t="inlineStr">
+        <is>
+          <t>https://support.google.com/google-ads/answer/17091270</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Repõe Prog - Uber Journey Ad e adiciona 3 placeholders ao Programático
Prog - Uber Journey Ad: reposto com as specs completas que já tinha
antes da redução do Programático (Display por fase Pedido/Espera/Viagem,
Video, copies e regras de URL), traduzido para EN/ES/FR.

Prog - Rewarded Video, Prog - Outstream: repostos/adicionados como
placeholders em branco — sem specs reais fornecidas ainda.

Prog - Rich Media: adicionado com a nota explícita "Specs a definir" em
vez de ficar em branco, traduzida para EN/ES/FR.

Base passa de 296 para 300 formatos. Testado nas 4 línguas via
Playwright, sem erros.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011oqQvDMfneVTKoco4dHUSc
</commit_message>
<xml_diff>
--- a/data/base-formatos.xlsx
+++ b/data/base-formatos.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L297"/>
+  <dimension ref="A1:L301"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="18.08984375" customWidth="1" style="2" min="1" max="1"/>
@@ -16398,12 +16398,171 @@
           <t>JPG, GIF ou PNG</t>
         </is>
       </c>
-      <c r="K297" t="inlineStr"/>
       <c r="L297" t="inlineStr">
         <is>
           <t>https://support.google.com/google-ads/answer/17091270</t>
         </is>
       </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>PROGRAMÁTICO</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>Programático</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>DV360</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>Uber</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr"/>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>Prog - Uber Journey Ad</t>
+        </is>
+      </c>
+      <c r="G298" t="inlineStr">
+        <is>
+          <t>DISPLAY — Pedido: 975x861, mín 1/máx 5 imagens (todas com logo e diferentes); Espera: 420x420 ou 314x420, máx 1 imagem; Viagem: 1146x393, mín 1/máx 5 imagens (todas com logo e diferentes). VIDEO (MP4, altura mín 486px, largura mín 864px) — Pedido: 3 a 6 seg; Espera: 6 a 60 seg; Viagem: 6 a 60 seg.</t>
+        </is>
+      </c>
+      <c r="H298" t="inlineStr">
+        <is>
+          <t>1:1 ou 3:4 ou 16:9 (vídeo)</t>
+        </is>
+      </c>
+      <c r="I298" t="inlineStr">
+        <is>
+          <t>Display: máx 1 MB (todas as fases). Video: máx 1 MB (Pedido); máx 3 MB (Espera e Viagem).</t>
+        </is>
+      </c>
+      <c r="J298" t="inlineStr">
+        <is>
+          <t>Display: imagens. Video: MP4.</t>
+        </is>
+      </c>
+      <c r="K298" t="inlineStr">
+        <is>
+          <t>DISPLAY — Pedido: título máx 25c, corpo máx 52c; Espera: título máx 25c, CTA máx 15c; Viagem: título máx 25c, corpo máx 52c, CTA máx 15c. VIDEO — Pedido: título máx 25c, corpo máx 52c; Espera: título máx 25c, CTA máx 15c; Viagem: título máx 25c, corpo máx 52c, CTA máx 15c. URL — Display: parametrizado, não parametrizado ou Click Tag (só disponível nas fases de Espera e Viagem); Video: parametrizado, não parametrizado ou Click Tag (todas as fases).</t>
+        </is>
+      </c>
+      <c r="L298" t="inlineStr"/>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>PROGRAMÁTICO</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>Programático</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>DV360</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>DV360</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr"/>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>Prog - Rewarded Video</t>
+        </is>
+      </c>
+      <c r="G299" t="inlineStr"/>
+      <c r="H299" t="inlineStr"/>
+      <c r="I299" t="inlineStr"/>
+      <c r="J299" t="inlineStr"/>
+      <c r="K299" t="inlineStr"/>
+      <c r="L299" t="inlineStr"/>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>PROGRAMÁTICO</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>Programático</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>DV360</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>DV360</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr"/>
+      <c r="F300" t="inlineStr">
+        <is>
+          <t>Prog - Outstream</t>
+        </is>
+      </c>
+      <c r="G300" t="inlineStr"/>
+      <c r="H300" t="inlineStr"/>
+      <c r="I300" t="inlineStr"/>
+      <c r="J300" t="inlineStr"/>
+      <c r="K300" t="inlineStr"/>
+      <c r="L300" t="inlineStr"/>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>PROGRAMÁTICO</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>Programático</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>DV360</t>
+        </is>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>DV360</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr"/>
+      <c r="F301" t="inlineStr">
+        <is>
+          <t>Prog - Rich Media</t>
+        </is>
+      </c>
+      <c r="G301" t="inlineStr">
+        <is>
+          <t>Specs a definir</t>
+        </is>
+      </c>
+      <c r="H301" t="inlineStr"/>
+      <c r="I301" t="inlineStr"/>
+      <c r="J301" t="inlineStr"/>
+      <c r="K301" t="inlineStr"/>
+      <c r="L301" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Adiciona formatos WeTransfer (via Azerion), Roblox (via Anzu) e OLX
Novos formatos de publishers diretos:
- Azerion|WeTransfer — "Static Starter": template PSD 2560x1600px de
  página completa com 3 layers (fundo, copy, logo) e opções de layout
  (CTA esquerda/direita; logo topo/esquerda/direita).
- Anzu|Roblox — "Display Ads": banners em 5 tamanhos/aspect ratios
  (480x320 a 640x360), até 1024px no lado maior, moderados pela Roblox.
- OLX — "Homepage Leaderboard": 320x100px, máx. 1 MB, JPEG/PNG/GIF/HTML5.

Base: 336 → 339 linhas. Traduções EN/ES/FR adicionadas para as 3 novas
linhas em data/traducoes-specs.json (336 → 339 entradas). README
atualizado com a nova contagem e publishers.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011oqQvDMfneVTKoco4dHUSc
</commit_message>
<xml_diff>
--- a/data/base-formatos.xlsx
+++ b/data/base-formatos.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L337"/>
+  <dimension ref="A1:L340"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="18.08984375" customWidth="1" style="2" min="1" max="1"/>
@@ -16648,7 +16648,6 @@
           <t>Imagem: JPG, PNG ou GIF. Vídeo: MP4, som off por defeito.</t>
         </is>
       </c>
-      <c r="K302" t="inlineStr"/>
       <c r="L302" t="inlineStr">
         <is>
           <t>https://noticiasilimitadas.pt/digital/window-splash-video/</t>
@@ -16706,7 +16705,6 @@
           <t>MP4, som off por defeito.</t>
         </is>
       </c>
-      <c r="K303" t="inlineStr"/>
       <c r="L303" t="inlineStr">
         <is>
           <t>https://noticiasilimitadas.pt/digital/intro-full-video/</t>
@@ -16764,7 +16762,6 @@
           <t>Imagem: JPG, PNG, GIF ou HTML5. Vídeo: MP4, som off por defeito.</t>
         </is>
       </c>
-      <c r="K304" t="inlineStr"/>
       <c r="L304" t="inlineStr">
         <is>
           <t>https://noticiasilimitadas.pt/digital/splash-intro/</t>
@@ -16822,7 +16819,6 @@
           <t>Imagem: JPG, PNG, GIF ou HTML5. Vídeo: MP4, som off por defeito.</t>
         </is>
       </c>
-      <c r="K305" t="inlineStr"/>
       <c r="L305" t="inlineStr">
         <is>
           <t>https://noticiasilimitadas.pt/digital/video-fullscreen-takeover/</t>
@@ -16880,7 +16876,6 @@
           <t>Imagem: JPG, PNG, GIF ou HTML5. Vídeo: MP4, som off por defeito.</t>
         </is>
       </c>
-      <c r="K306" t="inlineStr"/>
       <c r="L306" t="inlineStr">
         <is>
           <t>https://noticiasilimitadas.pt/digital/FullScreen-TakeOver/</t>
@@ -16923,7 +16918,6 @@
           <t>1260x200px + 728x150px + 320x100px, e também 300x600px ou 300x250px. Pode incluir vídeo (contactar para mais info).</t>
         </is>
       </c>
-      <c r="H307" t="inlineStr"/>
       <c r="I307" t="inlineStr">
         <is>
           <t>Máx. 200 KB por ficheiro.</t>
@@ -16934,7 +16928,6 @@
           <t>JPG, PNG, GIF ou HTML5.</t>
         </is>
       </c>
-      <c r="K307" t="inlineStr"/>
       <c r="L307" t="inlineStr">
         <is>
           <t>https://noticiasilimitadas.pt/digital/takeover/</t>
@@ -16977,7 +16970,6 @@
           <t>2 imagens laterais 330x1080px + 1 imagem de topo 1260x290px. Laterais não devem conter informação relevante (podem ficar cortadas em ecrãs mais pequenos).</t>
         </is>
       </c>
-      <c r="H308" t="inlineStr"/>
       <c r="I308" t="inlineStr">
         <is>
           <t>Máx. 200 KB por imagem.</t>
@@ -16988,7 +16980,6 @@
           <t>JPG, PNG ou GIF.</t>
         </is>
       </c>
-      <c r="K308" t="inlineStr"/>
       <c r="L308" t="inlineStr">
         <is>
           <t>https://noticiasilimitadas.pt/digital/skin/</t>
@@ -17046,7 +17037,6 @@
           <t>Imagem: JPG, PNG ou GIF. Vídeo: MP4, som off por defeito.</t>
         </is>
       </c>
-      <c r="K309" t="inlineStr"/>
       <c r="L309" t="inlineStr">
         <is>
           <t>https://noticiasilimitadas.pt/digital/skin-video/</t>
@@ -17089,7 +17079,6 @@
           <t>2 imagens laterais 310x1080px + 1 imagem de fundo 1300x250px. Laterais não devem conter informação relevante (podem ficar cortadas em ecrãs mais pequenos).</t>
         </is>
       </c>
-      <c r="H310" t="inlineStr"/>
       <c r="I310" t="inlineStr">
         <is>
           <t>Máx. 200 KB por imagem.</t>
@@ -17100,7 +17089,6 @@
           <t>JPG, PNG ou GIF.</t>
         </is>
       </c>
-      <c r="K310" t="inlineStr"/>
       <c r="L310" t="inlineStr">
         <is>
           <t>https://noticiasilimitadas.pt/digital/skin-invertida/</t>
@@ -17158,7 +17146,6 @@
           <t>Imagem: JPG, PNG ou GIF. Vídeo: MP4.</t>
         </is>
       </c>
-      <c r="K311" t="inlineStr"/>
       <c r="L311" t="inlineStr">
         <is>
           <t>https://noticiasilimitadas.pt/digital/skin-mobile/</t>
@@ -17201,7 +17188,6 @@
           <t>320x600px</t>
         </is>
       </c>
-      <c r="H312" t="inlineStr"/>
       <c r="I312" t="inlineStr">
         <is>
           <t>Máx. 200 KB.</t>
@@ -17212,7 +17198,6 @@
           <t>JPG, PNG ou GIF.</t>
         </is>
       </c>
-      <c r="K312" t="inlineStr"/>
       <c r="L312" t="inlineStr">
         <is>
           <t>https://noticiasilimitadas.pt/digital/parallax/</t>
@@ -17255,9 +17240,6 @@
           <t>Mín. 3 imagens, 320x320px cada; logótipo da marca 160x50px.</t>
         </is>
       </c>
-      <c r="H313" t="inlineStr"/>
-      <c r="I313" t="inlineStr"/>
-      <c r="J313" t="inlineStr"/>
       <c r="K313" t="inlineStr">
         <is>
           <t>Título: máx. 40c; Descrição: máx. 35c; Texto do botão CTA (ex.: Saber mais, Comprar agora, Reserve já, Entre em contacto).</t>
@@ -17320,7 +17302,6 @@
           <t>Imagem: JPG, PNG ou GIF. Vídeo: MP4, som off por defeito.</t>
         </is>
       </c>
-      <c r="K314" t="inlineStr"/>
       <c r="L314" t="inlineStr">
         <is>
           <t>https://noticiasilimitadas.pt/digital/flipbook/</t>
@@ -17363,7 +17344,6 @@
           <t>4 a 6 imagens, 300x300px cada.</t>
         </is>
       </c>
-      <c r="H315" t="inlineStr"/>
       <c r="I315" t="inlineStr">
         <is>
           <t>Máx. 100 KB por imagem.</t>
@@ -17374,7 +17354,6 @@
           <t>JPG ou PNG.</t>
         </is>
       </c>
-      <c r="K315" t="inlineStr"/>
       <c r="L315" t="inlineStr">
         <is>
           <t>https://noticiasilimitadas.pt/digital/mrec-cubo-3d/</t>
@@ -17417,7 +17396,6 @@
           <t>3 a 6 imagens, 300x600px cada.</t>
         </is>
       </c>
-      <c r="H316" t="inlineStr"/>
       <c r="I316" t="inlineStr">
         <is>
           <t>Máx. 100 KB por imagem.</t>
@@ -17428,7 +17406,6 @@
           <t>JPG ou PNG.</t>
         </is>
       </c>
-      <c r="K316" t="inlineStr"/>
       <c r="L316" t="inlineStr">
         <is>
           <t>https://noticiasilimitadas.pt/digital/half-page-cubo-3d/</t>
@@ -17486,7 +17463,6 @@
           <t>Imagem: JPG, PNG ou GIF. Vídeo: MP4.</t>
         </is>
       </c>
-      <c r="K317" t="inlineStr"/>
       <c r="L317" t="inlineStr">
         <is>
           <t>https://noticiasilimitadas.pt/digital/ticker/</t>
@@ -17544,7 +17520,6 @@
           <t>MP4, som off por defeito.</t>
         </is>
       </c>
-      <c r="K318" t="inlineStr"/>
       <c r="L318" t="inlineStr">
         <is>
           <t>https://noticiasilimitadas.pt/digital/spot-tv/</t>
@@ -17602,7 +17577,6 @@
           <t>Imagem: JPG, PNG ou GIF. Vídeo: MP4.</t>
         </is>
       </c>
-      <c r="K319" t="inlineStr"/>
       <c r="L319" t="inlineStr">
         <is>
           <t>https://noticiasilimitadas.pt/digital/flip-ad/</t>
@@ -17645,7 +17619,6 @@
           <t>2 imagens: 300x600px + 150x300px.</t>
         </is>
       </c>
-      <c r="H320" t="inlineStr"/>
       <c r="I320" t="inlineStr">
         <is>
           <t>Máx. 200 KB por imagem.</t>
@@ -17656,7 +17629,6 @@
           <t>JPG, PNG ou GIF.</t>
         </is>
       </c>
-      <c r="K320" t="inlineStr"/>
       <c r="L320" t="inlineStr">
         <is>
           <t>https://noticiasilimitadas.pt/digital/overslide/</t>
@@ -17714,7 +17686,6 @@
           <t>Imagem: JPG, PNG, GIF ou HTML5. Vídeo: MP4.</t>
         </is>
       </c>
-      <c r="K321" t="inlineStr"/>
       <c r="L321" t="inlineStr">
         <is>
           <t>https://noticiasilimitadas.pt/digital/layer/</t>
@@ -17772,7 +17743,6 @@
           <t>Imagem: JPG, PNG ou GIF. Vídeo: MP4, som off por defeito.</t>
         </is>
       </c>
-      <c r="K322" t="inlineStr"/>
       <c r="L322" t="inlineStr">
         <is>
           <t>https://noticiasilimitadas.pt/digital/peel-off/</t>
@@ -17815,7 +17785,6 @@
           <t>(1260x100px + 1260x370px) + (728x100px + 728x300px) + (320x100px + 320x250px).</t>
         </is>
       </c>
-      <c r="H323" t="inlineStr"/>
       <c r="I323" t="inlineStr">
         <is>
           <t>Máx. 200 KB por ficheiro.</t>
@@ -17826,7 +17795,6 @@
           <t>JPG, PNG ou GIF.</t>
         </is>
       </c>
-      <c r="K323" t="inlineStr"/>
       <c r="L323" t="inlineStr">
         <is>
           <t>https://noticiasilimitadas.pt/digital/push-down/</t>
@@ -17869,7 +17837,6 @@
           <t>Duração máx. recomendada 20s (CPV contabilizado aos 20s em campanhas por visualizações).</t>
         </is>
       </c>
-      <c r="H324" t="inlineStr"/>
       <c r="I324" t="inlineStr">
         <is>
           <t>Máx. 100 MB.</t>
@@ -17880,7 +17847,6 @@
           <t>MP3.</t>
         </is>
       </c>
-      <c r="K324" t="inlineStr"/>
       <c r="L324" t="inlineStr">
         <is>
           <t>https://noticiasilimitadas.pt/digital/audio-ad/</t>
@@ -17938,7 +17904,6 @@
           <t>MP4.</t>
         </is>
       </c>
-      <c r="K325" t="inlineStr"/>
       <c r="L325" t="inlineStr">
         <is>
           <t>https://noticiasilimitadas.pt/digital/pre-roll/</t>
@@ -17996,7 +17961,6 @@
           <t>MP4, som off por defeito.</t>
         </is>
       </c>
-      <c r="K326" t="inlineStr"/>
       <c r="L326" t="inlineStr">
         <is>
           <t>https://noticiasilimitadas.pt/digital/incontent-sticky/</t>
@@ -18054,7 +18018,6 @@
           <t>MP4, som off por defeito.</t>
         </is>
       </c>
-      <c r="K327" t="inlineStr"/>
       <c r="L327" t="inlineStr">
         <is>
           <t>https://noticiasilimitadas.pt/digital/incontent/</t>
@@ -18097,7 +18060,6 @@
           <t>1260x200px + 728x150px + 320x100px, ou 970x250px + 728x90px + 320x50px.</t>
         </is>
       </c>
-      <c r="H328" t="inlineStr"/>
       <c r="I328" t="inlineStr">
         <is>
           <t>Máx. 200 KB por ficheiro.</t>
@@ -18108,7 +18070,6 @@
           <t>JPG, PNG, GIF ou HTML5.</t>
         </is>
       </c>
-      <c r="K328" t="inlineStr"/>
       <c r="L328" t="inlineStr">
         <is>
           <t>https://noticiasilimitadas.pt/digital/superboard/</t>
@@ -18151,7 +18112,6 @@
           <t>300x250px</t>
         </is>
       </c>
-      <c r="H329" t="inlineStr"/>
       <c r="I329" t="inlineStr">
         <is>
           <t>Máx. 150 KB.</t>
@@ -18162,7 +18122,6 @@
           <t>JPG, PNG, GIF ou HTML5.</t>
         </is>
       </c>
-      <c r="K329" t="inlineStr"/>
       <c r="L329" t="inlineStr">
         <is>
           <t>https://noticiasilimitadas.pt/digital/mrec/</t>
@@ -18205,7 +18164,6 @@
           <t>300x600px</t>
         </is>
       </c>
-      <c r="H330" t="inlineStr"/>
       <c r="I330" t="inlineStr">
         <is>
           <t>Máx. 200 KB.</t>
@@ -18216,7 +18174,6 @@
           <t>JPG, PNG, GIF ou HTML5.</t>
         </is>
       </c>
-      <c r="K330" t="inlineStr"/>
       <c r="L330" t="inlineStr">
         <is>
           <t>https://noticiasilimitadas.pt/digital/half-page/</t>
@@ -18259,7 +18216,6 @@
           <t>1260x370px + 728x338px + 320x239px. Se tiver vídeo, deixar espaço nas imagens.</t>
         </is>
       </c>
-      <c r="H331" t="inlineStr"/>
       <c r="I331" t="inlineStr">
         <is>
           <t>Máx. 200 KB por ficheiro.</t>
@@ -18270,7 +18226,6 @@
           <t>JPG, PNG, GIF ou HTML5.</t>
         </is>
       </c>
-      <c r="K331" t="inlineStr"/>
       <c r="L331" t="inlineStr">
         <is>
           <t>https://noticiasilimitadas.pt/digital/megapub/</t>
@@ -18328,7 +18283,6 @@
           <t>MP4.</t>
         </is>
       </c>
-      <c r="K332" t="inlineStr"/>
       <c r="L332" t="inlineStr">
         <is>
           <t>https://noticiasilimitadas.pt/digital/mrec-video/</t>
@@ -18371,7 +18325,6 @@
           <t>300x600px.</t>
         </is>
       </c>
-      <c r="H333" t="inlineStr"/>
       <c r="I333" t="inlineStr">
         <is>
           <t>Imagem: máx. 150 KB. Vídeo: máx. 2 MB.</t>
@@ -18382,7 +18335,6 @@
           <t>Imagem: JPG, PNG ou GIF. Vídeo: MP4.</t>
         </is>
       </c>
-      <c r="K333" t="inlineStr"/>
       <c r="L333" t="inlineStr">
         <is>
           <t>https://noticiasilimitadas.pt/digital/half-page-video/</t>
@@ -18440,7 +18392,6 @@
           <t>MP4.</t>
         </is>
       </c>
-      <c r="K334" t="inlineStr"/>
       <c r="L334" t="inlineStr">
         <is>
           <t>https://noticiasilimitadas.pt/digital/half-page-full-video/</t>
@@ -18483,14 +18434,11 @@
           <t>Sem dimensão fixa — usa o post/link social já publicado.</t>
         </is>
       </c>
-      <c r="H335" t="inlineStr"/>
-      <c r="I335" t="inlineStr"/>
       <c r="J335" t="inlineStr">
         <is>
           <t>Link social do Facebook, Instagram, X (Twitter) ou LinkedIn.</t>
         </is>
       </c>
-      <c r="K335" t="inlineStr"/>
       <c r="L335" t="inlineStr">
         <is>
           <t>https://noticiasilimitadas.pt/digital/social-card/</t>
@@ -18533,7 +18481,6 @@
           <t>2 a 5 imagens, 300x600px cada.</t>
         </is>
       </c>
-      <c r="H336" t="inlineStr"/>
       <c r="I336" t="inlineStr">
         <is>
           <t>Máx. 100 KB por imagem.</t>
@@ -18544,7 +18491,6 @@
           <t>JPG, PNG ou GIF.</t>
         </is>
       </c>
-      <c r="K336" t="inlineStr"/>
       <c r="L336" t="inlineStr">
         <is>
           <t>https://noticiasilimitadas.pt/digital/filmstrip/</t>
@@ -18587,7 +18533,6 @@
           <t>2 imagens: 300x250px + 640x124px.</t>
         </is>
       </c>
-      <c r="H337" t="inlineStr"/>
       <c r="I337" t="inlineStr">
         <is>
           <t>Máx. 200 KB por imagem.</t>
@@ -18608,6 +18553,164 @@
           <t>https://noticiasilimitadas.pt/digital/newsletter/</t>
         </is>
       </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>INTERNET</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>Internet</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>Azerion</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>WeTransfer</t>
+        </is>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>Takeover</t>
+        </is>
+      </c>
+      <c r="F338" t="inlineStr">
+        <is>
+          <t>Static Starter</t>
+        </is>
+      </c>
+      <c r="G338" t="inlineStr">
+        <is>
+          <t>Ficheiro PSD 2560x1600px (perfil de cores RGB). 3 elementos gráficos em layers: imagem de fundo; copy (em imagem ou texto); logo.</t>
+        </is>
+      </c>
+      <c r="H338" t="inlineStr">
+        <is>
+          <t>8:5</t>
+        </is>
+      </c>
+      <c r="I338" t="inlineStr"/>
+      <c r="J338" t="inlineStr">
+        <is>
+          <t>PSD</t>
+        </is>
+      </c>
+      <c r="K338" t="inlineStr">
+        <is>
+          <t>Opções de layout: fundo com copy (base); + CTA à esquerda ou à direita (opcional); + logo no topo, à esquerda ou à direita.</t>
+        </is>
+      </c>
+      <c r="L338" t="inlineStr"/>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>INTERNET</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>Internet</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>Anzu</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>Roblox</t>
+        </is>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>Banner</t>
+        </is>
+      </c>
+      <c r="F339" t="inlineStr">
+        <is>
+          <t>Display Ads</t>
+        </is>
+      </c>
+      <c r="G339" t="inlineStr">
+        <is>
+          <t>480x320px, 320x480px, 320x50px, 300x250px ou 640x360px. Máx. 1024px no lado maior; recomendado mín. 512px no lado maior, mantendo o aspect ratio.</t>
+        </is>
+      </c>
+      <c r="H339" t="inlineStr">
+        <is>
+          <t>3:2, 2:3, 6.4:1, 6:5 ou 16:9 (consoante o tamanho escolhido)</t>
+        </is>
+      </c>
+      <c r="I339" t="inlineStr"/>
+      <c r="J339" t="inlineStr">
+        <is>
+          <t>PNG, JPG ou BMP (também aceite em GIF, redimensionado automaticamente pela Anzu).</t>
+        </is>
+      </c>
+      <c r="K339" t="inlineStr">
+        <is>
+          <t>Até 10 criativos por deal. Todos os criativos são moderados pela equipa Roblox e podem sofrer alterações para cumprir as regras de compliance da Roblox.</t>
+        </is>
+      </c>
+      <c r="L339" t="inlineStr"/>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>INTERNET</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>Internet</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>OLX</t>
+        </is>
+      </c>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>OLX</t>
+        </is>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>Leaderboard</t>
+        </is>
+      </c>
+      <c r="F340" t="inlineStr">
+        <is>
+          <t>Homepage Leaderboard</t>
+        </is>
+      </c>
+      <c r="G340" t="inlineStr">
+        <is>
+          <t>320x100px</t>
+        </is>
+      </c>
+      <c r="H340" t="inlineStr"/>
+      <c r="I340" t="inlineStr">
+        <is>
+          <t>Máx. 1 MB</t>
+        </is>
+      </c>
+      <c r="J340" t="inlineStr">
+        <is>
+          <t>JPEG, JPG, PNG, GIF ou HTML5 (GWD)</t>
+        </is>
+      </c>
+      <c r="K340" t="inlineStr"/>
+      <c r="L340" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>